<commit_message>
Stream link suggestions with YouTube default, template dropdowns
- Stream link field (form and spreadsheet) suggests the YouTube channel first plus previously used links labelled by platform
- Empty link cells show the YouTube default as placeholder
- Excel template: dropdowns for stream link (YouTube default), degree and place; updated notes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqjysm6ZxBaYZPctG6chPQ
</commit_message>
<xml_diff>
--- a/assets/templates/template.xlsx
+++ b/assets/templates/template.xlsx
@@ -267,7 +267,7 @@
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>اختياري: رابط يوتيوب أو زوم أو بلاك بورد (يظهر كرمز QR إذا فعّلته في الموقع)</t>
+        <t>الافتراضي: قناة اليوتيوب https://www.youtube.com/@src.sds1 (اتركه فاضي أو اختره من القائمة). تقدر تلصق رابط زوم أو بلاك بورد أو أي منصة.</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
@@ -8896,9 +8896,18 @@
       <c r="Y301" s="6" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="11">
     <dataValidation sqref="B2:B301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="ذكر أو أنثى" type="list">
       <formula1>"ذكر,أنثى"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="الافتراضي قناة اليوتيوب — أو الصق أي رابط آخر" type="list">
+      <formula1>"https://www.youtube.com/@src.sds1"</formula1>
+    </dataValidation>
+    <dataValidation sqref="A2:A301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر أو اكتب الدرجة" type="list">
+      <formula1>"الماجستير في الفقه المقارن,الماجستير في الفقه,الماجستير في أصول الفقه,الدكتوراه في الفقه,الدكتوراه في الفقه المقارن,الدكتوراه في أصول الفقه"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر أو اكتب المكان" type="list">
+      <formula1>"قاعة ابن عثيمين,القاعة الكبرى بمبنى الطالبات"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر اليوم" type="list">
       <formula1>"الأحد,الاثنين,الثلاثاء,الأربعاء,الخميس,الجمعة,السبت"</formula1>
@@ -8984,7 +8993,7 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>6) رابط البث اختياري (يوتيوب، زوم، بلاك بورد...) ويظهر كرمز QR إذا فعّلته في الموقع.</t>
+          <t>6) رابط البث: الافتراضي قناة اليوتيوب (اختره من القائمة أو اتركه فاضي). تقدر تلصق رابط زوم أو بلاك بورد أو أي منصة. يظهر كرمز QR إذا فعّلته في الموقع.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WhatsApp invitation and recording messages, committee and recording links, live sync
- New optional fields: committee Zoom link and recording link (form, spreadsheet, Excel and Google Sheets templates)
- Copy buttons for the invitation and recording messages in the college's format, per row and in the form; Gregorian date computed from Hijri; editable templates with optional blocks
- Editing a row opened from the table syncs only the changed fields back to it; designs opened from history autosave
- Same committee Zoom link at the same time is flagged as a conflict; saved spreadsheets migrated to the new columns

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqjysm6ZxBaYZPctG6chPQ
</commit_message>
<xml_diff>
--- a/assets/templates/template.xlsx
+++ b/assets/templates/template.xlsx
@@ -272,75 +272,85 @@
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+        <t>اختياري: رابط زوم خاص باللجنة (غالباً للدكتوراه مع مناقش خارجي). يظهر في رسالة الدعوة فقط إذا عبّأته.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: الأستاذ في قسم الفقه</t>
+        <t>يُضاف بعد انتهاء المناقشة: رابط تسجيل اليوتيوب (يختلف عن رابط البث). يُستخدم في رسالة التسجيل.</t>
       </text>
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
+        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
       </text>
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+        <t>مثال: الأستاذ في قسم الفقه</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: الأستاذ في قسم الفقه</t>
+        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
       </text>
     </comment>
     <comment ref="P1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
+        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
       </text>
     </comment>
     <comment ref="Q1" authorId="0" shapeId="0">
       <text>
-        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+        <t>مثال: الأستاذ في قسم الفقه</t>
       </text>
     </comment>
     <comment ref="R1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: الأستاذ في قسم الفقه</t>
+        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
       </text>
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
+        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
       </text>
     </comment>
     <comment ref="T1" authorId="0" shapeId="0">
       <text>
-        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+        <t>مثال: الأستاذ في قسم الفقه</t>
       </text>
     </comment>
     <comment ref="U1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: الأستاذ في قسم الفقه</t>
+        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
       </text>
     </comment>
     <comment ref="V1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
+        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
       </text>
     </comment>
     <comment ref="W1" authorId="0" shapeId="0">
       <text>
-        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+        <t>مثال: الأستاذ في قسم الفقه</t>
       </text>
     </comment>
     <comment ref="X1" authorId="0" shapeId="0">
       <text>
+        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
+      <text>
         <t>مثال: الأستاذ في قسم الفقه</t>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
+    <comment ref="AA1" authorId="0" shapeId="0">
       <text>
         <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
       </text>
@@ -638,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y301"/>
+  <dimension ref="A1:AA301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -651,8 +661,8 @@
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="24" customWidth="1" min="14" max="14"/>
     <col width="24" customWidth="1" min="15" max="15"/>
@@ -666,6 +676,8 @@
     <col width="24" customWidth="1" min="23" max="23"/>
     <col width="24" customWidth="1" min="24" max="24"/>
     <col width="24" customWidth="1" min="25" max="25"/>
+    <col width="24" customWidth="1" min="26" max="26"/>
+    <col width="24" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -719,77 +731,87 @@
           <t>رابط البث</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>رابط اللجنة</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>رابط التسجيل</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>عضو1 الاسم</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>عضو1 الصفة</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>عضو1 الدور</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>عضو2 الاسم</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>عضو2 الصفة</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>عضو2 الدور</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>عضو3 الاسم</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>عضو3 الصفة</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>عضو3 الدور</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>عضو4 الاسم</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>عضو4 الصفة</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>عضو4 الدور</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>عضو5 الاسم</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>عضو5 الصفة</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>عضو5 الدور</t>
         </is>
@@ -806,8 +828,8 @@
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
-      <c r="K2" s="5" t="n"/>
-      <c r="L2" s="5" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
       <c r="M2" s="5" t="n"/>
       <c r="N2" s="5" t="n"/>
       <c r="O2" s="5" t="n"/>
@@ -821,6 +843,8 @@
       <c r="W2" s="5" t="n"/>
       <c r="X2" s="5" t="n"/>
       <c r="Y2" s="5" t="n"/>
+      <c r="Z2" s="5" t="n"/>
+      <c r="AA2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="n"/>
@@ -848,6 +872,8 @@
       <c r="W3" s="6" t="n"/>
       <c r="X3" s="6" t="n"/>
       <c r="Y3" s="6" t="n"/>
+      <c r="Z3" s="6" t="n"/>
+      <c r="AA3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -860,8 +886,8 @@
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
       <c r="M4" s="5" t="n"/>
       <c r="N4" s="5" t="n"/>
       <c r="O4" s="5" t="n"/>
@@ -875,6 +901,8 @@
       <c r="W4" s="5" t="n"/>
       <c r="X4" s="5" t="n"/>
       <c r="Y4" s="5" t="n"/>
+      <c r="Z4" s="5" t="n"/>
+      <c r="AA4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n"/>
@@ -902,6 +930,8 @@
       <c r="W5" s="6" t="n"/>
       <c r="X5" s="6" t="n"/>
       <c r="Y5" s="6" t="n"/>
+      <c r="Z5" s="6" t="n"/>
+      <c r="AA5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -914,8 +944,8 @@
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
       <c r="M6" s="5" t="n"/>
       <c r="N6" s="5" t="n"/>
       <c r="O6" s="5" t="n"/>
@@ -929,6 +959,8 @@
       <c r="W6" s="5" t="n"/>
       <c r="X6" s="5" t="n"/>
       <c r="Y6" s="5" t="n"/>
+      <c r="Z6" s="5" t="n"/>
+      <c r="AA6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n"/>
@@ -956,6 +988,8 @@
       <c r="W7" s="6" t="n"/>
       <c r="X7" s="6" t="n"/>
       <c r="Y7" s="6" t="n"/>
+      <c r="Z7" s="6" t="n"/>
+      <c r="AA7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -968,8 +1002,8 @@
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="5" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
       <c r="M8" s="5" t="n"/>
       <c r="N8" s="5" t="n"/>
       <c r="O8" s="5" t="n"/>
@@ -983,6 +1017,8 @@
       <c r="W8" s="5" t="n"/>
       <c r="X8" s="5" t="n"/>
       <c r="Y8" s="5" t="n"/>
+      <c r="Z8" s="5" t="n"/>
+      <c r="AA8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
@@ -1010,6 +1046,8 @@
       <c r="W9" s="6" t="n"/>
       <c r="X9" s="6" t="n"/>
       <c r="Y9" s="6" t="n"/>
+      <c r="Z9" s="6" t="n"/>
+      <c r="AA9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -1022,8 +1060,8 @@
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="5" t="n"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
       <c r="M10" s="5" t="n"/>
       <c r="N10" s="5" t="n"/>
       <c r="O10" s="5" t="n"/>
@@ -1037,6 +1075,8 @@
       <c r="W10" s="5" t="n"/>
       <c r="X10" s="5" t="n"/>
       <c r="Y10" s="5" t="n"/>
+      <c r="Z10" s="5" t="n"/>
+      <c r="AA10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
@@ -1064,6 +1104,8 @@
       <c r="W11" s="6" t="n"/>
       <c r="X11" s="6" t="n"/>
       <c r="Y11" s="6" t="n"/>
+      <c r="Z11" s="6" t="n"/>
+      <c r="AA11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -1076,8 +1118,8 @@
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
-      <c r="K12" s="5" t="n"/>
-      <c r="L12" s="5" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
       <c r="M12" s="5" t="n"/>
       <c r="N12" s="5" t="n"/>
       <c r="O12" s="5" t="n"/>
@@ -1091,6 +1133,8 @@
       <c r="W12" s="5" t="n"/>
       <c r="X12" s="5" t="n"/>
       <c r="Y12" s="5" t="n"/>
+      <c r="Z12" s="5" t="n"/>
+      <c r="AA12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
@@ -1118,6 +1162,8 @@
       <c r="W13" s="6" t="n"/>
       <c r="X13" s="6" t="n"/>
       <c r="Y13" s="6" t="n"/>
+      <c r="Z13" s="6" t="n"/>
+      <c r="AA13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -1130,8 +1176,8 @@
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
-      <c r="K14" s="5" t="n"/>
-      <c r="L14" s="5" t="n"/>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
       <c r="M14" s="5" t="n"/>
       <c r="N14" s="5" t="n"/>
       <c r="O14" s="5" t="n"/>
@@ -1145,6 +1191,8 @@
       <c r="W14" s="5" t="n"/>
       <c r="X14" s="5" t="n"/>
       <c r="Y14" s="5" t="n"/>
+      <c r="Z14" s="5" t="n"/>
+      <c r="AA14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
@@ -1172,6 +1220,8 @@
       <c r="W15" s="6" t="n"/>
       <c r="X15" s="6" t="n"/>
       <c r="Y15" s="6" t="n"/>
+      <c r="Z15" s="6" t="n"/>
+      <c r="AA15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -1184,8 +1234,8 @@
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
-      <c r="K16" s="5" t="n"/>
-      <c r="L16" s="5" t="n"/>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
       <c r="M16" s="5" t="n"/>
       <c r="N16" s="5" t="n"/>
       <c r="O16" s="5" t="n"/>
@@ -1199,6 +1249,8 @@
       <c r="W16" s="5" t="n"/>
       <c r="X16" s="5" t="n"/>
       <c r="Y16" s="5" t="n"/>
+      <c r="Z16" s="5" t="n"/>
+      <c r="AA16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
@@ -1226,6 +1278,8 @@
       <c r="W17" s="6" t="n"/>
       <c r="X17" s="6" t="n"/>
       <c r="Y17" s="6" t="n"/>
+      <c r="Z17" s="6" t="n"/>
+      <c r="AA17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -1238,8 +1292,8 @@
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
-      <c r="K18" s="5" t="n"/>
-      <c r="L18" s="5" t="n"/>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="n"/>
       <c r="M18" s="5" t="n"/>
       <c r="N18" s="5" t="n"/>
       <c r="O18" s="5" t="n"/>
@@ -1253,6 +1307,8 @@
       <c r="W18" s="5" t="n"/>
       <c r="X18" s="5" t="n"/>
       <c r="Y18" s="5" t="n"/>
+      <c r="Z18" s="5" t="n"/>
+      <c r="AA18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
@@ -1280,6 +1336,8 @@
       <c r="W19" s="6" t="n"/>
       <c r="X19" s="6" t="n"/>
       <c r="Y19" s="6" t="n"/>
+      <c r="Z19" s="6" t="n"/>
+      <c r="AA19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -1292,8 +1350,8 @@
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
-      <c r="K20" s="5" t="n"/>
-      <c r="L20" s="5" t="n"/>
+      <c r="K20" s="3" t="n"/>
+      <c r="L20" s="3" t="n"/>
       <c r="M20" s="5" t="n"/>
       <c r="N20" s="5" t="n"/>
       <c r="O20" s="5" t="n"/>
@@ -1307,6 +1365,8 @@
       <c r="W20" s="5" t="n"/>
       <c r="X20" s="5" t="n"/>
       <c r="Y20" s="5" t="n"/>
+      <c r="Z20" s="5" t="n"/>
+      <c r="AA20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n"/>
@@ -1334,6 +1394,8 @@
       <c r="W21" s="6" t="n"/>
       <c r="X21" s="6" t="n"/>
       <c r="Y21" s="6" t="n"/>
+      <c r="Z21" s="6" t="n"/>
+      <c r="AA21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -1346,8 +1408,8 @@
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
-      <c r="K22" s="5" t="n"/>
-      <c r="L22" s="5" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="3" t="n"/>
       <c r="M22" s="5" t="n"/>
       <c r="N22" s="5" t="n"/>
       <c r="O22" s="5" t="n"/>
@@ -1361,6 +1423,8 @@
       <c r="W22" s="5" t="n"/>
       <c r="X22" s="5" t="n"/>
       <c r="Y22" s="5" t="n"/>
+      <c r="Z22" s="5" t="n"/>
+      <c r="AA22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
@@ -1388,6 +1452,8 @@
       <c r="W23" s="6" t="n"/>
       <c r="X23" s="6" t="n"/>
       <c r="Y23" s="6" t="n"/>
+      <c r="Z23" s="6" t="n"/>
+      <c r="AA23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -1400,8 +1466,8 @@
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
-      <c r="K24" s="5" t="n"/>
-      <c r="L24" s="5" t="n"/>
+      <c r="K24" s="3" t="n"/>
+      <c r="L24" s="3" t="n"/>
       <c r="M24" s="5" t="n"/>
       <c r="N24" s="5" t="n"/>
       <c r="O24" s="5" t="n"/>
@@ -1415,6 +1481,8 @@
       <c r="W24" s="5" t="n"/>
       <c r="X24" s="5" t="n"/>
       <c r="Y24" s="5" t="n"/>
+      <c r="Z24" s="5" t="n"/>
+      <c r="AA24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n"/>
@@ -1442,6 +1510,8 @@
       <c r="W25" s="6" t="n"/>
       <c r="X25" s="6" t="n"/>
       <c r="Y25" s="6" t="n"/>
+      <c r="Z25" s="6" t="n"/>
+      <c r="AA25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -1454,8 +1524,8 @@
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
-      <c r="K26" s="5" t="n"/>
-      <c r="L26" s="5" t="n"/>
+      <c r="K26" s="3" t="n"/>
+      <c r="L26" s="3" t="n"/>
       <c r="M26" s="5" t="n"/>
       <c r="N26" s="5" t="n"/>
       <c r="O26" s="5" t="n"/>
@@ -1469,6 +1539,8 @@
       <c r="W26" s="5" t="n"/>
       <c r="X26" s="5" t="n"/>
       <c r="Y26" s="5" t="n"/>
+      <c r="Z26" s="5" t="n"/>
+      <c r="AA26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n"/>
@@ -1496,6 +1568,8 @@
       <c r="W27" s="6" t="n"/>
       <c r="X27" s="6" t="n"/>
       <c r="Y27" s="6" t="n"/>
+      <c r="Z27" s="6" t="n"/>
+      <c r="AA27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -1508,8 +1582,8 @@
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
-      <c r="K28" s="5" t="n"/>
-      <c r="L28" s="5" t="n"/>
+      <c r="K28" s="3" t="n"/>
+      <c r="L28" s="3" t="n"/>
       <c r="M28" s="5" t="n"/>
       <c r="N28" s="5" t="n"/>
       <c r="O28" s="5" t="n"/>
@@ -1523,6 +1597,8 @@
       <c r="W28" s="5" t="n"/>
       <c r="X28" s="5" t="n"/>
       <c r="Y28" s="5" t="n"/>
+      <c r="Z28" s="5" t="n"/>
+      <c r="AA28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n"/>
@@ -1550,6 +1626,8 @@
       <c r="W29" s="6" t="n"/>
       <c r="X29" s="6" t="n"/>
       <c r="Y29" s="6" t="n"/>
+      <c r="Z29" s="6" t="n"/>
+      <c r="AA29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -1562,8 +1640,8 @@
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
-      <c r="K30" s="5" t="n"/>
-      <c r="L30" s="5" t="n"/>
+      <c r="K30" s="3" t="n"/>
+      <c r="L30" s="3" t="n"/>
       <c r="M30" s="5" t="n"/>
       <c r="N30" s="5" t="n"/>
       <c r="O30" s="5" t="n"/>
@@ -1577,6 +1655,8 @@
       <c r="W30" s="5" t="n"/>
       <c r="X30" s="5" t="n"/>
       <c r="Y30" s="5" t="n"/>
+      <c r="Z30" s="5" t="n"/>
+      <c r="AA30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n"/>
@@ -1604,6 +1684,8 @@
       <c r="W31" s="6" t="n"/>
       <c r="X31" s="6" t="n"/>
       <c r="Y31" s="6" t="n"/>
+      <c r="Z31" s="6" t="n"/>
+      <c r="AA31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -1616,8 +1698,8 @@
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
-      <c r="K32" s="5" t="n"/>
-      <c r="L32" s="5" t="n"/>
+      <c r="K32" s="3" t="n"/>
+      <c r="L32" s="3" t="n"/>
       <c r="M32" s="5" t="n"/>
       <c r="N32" s="5" t="n"/>
       <c r="O32" s="5" t="n"/>
@@ -1631,6 +1713,8 @@
       <c r="W32" s="5" t="n"/>
       <c r="X32" s="5" t="n"/>
       <c r="Y32" s="5" t="n"/>
+      <c r="Z32" s="5" t="n"/>
+      <c r="AA32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
@@ -1658,6 +1742,8 @@
       <c r="W33" s="6" t="n"/>
       <c r="X33" s="6" t="n"/>
       <c r="Y33" s="6" t="n"/>
+      <c r="Z33" s="6" t="n"/>
+      <c r="AA33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -1670,8 +1756,8 @@
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
-      <c r="K34" s="5" t="n"/>
-      <c r="L34" s="5" t="n"/>
+      <c r="K34" s="3" t="n"/>
+      <c r="L34" s="3" t="n"/>
       <c r="M34" s="5" t="n"/>
       <c r="N34" s="5" t="n"/>
       <c r="O34" s="5" t="n"/>
@@ -1685,6 +1771,8 @@
       <c r="W34" s="5" t="n"/>
       <c r="X34" s="5" t="n"/>
       <c r="Y34" s="5" t="n"/>
+      <c r="Z34" s="5" t="n"/>
+      <c r="AA34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
@@ -1712,6 +1800,8 @@
       <c r="W35" s="6" t="n"/>
       <c r="X35" s="6" t="n"/>
       <c r="Y35" s="6" t="n"/>
+      <c r="Z35" s="6" t="n"/>
+      <c r="AA35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -1724,8 +1814,8 @@
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
-      <c r="K36" s="5" t="n"/>
-      <c r="L36" s="5" t="n"/>
+      <c r="K36" s="3" t="n"/>
+      <c r="L36" s="3" t="n"/>
       <c r="M36" s="5" t="n"/>
       <c r="N36" s="5" t="n"/>
       <c r="O36" s="5" t="n"/>
@@ -1739,6 +1829,8 @@
       <c r="W36" s="5" t="n"/>
       <c r="X36" s="5" t="n"/>
       <c r="Y36" s="5" t="n"/>
+      <c r="Z36" s="5" t="n"/>
+      <c r="AA36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n"/>
@@ -1766,6 +1858,8 @@
       <c r="W37" s="6" t="n"/>
       <c r="X37" s="6" t="n"/>
       <c r="Y37" s="6" t="n"/>
+      <c r="Z37" s="6" t="n"/>
+      <c r="AA37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -1778,8 +1872,8 @@
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
-      <c r="K38" s="5" t="n"/>
-      <c r="L38" s="5" t="n"/>
+      <c r="K38" s="3" t="n"/>
+      <c r="L38" s="3" t="n"/>
       <c r="M38" s="5" t="n"/>
       <c r="N38" s="5" t="n"/>
       <c r="O38" s="5" t="n"/>
@@ -1793,6 +1887,8 @@
       <c r="W38" s="5" t="n"/>
       <c r="X38" s="5" t="n"/>
       <c r="Y38" s="5" t="n"/>
+      <c r="Z38" s="5" t="n"/>
+      <c r="AA38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
@@ -1820,6 +1916,8 @@
       <c r="W39" s="6" t="n"/>
       <c r="X39" s="6" t="n"/>
       <c r="Y39" s="6" t="n"/>
+      <c r="Z39" s="6" t="n"/>
+      <c r="AA39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -1832,8 +1930,8 @@
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
-      <c r="K40" s="5" t="n"/>
-      <c r="L40" s="5" t="n"/>
+      <c r="K40" s="3" t="n"/>
+      <c r="L40" s="3" t="n"/>
       <c r="M40" s="5" t="n"/>
       <c r="N40" s="5" t="n"/>
       <c r="O40" s="5" t="n"/>
@@ -1847,6 +1945,8 @@
       <c r="W40" s="5" t="n"/>
       <c r="X40" s="5" t="n"/>
       <c r="Y40" s="5" t="n"/>
+      <c r="Z40" s="5" t="n"/>
+      <c r="AA40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n"/>
@@ -1874,6 +1974,8 @@
       <c r="W41" s="6" t="n"/>
       <c r="X41" s="6" t="n"/>
       <c r="Y41" s="6" t="n"/>
+      <c r="Z41" s="6" t="n"/>
+      <c r="AA41" s="6" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -1886,8 +1988,8 @@
       <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="3" t="n"/>
-      <c r="K42" s="5" t="n"/>
-      <c r="L42" s="5" t="n"/>
+      <c r="K42" s="3" t="n"/>
+      <c r="L42" s="3" t="n"/>
       <c r="M42" s="5" t="n"/>
       <c r="N42" s="5" t="n"/>
       <c r="O42" s="5" t="n"/>
@@ -1901,6 +2003,8 @@
       <c r="W42" s="5" t="n"/>
       <c r="X42" s="5" t="n"/>
       <c r="Y42" s="5" t="n"/>
+      <c r="Z42" s="5" t="n"/>
+      <c r="AA42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n"/>
@@ -1928,6 +2032,8 @@
       <c r="W43" s="6" t="n"/>
       <c r="X43" s="6" t="n"/>
       <c r="Y43" s="6" t="n"/>
+      <c r="Z43" s="6" t="n"/>
+      <c r="AA43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
@@ -1940,8 +2046,8 @@
       <c r="H44" s="3" t="n"/>
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="3" t="n"/>
-      <c r="K44" s="5" t="n"/>
-      <c r="L44" s="5" t="n"/>
+      <c r="K44" s="3" t="n"/>
+      <c r="L44" s="3" t="n"/>
       <c r="M44" s="5" t="n"/>
       <c r="N44" s="5" t="n"/>
       <c r="O44" s="5" t="n"/>
@@ -1955,6 +2061,8 @@
       <c r="W44" s="5" t="n"/>
       <c r="X44" s="5" t="n"/>
       <c r="Y44" s="5" t="n"/>
+      <c r="Z44" s="5" t="n"/>
+      <c r="AA44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n"/>
@@ -1982,6 +2090,8 @@
       <c r="W45" s="6" t="n"/>
       <c r="X45" s="6" t="n"/>
       <c r="Y45" s="6" t="n"/>
+      <c r="Z45" s="6" t="n"/>
+      <c r="AA45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
@@ -1994,8 +2104,8 @@
       <c r="H46" s="3" t="n"/>
       <c r="I46" s="3" t="n"/>
       <c r="J46" s="3" t="n"/>
-      <c r="K46" s="5" t="n"/>
-      <c r="L46" s="5" t="n"/>
+      <c r="K46" s="3" t="n"/>
+      <c r="L46" s="3" t="n"/>
       <c r="M46" s="5" t="n"/>
       <c r="N46" s="5" t="n"/>
       <c r="O46" s="5" t="n"/>
@@ -2009,6 +2119,8 @@
       <c r="W46" s="5" t="n"/>
       <c r="X46" s="5" t="n"/>
       <c r="Y46" s="5" t="n"/>
+      <c r="Z46" s="5" t="n"/>
+      <c r="AA46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n"/>
@@ -2036,6 +2148,8 @@
       <c r="W47" s="6" t="n"/>
       <c r="X47" s="6" t="n"/>
       <c r="Y47" s="6" t="n"/>
+      <c r="Z47" s="6" t="n"/>
+      <c r="AA47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -2048,8 +2162,8 @@
       <c r="H48" s="3" t="n"/>
       <c r="I48" s="3" t="n"/>
       <c r="J48" s="3" t="n"/>
-      <c r="K48" s="5" t="n"/>
-      <c r="L48" s="5" t="n"/>
+      <c r="K48" s="3" t="n"/>
+      <c r="L48" s="3" t="n"/>
       <c r="M48" s="5" t="n"/>
       <c r="N48" s="5" t="n"/>
       <c r="O48" s="5" t="n"/>
@@ -2063,6 +2177,8 @@
       <c r="W48" s="5" t="n"/>
       <c r="X48" s="5" t="n"/>
       <c r="Y48" s="5" t="n"/>
+      <c r="Z48" s="5" t="n"/>
+      <c r="AA48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n"/>
@@ -2090,6 +2206,8 @@
       <c r="W49" s="6" t="n"/>
       <c r="X49" s="6" t="n"/>
       <c r="Y49" s="6" t="n"/>
+      <c r="Z49" s="6" t="n"/>
+      <c r="AA49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
@@ -2102,8 +2220,8 @@
       <c r="H50" s="3" t="n"/>
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="3" t="n"/>
-      <c r="K50" s="5" t="n"/>
-      <c r="L50" s="5" t="n"/>
+      <c r="K50" s="3" t="n"/>
+      <c r="L50" s="3" t="n"/>
       <c r="M50" s="5" t="n"/>
       <c r="N50" s="5" t="n"/>
       <c r="O50" s="5" t="n"/>
@@ -2117,6 +2235,8 @@
       <c r="W50" s="5" t="n"/>
       <c r="X50" s="5" t="n"/>
       <c r="Y50" s="5" t="n"/>
+      <c r="Z50" s="5" t="n"/>
+      <c r="AA50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n"/>
@@ -2144,6 +2264,8 @@
       <c r="W51" s="6" t="n"/>
       <c r="X51" s="6" t="n"/>
       <c r="Y51" s="6" t="n"/>
+      <c r="Z51" s="6" t="n"/>
+      <c r="AA51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -2156,8 +2278,8 @@
       <c r="H52" s="3" t="n"/>
       <c r="I52" s="3" t="n"/>
       <c r="J52" s="3" t="n"/>
-      <c r="K52" s="5" t="n"/>
-      <c r="L52" s="5" t="n"/>
+      <c r="K52" s="3" t="n"/>
+      <c r="L52" s="3" t="n"/>
       <c r="M52" s="5" t="n"/>
       <c r="N52" s="5" t="n"/>
       <c r="O52" s="5" t="n"/>
@@ -2171,6 +2293,8 @@
       <c r="W52" s="5" t="n"/>
       <c r="X52" s="5" t="n"/>
       <c r="Y52" s="5" t="n"/>
+      <c r="Z52" s="5" t="n"/>
+      <c r="AA52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n"/>
@@ -2198,6 +2322,8 @@
       <c r="W53" s="6" t="n"/>
       <c r="X53" s="6" t="n"/>
       <c r="Y53" s="6" t="n"/>
+      <c r="Z53" s="6" t="n"/>
+      <c r="AA53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
@@ -2210,8 +2336,8 @@
       <c r="H54" s="3" t="n"/>
       <c r="I54" s="3" t="n"/>
       <c r="J54" s="3" t="n"/>
-      <c r="K54" s="5" t="n"/>
-      <c r="L54" s="5" t="n"/>
+      <c r="K54" s="3" t="n"/>
+      <c r="L54" s="3" t="n"/>
       <c r="M54" s="5" t="n"/>
       <c r="N54" s="5" t="n"/>
       <c r="O54" s="5" t="n"/>
@@ -2225,6 +2351,8 @@
       <c r="W54" s="5" t="n"/>
       <c r="X54" s="5" t="n"/>
       <c r="Y54" s="5" t="n"/>
+      <c r="Z54" s="5" t="n"/>
+      <c r="AA54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n"/>
@@ -2252,6 +2380,8 @@
       <c r="W55" s="6" t="n"/>
       <c r="X55" s="6" t="n"/>
       <c r="Y55" s="6" t="n"/>
+      <c r="Z55" s="6" t="n"/>
+      <c r="AA55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
@@ -2264,8 +2394,8 @@
       <c r="H56" s="3" t="n"/>
       <c r="I56" s="3" t="n"/>
       <c r="J56" s="3" t="n"/>
-      <c r="K56" s="5" t="n"/>
-      <c r="L56" s="5" t="n"/>
+      <c r="K56" s="3" t="n"/>
+      <c r="L56" s="3" t="n"/>
       <c r="M56" s="5" t="n"/>
       <c r="N56" s="5" t="n"/>
       <c r="O56" s="5" t="n"/>
@@ -2279,6 +2409,8 @@
       <c r="W56" s="5" t="n"/>
       <c r="X56" s="5" t="n"/>
       <c r="Y56" s="5" t="n"/>
+      <c r="Z56" s="5" t="n"/>
+      <c r="AA56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="n"/>
@@ -2306,6 +2438,8 @@
       <c r="W57" s="6" t="n"/>
       <c r="X57" s="6" t="n"/>
       <c r="Y57" s="6" t="n"/>
+      <c r="Z57" s="6" t="n"/>
+      <c r="AA57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
@@ -2318,8 +2452,8 @@
       <c r="H58" s="3" t="n"/>
       <c r="I58" s="3" t="n"/>
       <c r="J58" s="3" t="n"/>
-      <c r="K58" s="5" t="n"/>
-      <c r="L58" s="5" t="n"/>
+      <c r="K58" s="3" t="n"/>
+      <c r="L58" s="3" t="n"/>
       <c r="M58" s="5" t="n"/>
       <c r="N58" s="5" t="n"/>
       <c r="O58" s="5" t="n"/>
@@ -2333,6 +2467,8 @@
       <c r="W58" s="5" t="n"/>
       <c r="X58" s="5" t="n"/>
       <c r="Y58" s="5" t="n"/>
+      <c r="Z58" s="5" t="n"/>
+      <c r="AA58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="6" t="n"/>
@@ -2360,6 +2496,8 @@
       <c r="W59" s="6" t="n"/>
       <c r="X59" s="6" t="n"/>
       <c r="Y59" s="6" t="n"/>
+      <c r="Z59" s="6" t="n"/>
+      <c r="AA59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
@@ -2372,8 +2510,8 @@
       <c r="H60" s="3" t="n"/>
       <c r="I60" s="3" t="n"/>
       <c r="J60" s="3" t="n"/>
-      <c r="K60" s="5" t="n"/>
-      <c r="L60" s="5" t="n"/>
+      <c r="K60" s="3" t="n"/>
+      <c r="L60" s="3" t="n"/>
       <c r="M60" s="5" t="n"/>
       <c r="N60" s="5" t="n"/>
       <c r="O60" s="5" t="n"/>
@@ -2387,6 +2525,8 @@
       <c r="W60" s="5" t="n"/>
       <c r="X60" s="5" t="n"/>
       <c r="Y60" s="5" t="n"/>
+      <c r="Z60" s="5" t="n"/>
+      <c r="AA60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="6" t="n"/>
@@ -2414,6 +2554,8 @@
       <c r="W61" s="6" t="n"/>
       <c r="X61" s="6" t="n"/>
       <c r="Y61" s="6" t="n"/>
+      <c r="Z61" s="6" t="n"/>
+      <c r="AA61" s="6" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
@@ -2426,8 +2568,8 @@
       <c r="H62" s="3" t="n"/>
       <c r="I62" s="3" t="n"/>
       <c r="J62" s="3" t="n"/>
-      <c r="K62" s="5" t="n"/>
-      <c r="L62" s="5" t="n"/>
+      <c r="K62" s="3" t="n"/>
+      <c r="L62" s="3" t="n"/>
       <c r="M62" s="5" t="n"/>
       <c r="N62" s="5" t="n"/>
       <c r="O62" s="5" t="n"/>
@@ -2441,6 +2583,8 @@
       <c r="W62" s="5" t="n"/>
       <c r="X62" s="5" t="n"/>
       <c r="Y62" s="5" t="n"/>
+      <c r="Z62" s="5" t="n"/>
+      <c r="AA62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="6" t="n"/>
@@ -2468,6 +2612,8 @@
       <c r="W63" s="6" t="n"/>
       <c r="X63" s="6" t="n"/>
       <c r="Y63" s="6" t="n"/>
+      <c r="Z63" s="6" t="n"/>
+      <c r="AA63" s="6" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
@@ -2480,8 +2626,8 @@
       <c r="H64" s="3" t="n"/>
       <c r="I64" s="3" t="n"/>
       <c r="J64" s="3" t="n"/>
-      <c r="K64" s="5" t="n"/>
-      <c r="L64" s="5" t="n"/>
+      <c r="K64" s="3" t="n"/>
+      <c r="L64" s="3" t="n"/>
       <c r="M64" s="5" t="n"/>
       <c r="N64" s="5" t="n"/>
       <c r="O64" s="5" t="n"/>
@@ -2495,6 +2641,8 @@
       <c r="W64" s="5" t="n"/>
       <c r="X64" s="5" t="n"/>
       <c r="Y64" s="5" t="n"/>
+      <c r="Z64" s="5" t="n"/>
+      <c r="AA64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="n"/>
@@ -2522,6 +2670,8 @@
       <c r="W65" s="6" t="n"/>
       <c r="X65" s="6" t="n"/>
       <c r="Y65" s="6" t="n"/>
+      <c r="Z65" s="6" t="n"/>
+      <c r="AA65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -2534,8 +2684,8 @@
       <c r="H66" s="3" t="n"/>
       <c r="I66" s="3" t="n"/>
       <c r="J66" s="3" t="n"/>
-      <c r="K66" s="5" t="n"/>
-      <c r="L66" s="5" t="n"/>
+      <c r="K66" s="3" t="n"/>
+      <c r="L66" s="3" t="n"/>
       <c r="M66" s="5" t="n"/>
       <c r="N66" s="5" t="n"/>
       <c r="O66" s="5" t="n"/>
@@ -2549,6 +2699,8 @@
       <c r="W66" s="5" t="n"/>
       <c r="X66" s="5" t="n"/>
       <c r="Y66" s="5" t="n"/>
+      <c r="Z66" s="5" t="n"/>
+      <c r="AA66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="6" t="n"/>
@@ -2576,6 +2728,8 @@
       <c r="W67" s="6" t="n"/>
       <c r="X67" s="6" t="n"/>
       <c r="Y67" s="6" t="n"/>
+      <c r="Z67" s="6" t="n"/>
+      <c r="AA67" s="6" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
@@ -2588,8 +2742,8 @@
       <c r="H68" s="3" t="n"/>
       <c r="I68" s="3" t="n"/>
       <c r="J68" s="3" t="n"/>
-      <c r="K68" s="5" t="n"/>
-      <c r="L68" s="5" t="n"/>
+      <c r="K68" s="3" t="n"/>
+      <c r="L68" s="3" t="n"/>
       <c r="M68" s="5" t="n"/>
       <c r="N68" s="5" t="n"/>
       <c r="O68" s="5" t="n"/>
@@ -2603,6 +2757,8 @@
       <c r="W68" s="5" t="n"/>
       <c r="X68" s="5" t="n"/>
       <c r="Y68" s="5" t="n"/>
+      <c r="Z68" s="5" t="n"/>
+      <c r="AA68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="n"/>
@@ -2630,6 +2786,8 @@
       <c r="W69" s="6" t="n"/>
       <c r="X69" s="6" t="n"/>
       <c r="Y69" s="6" t="n"/>
+      <c r="Z69" s="6" t="n"/>
+      <c r="AA69" s="6" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n"/>
@@ -2642,8 +2800,8 @@
       <c r="H70" s="3" t="n"/>
       <c r="I70" s="3" t="n"/>
       <c r="J70" s="3" t="n"/>
-      <c r="K70" s="5" t="n"/>
-      <c r="L70" s="5" t="n"/>
+      <c r="K70" s="3" t="n"/>
+      <c r="L70" s="3" t="n"/>
       <c r="M70" s="5" t="n"/>
       <c r="N70" s="5" t="n"/>
       <c r="O70" s="5" t="n"/>
@@ -2657,6 +2815,8 @@
       <c r="W70" s="5" t="n"/>
       <c r="X70" s="5" t="n"/>
       <c r="Y70" s="5" t="n"/>
+      <c r="Z70" s="5" t="n"/>
+      <c r="AA70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n"/>
@@ -2684,6 +2844,8 @@
       <c r="W71" s="6" t="n"/>
       <c r="X71" s="6" t="n"/>
       <c r="Y71" s="6" t="n"/>
+      <c r="Z71" s="6" t="n"/>
+      <c r="AA71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n"/>
@@ -2696,8 +2858,8 @@
       <c r="H72" s="3" t="n"/>
       <c r="I72" s="3" t="n"/>
       <c r="J72" s="3" t="n"/>
-      <c r="K72" s="5" t="n"/>
-      <c r="L72" s="5" t="n"/>
+      <c r="K72" s="3" t="n"/>
+      <c r="L72" s="3" t="n"/>
       <c r="M72" s="5" t="n"/>
       <c r="N72" s="5" t="n"/>
       <c r="O72" s="5" t="n"/>
@@ -2711,6 +2873,8 @@
       <c r="W72" s="5" t="n"/>
       <c r="X72" s="5" t="n"/>
       <c r="Y72" s="5" t="n"/>
+      <c r="Z72" s="5" t="n"/>
+      <c r="AA72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="n"/>
@@ -2738,6 +2902,8 @@
       <c r="W73" s="6" t="n"/>
       <c r="X73" s="6" t="n"/>
       <c r="Y73" s="6" t="n"/>
+      <c r="Z73" s="6" t="n"/>
+      <c r="AA73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n"/>
@@ -2750,8 +2916,8 @@
       <c r="H74" s="3" t="n"/>
       <c r="I74" s="3" t="n"/>
       <c r="J74" s="3" t="n"/>
-      <c r="K74" s="5" t="n"/>
-      <c r="L74" s="5" t="n"/>
+      <c r="K74" s="3" t="n"/>
+      <c r="L74" s="3" t="n"/>
       <c r="M74" s="5" t="n"/>
       <c r="N74" s="5" t="n"/>
       <c r="O74" s="5" t="n"/>
@@ -2765,6 +2931,8 @@
       <c r="W74" s="5" t="n"/>
       <c r="X74" s="5" t="n"/>
       <c r="Y74" s="5" t="n"/>
+      <c r="Z74" s="5" t="n"/>
+      <c r="AA74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n"/>
@@ -2792,6 +2960,8 @@
       <c r="W75" s="6" t="n"/>
       <c r="X75" s="6" t="n"/>
       <c r="Y75" s="6" t="n"/>
+      <c r="Z75" s="6" t="n"/>
+      <c r="AA75" s="6" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n"/>
@@ -2804,8 +2974,8 @@
       <c r="H76" s="3" t="n"/>
       <c r="I76" s="3" t="n"/>
       <c r="J76" s="3" t="n"/>
-      <c r="K76" s="5" t="n"/>
-      <c r="L76" s="5" t="n"/>
+      <c r="K76" s="3" t="n"/>
+      <c r="L76" s="3" t="n"/>
       <c r="M76" s="5" t="n"/>
       <c r="N76" s="5" t="n"/>
       <c r="O76" s="5" t="n"/>
@@ -2819,6 +2989,8 @@
       <c r="W76" s="5" t="n"/>
       <c r="X76" s="5" t="n"/>
       <c r="Y76" s="5" t="n"/>
+      <c r="Z76" s="5" t="n"/>
+      <c r="AA76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="6" t="n"/>
@@ -2846,6 +3018,8 @@
       <c r="W77" s="6" t="n"/>
       <c r="X77" s="6" t="n"/>
       <c r="Y77" s="6" t="n"/>
+      <c r="Z77" s="6" t="n"/>
+      <c r="AA77" s="6" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n"/>
@@ -2858,8 +3032,8 @@
       <c r="H78" s="3" t="n"/>
       <c r="I78" s="3" t="n"/>
       <c r="J78" s="3" t="n"/>
-      <c r="K78" s="5" t="n"/>
-      <c r="L78" s="5" t="n"/>
+      <c r="K78" s="3" t="n"/>
+      <c r="L78" s="3" t="n"/>
       <c r="M78" s="5" t="n"/>
       <c r="N78" s="5" t="n"/>
       <c r="O78" s="5" t="n"/>
@@ -2873,6 +3047,8 @@
       <c r="W78" s="5" t="n"/>
       <c r="X78" s="5" t="n"/>
       <c r="Y78" s="5" t="n"/>
+      <c r="Z78" s="5" t="n"/>
+      <c r="AA78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="n"/>
@@ -2900,6 +3076,8 @@
       <c r="W79" s="6" t="n"/>
       <c r="X79" s="6" t="n"/>
       <c r="Y79" s="6" t="n"/>
+      <c r="Z79" s="6" t="n"/>
+      <c r="AA79" s="6" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n"/>
@@ -2912,8 +3090,8 @@
       <c r="H80" s="3" t="n"/>
       <c r="I80" s="3" t="n"/>
       <c r="J80" s="3" t="n"/>
-      <c r="K80" s="5" t="n"/>
-      <c r="L80" s="5" t="n"/>
+      <c r="K80" s="3" t="n"/>
+      <c r="L80" s="3" t="n"/>
       <c r="M80" s="5" t="n"/>
       <c r="N80" s="5" t="n"/>
       <c r="O80" s="5" t="n"/>
@@ -2927,6 +3105,8 @@
       <c r="W80" s="5" t="n"/>
       <c r="X80" s="5" t="n"/>
       <c r="Y80" s="5" t="n"/>
+      <c r="Z80" s="5" t="n"/>
+      <c r="AA80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="n"/>
@@ -2954,6 +3134,8 @@
       <c r="W81" s="6" t="n"/>
       <c r="X81" s="6" t="n"/>
       <c r="Y81" s="6" t="n"/>
+      <c r="Z81" s="6" t="n"/>
+      <c r="AA81" s="6" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n"/>
@@ -2966,8 +3148,8 @@
       <c r="H82" s="3" t="n"/>
       <c r="I82" s="3" t="n"/>
       <c r="J82" s="3" t="n"/>
-      <c r="K82" s="5" t="n"/>
-      <c r="L82" s="5" t="n"/>
+      <c r="K82" s="3" t="n"/>
+      <c r="L82" s="3" t="n"/>
       <c r="M82" s="5" t="n"/>
       <c r="N82" s="5" t="n"/>
       <c r="O82" s="5" t="n"/>
@@ -2981,6 +3163,8 @@
       <c r="W82" s="5" t="n"/>
       <c r="X82" s="5" t="n"/>
       <c r="Y82" s="5" t="n"/>
+      <c r="Z82" s="5" t="n"/>
+      <c r="AA82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="6" t="n"/>
@@ -3008,6 +3192,8 @@
       <c r="W83" s="6" t="n"/>
       <c r="X83" s="6" t="n"/>
       <c r="Y83" s="6" t="n"/>
+      <c r="Z83" s="6" t="n"/>
+      <c r="AA83" s="6" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n"/>
@@ -3020,8 +3206,8 @@
       <c r="H84" s="3" t="n"/>
       <c r="I84" s="3" t="n"/>
       <c r="J84" s="3" t="n"/>
-      <c r="K84" s="5" t="n"/>
-      <c r="L84" s="5" t="n"/>
+      <c r="K84" s="3" t="n"/>
+      <c r="L84" s="3" t="n"/>
       <c r="M84" s="5" t="n"/>
       <c r="N84" s="5" t="n"/>
       <c r="O84" s="5" t="n"/>
@@ -3035,6 +3221,8 @@
       <c r="W84" s="5" t="n"/>
       <c r="X84" s="5" t="n"/>
       <c r="Y84" s="5" t="n"/>
+      <c r="Z84" s="5" t="n"/>
+      <c r="AA84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="n"/>
@@ -3062,6 +3250,8 @@
       <c r="W85" s="6" t="n"/>
       <c r="X85" s="6" t="n"/>
       <c r="Y85" s="6" t="n"/>
+      <c r="Z85" s="6" t="n"/>
+      <c r="AA85" s="6" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n"/>
@@ -3074,8 +3264,8 @@
       <c r="H86" s="3" t="n"/>
       <c r="I86" s="3" t="n"/>
       <c r="J86" s="3" t="n"/>
-      <c r="K86" s="5" t="n"/>
-      <c r="L86" s="5" t="n"/>
+      <c r="K86" s="3" t="n"/>
+      <c r="L86" s="3" t="n"/>
       <c r="M86" s="5" t="n"/>
       <c r="N86" s="5" t="n"/>
       <c r="O86" s="5" t="n"/>
@@ -3089,6 +3279,8 @@
       <c r="W86" s="5" t="n"/>
       <c r="X86" s="5" t="n"/>
       <c r="Y86" s="5" t="n"/>
+      <c r="Z86" s="5" t="n"/>
+      <c r="AA86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="6" t="n"/>
@@ -3116,6 +3308,8 @@
       <c r="W87" s="6" t="n"/>
       <c r="X87" s="6" t="n"/>
       <c r="Y87" s="6" t="n"/>
+      <c r="Z87" s="6" t="n"/>
+      <c r="AA87" s="6" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n"/>
@@ -3128,8 +3322,8 @@
       <c r="H88" s="3" t="n"/>
       <c r="I88" s="3" t="n"/>
       <c r="J88" s="3" t="n"/>
-      <c r="K88" s="5" t="n"/>
-      <c r="L88" s="5" t="n"/>
+      <c r="K88" s="3" t="n"/>
+      <c r="L88" s="3" t="n"/>
       <c r="M88" s="5" t="n"/>
       <c r="N88" s="5" t="n"/>
       <c r="O88" s="5" t="n"/>
@@ -3143,6 +3337,8 @@
       <c r="W88" s="5" t="n"/>
       <c r="X88" s="5" t="n"/>
       <c r="Y88" s="5" t="n"/>
+      <c r="Z88" s="5" t="n"/>
+      <c r="AA88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="n"/>
@@ -3170,6 +3366,8 @@
       <c r="W89" s="6" t="n"/>
       <c r="X89" s="6" t="n"/>
       <c r="Y89" s="6" t="n"/>
+      <c r="Z89" s="6" t="n"/>
+      <c r="AA89" s="6" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n"/>
@@ -3182,8 +3380,8 @@
       <c r="H90" s="3" t="n"/>
       <c r="I90" s="3" t="n"/>
       <c r="J90" s="3" t="n"/>
-      <c r="K90" s="5" t="n"/>
-      <c r="L90" s="5" t="n"/>
+      <c r="K90" s="3" t="n"/>
+      <c r="L90" s="3" t="n"/>
       <c r="M90" s="5" t="n"/>
       <c r="N90" s="5" t="n"/>
       <c r="O90" s="5" t="n"/>
@@ -3197,6 +3395,8 @@
       <c r="W90" s="5" t="n"/>
       <c r="X90" s="5" t="n"/>
       <c r="Y90" s="5" t="n"/>
+      <c r="Z90" s="5" t="n"/>
+      <c r="AA90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="6" t="n"/>
@@ -3224,6 +3424,8 @@
       <c r="W91" s="6" t="n"/>
       <c r="X91" s="6" t="n"/>
       <c r="Y91" s="6" t="n"/>
+      <c r="Z91" s="6" t="n"/>
+      <c r="AA91" s="6" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n"/>
@@ -3236,8 +3438,8 @@
       <c r="H92" s="3" t="n"/>
       <c r="I92" s="3" t="n"/>
       <c r="J92" s="3" t="n"/>
-      <c r="K92" s="5" t="n"/>
-      <c r="L92" s="5" t="n"/>
+      <c r="K92" s="3" t="n"/>
+      <c r="L92" s="3" t="n"/>
       <c r="M92" s="5" t="n"/>
       <c r="N92" s="5" t="n"/>
       <c r="O92" s="5" t="n"/>
@@ -3251,6 +3453,8 @@
       <c r="W92" s="5" t="n"/>
       <c r="X92" s="5" t="n"/>
       <c r="Y92" s="5" t="n"/>
+      <c r="Z92" s="5" t="n"/>
+      <c r="AA92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="6" t="n"/>
@@ -3278,6 +3482,8 @@
       <c r="W93" s="6" t="n"/>
       <c r="X93" s="6" t="n"/>
       <c r="Y93" s="6" t="n"/>
+      <c r="Z93" s="6" t="n"/>
+      <c r="AA93" s="6" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n"/>
@@ -3290,8 +3496,8 @@
       <c r="H94" s="3" t="n"/>
       <c r="I94" s="3" t="n"/>
       <c r="J94" s="3" t="n"/>
-      <c r="K94" s="5" t="n"/>
-      <c r="L94" s="5" t="n"/>
+      <c r="K94" s="3" t="n"/>
+      <c r="L94" s="3" t="n"/>
       <c r="M94" s="5" t="n"/>
       <c r="N94" s="5" t="n"/>
       <c r="O94" s="5" t="n"/>
@@ -3305,6 +3511,8 @@
       <c r="W94" s="5" t="n"/>
       <c r="X94" s="5" t="n"/>
       <c r="Y94" s="5" t="n"/>
+      <c r="Z94" s="5" t="n"/>
+      <c r="AA94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="6" t="n"/>
@@ -3332,6 +3540,8 @@
       <c r="W95" s="6" t="n"/>
       <c r="X95" s="6" t="n"/>
       <c r="Y95" s="6" t="n"/>
+      <c r="Z95" s="6" t="n"/>
+      <c r="AA95" s="6" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n"/>
@@ -3344,8 +3554,8 @@
       <c r="H96" s="3" t="n"/>
       <c r="I96" s="3" t="n"/>
       <c r="J96" s="3" t="n"/>
-      <c r="K96" s="5" t="n"/>
-      <c r="L96" s="5" t="n"/>
+      <c r="K96" s="3" t="n"/>
+      <c r="L96" s="3" t="n"/>
       <c r="M96" s="5" t="n"/>
       <c r="N96" s="5" t="n"/>
       <c r="O96" s="5" t="n"/>
@@ -3359,6 +3569,8 @@
       <c r="W96" s="5" t="n"/>
       <c r="X96" s="5" t="n"/>
       <c r="Y96" s="5" t="n"/>
+      <c r="Z96" s="5" t="n"/>
+      <c r="AA96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="6" t="n"/>
@@ -3386,6 +3598,8 @@
       <c r="W97" s="6" t="n"/>
       <c r="X97" s="6" t="n"/>
       <c r="Y97" s="6" t="n"/>
+      <c r="Z97" s="6" t="n"/>
+      <c r="AA97" s="6" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n"/>
@@ -3398,8 +3612,8 @@
       <c r="H98" s="3" t="n"/>
       <c r="I98" s="3" t="n"/>
       <c r="J98" s="3" t="n"/>
-      <c r="K98" s="5" t="n"/>
-      <c r="L98" s="5" t="n"/>
+      <c r="K98" s="3" t="n"/>
+      <c r="L98" s="3" t="n"/>
       <c r="M98" s="5" t="n"/>
       <c r="N98" s="5" t="n"/>
       <c r="O98" s="5" t="n"/>
@@ -3413,6 +3627,8 @@
       <c r="W98" s="5" t="n"/>
       <c r="X98" s="5" t="n"/>
       <c r="Y98" s="5" t="n"/>
+      <c r="Z98" s="5" t="n"/>
+      <c r="AA98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="6" t="n"/>
@@ -3440,6 +3656,8 @@
       <c r="W99" s="6" t="n"/>
       <c r="X99" s="6" t="n"/>
       <c r="Y99" s="6" t="n"/>
+      <c r="Z99" s="6" t="n"/>
+      <c r="AA99" s="6" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n"/>
@@ -3452,8 +3670,8 @@
       <c r="H100" s="3" t="n"/>
       <c r="I100" s="3" t="n"/>
       <c r="J100" s="3" t="n"/>
-      <c r="K100" s="5" t="n"/>
-      <c r="L100" s="5" t="n"/>
+      <c r="K100" s="3" t="n"/>
+      <c r="L100" s="3" t="n"/>
       <c r="M100" s="5" t="n"/>
       <c r="N100" s="5" t="n"/>
       <c r="O100" s="5" t="n"/>
@@ -3467,6 +3685,8 @@
       <c r="W100" s="5" t="n"/>
       <c r="X100" s="5" t="n"/>
       <c r="Y100" s="5" t="n"/>
+      <c r="Z100" s="5" t="n"/>
+      <c r="AA100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="6" t="n"/>
@@ -3494,6 +3714,8 @@
       <c r="W101" s="6" t="n"/>
       <c r="X101" s="6" t="n"/>
       <c r="Y101" s="6" t="n"/>
+      <c r="Z101" s="6" t="n"/>
+      <c r="AA101" s="6" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n"/>
@@ -3506,8 +3728,8 @@
       <c r="H102" s="3" t="n"/>
       <c r="I102" s="3" t="n"/>
       <c r="J102" s="3" t="n"/>
-      <c r="K102" s="5" t="n"/>
-      <c r="L102" s="5" t="n"/>
+      <c r="K102" s="3" t="n"/>
+      <c r="L102" s="3" t="n"/>
       <c r="M102" s="5" t="n"/>
       <c r="N102" s="5" t="n"/>
       <c r="O102" s="5" t="n"/>
@@ -3521,6 +3743,8 @@
       <c r="W102" s="5" t="n"/>
       <c r="X102" s="5" t="n"/>
       <c r="Y102" s="5" t="n"/>
+      <c r="Z102" s="5" t="n"/>
+      <c r="AA102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="6" t="n"/>
@@ -3548,6 +3772,8 @@
       <c r="W103" s="6" t="n"/>
       <c r="X103" s="6" t="n"/>
       <c r="Y103" s="6" t="n"/>
+      <c r="Z103" s="6" t="n"/>
+      <c r="AA103" s="6" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n"/>
@@ -3560,8 +3786,8 @@
       <c r="H104" s="3" t="n"/>
       <c r="I104" s="3" t="n"/>
       <c r="J104" s="3" t="n"/>
-      <c r="K104" s="5" t="n"/>
-      <c r="L104" s="5" t="n"/>
+      <c r="K104" s="3" t="n"/>
+      <c r="L104" s="3" t="n"/>
       <c r="M104" s="5" t="n"/>
       <c r="N104" s="5" t="n"/>
       <c r="O104" s="5" t="n"/>
@@ -3575,6 +3801,8 @@
       <c r="W104" s="5" t="n"/>
       <c r="X104" s="5" t="n"/>
       <c r="Y104" s="5" t="n"/>
+      <c r="Z104" s="5" t="n"/>
+      <c r="AA104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="6" t="n"/>
@@ -3602,6 +3830,8 @@
       <c r="W105" s="6" t="n"/>
       <c r="X105" s="6" t="n"/>
       <c r="Y105" s="6" t="n"/>
+      <c r="Z105" s="6" t="n"/>
+      <c r="AA105" s="6" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n"/>
@@ -3614,8 +3844,8 @@
       <c r="H106" s="3" t="n"/>
       <c r="I106" s="3" t="n"/>
       <c r="J106" s="3" t="n"/>
-      <c r="K106" s="5" t="n"/>
-      <c r="L106" s="5" t="n"/>
+      <c r="K106" s="3" t="n"/>
+      <c r="L106" s="3" t="n"/>
       <c r="M106" s="5" t="n"/>
       <c r="N106" s="5" t="n"/>
       <c r="O106" s="5" t="n"/>
@@ -3629,6 +3859,8 @@
       <c r="W106" s="5" t="n"/>
       <c r="X106" s="5" t="n"/>
       <c r="Y106" s="5" t="n"/>
+      <c r="Z106" s="5" t="n"/>
+      <c r="AA106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="6" t="n"/>
@@ -3656,6 +3888,8 @@
       <c r="W107" s="6" t="n"/>
       <c r="X107" s="6" t="n"/>
       <c r="Y107" s="6" t="n"/>
+      <c r="Z107" s="6" t="n"/>
+      <c r="AA107" s="6" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n"/>
@@ -3668,8 +3902,8 @@
       <c r="H108" s="3" t="n"/>
       <c r="I108" s="3" t="n"/>
       <c r="J108" s="3" t="n"/>
-      <c r="K108" s="5" t="n"/>
-      <c r="L108" s="5" t="n"/>
+      <c r="K108" s="3" t="n"/>
+      <c r="L108" s="3" t="n"/>
       <c r="M108" s="5" t="n"/>
       <c r="N108" s="5" t="n"/>
       <c r="O108" s="5" t="n"/>
@@ -3683,6 +3917,8 @@
       <c r="W108" s="5" t="n"/>
       <c r="X108" s="5" t="n"/>
       <c r="Y108" s="5" t="n"/>
+      <c r="Z108" s="5" t="n"/>
+      <c r="AA108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="6" t="n"/>
@@ -3710,6 +3946,8 @@
       <c r="W109" s="6" t="n"/>
       <c r="X109" s="6" t="n"/>
       <c r="Y109" s="6" t="n"/>
+      <c r="Z109" s="6" t="n"/>
+      <c r="AA109" s="6" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="3" t="n"/>
@@ -3722,8 +3960,8 @@
       <c r="H110" s="3" t="n"/>
       <c r="I110" s="3" t="n"/>
       <c r="J110" s="3" t="n"/>
-      <c r="K110" s="5" t="n"/>
-      <c r="L110" s="5" t="n"/>
+      <c r="K110" s="3" t="n"/>
+      <c r="L110" s="3" t="n"/>
       <c r="M110" s="5" t="n"/>
       <c r="N110" s="5" t="n"/>
       <c r="O110" s="5" t="n"/>
@@ -3737,6 +3975,8 @@
       <c r="W110" s="5" t="n"/>
       <c r="X110" s="5" t="n"/>
       <c r="Y110" s="5" t="n"/>
+      <c r="Z110" s="5" t="n"/>
+      <c r="AA110" s="5" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="6" t="n"/>
@@ -3764,6 +4004,8 @@
       <c r="W111" s="6" t="n"/>
       <c r="X111" s="6" t="n"/>
       <c r="Y111" s="6" t="n"/>
+      <c r="Z111" s="6" t="n"/>
+      <c r="AA111" s="6" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="3" t="n"/>
@@ -3776,8 +4018,8 @@
       <c r="H112" s="3" t="n"/>
       <c r="I112" s="3" t="n"/>
       <c r="J112" s="3" t="n"/>
-      <c r="K112" s="5" t="n"/>
-      <c r="L112" s="5" t="n"/>
+      <c r="K112" s="3" t="n"/>
+      <c r="L112" s="3" t="n"/>
       <c r="M112" s="5" t="n"/>
       <c r="N112" s="5" t="n"/>
       <c r="O112" s="5" t="n"/>
@@ -3791,6 +4033,8 @@
       <c r="W112" s="5" t="n"/>
       <c r="X112" s="5" t="n"/>
       <c r="Y112" s="5" t="n"/>
+      <c r="Z112" s="5" t="n"/>
+      <c r="AA112" s="5" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="6" t="n"/>
@@ -3818,6 +4062,8 @@
       <c r="W113" s="6" t="n"/>
       <c r="X113" s="6" t="n"/>
       <c r="Y113" s="6" t="n"/>
+      <c r="Z113" s="6" t="n"/>
+      <c r="AA113" s="6" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="n"/>
@@ -3830,8 +4076,8 @@
       <c r="H114" s="3" t="n"/>
       <c r="I114" s="3" t="n"/>
       <c r="J114" s="3" t="n"/>
-      <c r="K114" s="5" t="n"/>
-      <c r="L114" s="5" t="n"/>
+      <c r="K114" s="3" t="n"/>
+      <c r="L114" s="3" t="n"/>
       <c r="M114" s="5" t="n"/>
       <c r="N114" s="5" t="n"/>
       <c r="O114" s="5" t="n"/>
@@ -3845,6 +4091,8 @@
       <c r="W114" s="5" t="n"/>
       <c r="X114" s="5" t="n"/>
       <c r="Y114" s="5" t="n"/>
+      <c r="Z114" s="5" t="n"/>
+      <c r="AA114" s="5" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="6" t="n"/>
@@ -3872,6 +4120,8 @@
       <c r="W115" s="6" t="n"/>
       <c r="X115" s="6" t="n"/>
       <c r="Y115" s="6" t="n"/>
+      <c r="Z115" s="6" t="n"/>
+      <c r="AA115" s="6" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="3" t="n"/>
@@ -3884,8 +4134,8 @@
       <c r="H116" s="3" t="n"/>
       <c r="I116" s="3" t="n"/>
       <c r="J116" s="3" t="n"/>
-      <c r="K116" s="5" t="n"/>
-      <c r="L116" s="5" t="n"/>
+      <c r="K116" s="3" t="n"/>
+      <c r="L116" s="3" t="n"/>
       <c r="M116" s="5" t="n"/>
       <c r="N116" s="5" t="n"/>
       <c r="O116" s="5" t="n"/>
@@ -3899,6 +4149,8 @@
       <c r="W116" s="5" t="n"/>
       <c r="X116" s="5" t="n"/>
       <c r="Y116" s="5" t="n"/>
+      <c r="Z116" s="5" t="n"/>
+      <c r="AA116" s="5" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="6" t="n"/>
@@ -3926,6 +4178,8 @@
       <c r="W117" s="6" t="n"/>
       <c r="X117" s="6" t="n"/>
       <c r="Y117" s="6" t="n"/>
+      <c r="Z117" s="6" t="n"/>
+      <c r="AA117" s="6" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="3" t="n"/>
@@ -3938,8 +4192,8 @@
       <c r="H118" s="3" t="n"/>
       <c r="I118" s="3" t="n"/>
       <c r="J118" s="3" t="n"/>
-      <c r="K118" s="5" t="n"/>
-      <c r="L118" s="5" t="n"/>
+      <c r="K118" s="3" t="n"/>
+      <c r="L118" s="3" t="n"/>
       <c r="M118" s="5" t="n"/>
       <c r="N118" s="5" t="n"/>
       <c r="O118" s="5" t="n"/>
@@ -3953,6 +4207,8 @@
       <c r="W118" s="5" t="n"/>
       <c r="X118" s="5" t="n"/>
       <c r="Y118" s="5" t="n"/>
+      <c r="Z118" s="5" t="n"/>
+      <c r="AA118" s="5" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="6" t="n"/>
@@ -3980,6 +4236,8 @@
       <c r="W119" s="6" t="n"/>
       <c r="X119" s="6" t="n"/>
       <c r="Y119" s="6" t="n"/>
+      <c r="Z119" s="6" t="n"/>
+      <c r="AA119" s="6" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="3" t="n"/>
@@ -3992,8 +4250,8 @@
       <c r="H120" s="3" t="n"/>
       <c r="I120" s="3" t="n"/>
       <c r="J120" s="3" t="n"/>
-      <c r="K120" s="5" t="n"/>
-      <c r="L120" s="5" t="n"/>
+      <c r="K120" s="3" t="n"/>
+      <c r="L120" s="3" t="n"/>
       <c r="M120" s="5" t="n"/>
       <c r="N120" s="5" t="n"/>
       <c r="O120" s="5" t="n"/>
@@ -4007,6 +4265,8 @@
       <c r="W120" s="5" t="n"/>
       <c r="X120" s="5" t="n"/>
       <c r="Y120" s="5" t="n"/>
+      <c r="Z120" s="5" t="n"/>
+      <c r="AA120" s="5" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="6" t="n"/>
@@ -4034,6 +4294,8 @@
       <c r="W121" s="6" t="n"/>
       <c r="X121" s="6" t="n"/>
       <c r="Y121" s="6" t="n"/>
+      <c r="Z121" s="6" t="n"/>
+      <c r="AA121" s="6" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="3" t="n"/>
@@ -4046,8 +4308,8 @@
       <c r="H122" s="3" t="n"/>
       <c r="I122" s="3" t="n"/>
       <c r="J122" s="3" t="n"/>
-      <c r="K122" s="5" t="n"/>
-      <c r="L122" s="5" t="n"/>
+      <c r="K122" s="3" t="n"/>
+      <c r="L122" s="3" t="n"/>
       <c r="M122" s="5" t="n"/>
       <c r="N122" s="5" t="n"/>
       <c r="O122" s="5" t="n"/>
@@ -4061,6 +4323,8 @@
       <c r="W122" s="5" t="n"/>
       <c r="X122" s="5" t="n"/>
       <c r="Y122" s="5" t="n"/>
+      <c r="Z122" s="5" t="n"/>
+      <c r="AA122" s="5" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="6" t="n"/>
@@ -4088,6 +4352,8 @@
       <c r="W123" s="6" t="n"/>
       <c r="X123" s="6" t="n"/>
       <c r="Y123" s="6" t="n"/>
+      <c r="Z123" s="6" t="n"/>
+      <c r="AA123" s="6" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="3" t="n"/>
@@ -4100,8 +4366,8 @@
       <c r="H124" s="3" t="n"/>
       <c r="I124" s="3" t="n"/>
       <c r="J124" s="3" t="n"/>
-      <c r="K124" s="5" t="n"/>
-      <c r="L124" s="5" t="n"/>
+      <c r="K124" s="3" t="n"/>
+      <c r="L124" s="3" t="n"/>
       <c r="M124" s="5" t="n"/>
       <c r="N124" s="5" t="n"/>
       <c r="O124" s="5" t="n"/>
@@ -4115,6 +4381,8 @@
       <c r="W124" s="5" t="n"/>
       <c r="X124" s="5" t="n"/>
       <c r="Y124" s="5" t="n"/>
+      <c r="Z124" s="5" t="n"/>
+      <c r="AA124" s="5" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="6" t="n"/>
@@ -4142,6 +4410,8 @@
       <c r="W125" s="6" t="n"/>
       <c r="X125" s="6" t="n"/>
       <c r="Y125" s="6" t="n"/>
+      <c r="Z125" s="6" t="n"/>
+      <c r="AA125" s="6" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="3" t="n"/>
@@ -4154,8 +4424,8 @@
       <c r="H126" s="3" t="n"/>
       <c r="I126" s="3" t="n"/>
       <c r="J126" s="3" t="n"/>
-      <c r="K126" s="5" t="n"/>
-      <c r="L126" s="5" t="n"/>
+      <c r="K126" s="3" t="n"/>
+      <c r="L126" s="3" t="n"/>
       <c r="M126" s="5" t="n"/>
       <c r="N126" s="5" t="n"/>
       <c r="O126" s="5" t="n"/>
@@ -4169,6 +4439,8 @@
       <c r="W126" s="5" t="n"/>
       <c r="X126" s="5" t="n"/>
       <c r="Y126" s="5" t="n"/>
+      <c r="Z126" s="5" t="n"/>
+      <c r="AA126" s="5" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="6" t="n"/>
@@ -4196,6 +4468,8 @@
       <c r="W127" s="6" t="n"/>
       <c r="X127" s="6" t="n"/>
       <c r="Y127" s="6" t="n"/>
+      <c r="Z127" s="6" t="n"/>
+      <c r="AA127" s="6" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="3" t="n"/>
@@ -4208,8 +4482,8 @@
       <c r="H128" s="3" t="n"/>
       <c r="I128" s="3" t="n"/>
       <c r="J128" s="3" t="n"/>
-      <c r="K128" s="5" t="n"/>
-      <c r="L128" s="5" t="n"/>
+      <c r="K128" s="3" t="n"/>
+      <c r="L128" s="3" t="n"/>
       <c r="M128" s="5" t="n"/>
       <c r="N128" s="5" t="n"/>
       <c r="O128" s="5" t="n"/>
@@ -4223,6 +4497,8 @@
       <c r="W128" s="5" t="n"/>
       <c r="X128" s="5" t="n"/>
       <c r="Y128" s="5" t="n"/>
+      <c r="Z128" s="5" t="n"/>
+      <c r="AA128" s="5" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="6" t="n"/>
@@ -4250,6 +4526,8 @@
       <c r="W129" s="6" t="n"/>
       <c r="X129" s="6" t="n"/>
       <c r="Y129" s="6" t="n"/>
+      <c r="Z129" s="6" t="n"/>
+      <c r="AA129" s="6" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="3" t="n"/>
@@ -4262,8 +4540,8 @@
       <c r="H130" s="3" t="n"/>
       <c r="I130" s="3" t="n"/>
       <c r="J130" s="3" t="n"/>
-      <c r="K130" s="5" t="n"/>
-      <c r="L130" s="5" t="n"/>
+      <c r="K130" s="3" t="n"/>
+      <c r="L130" s="3" t="n"/>
       <c r="M130" s="5" t="n"/>
       <c r="N130" s="5" t="n"/>
       <c r="O130" s="5" t="n"/>
@@ -4277,6 +4555,8 @@
       <c r="W130" s="5" t="n"/>
       <c r="X130" s="5" t="n"/>
       <c r="Y130" s="5" t="n"/>
+      <c r="Z130" s="5" t="n"/>
+      <c r="AA130" s="5" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="6" t="n"/>
@@ -4304,6 +4584,8 @@
       <c r="W131" s="6" t="n"/>
       <c r="X131" s="6" t="n"/>
       <c r="Y131" s="6" t="n"/>
+      <c r="Z131" s="6" t="n"/>
+      <c r="AA131" s="6" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="3" t="n"/>
@@ -4316,8 +4598,8 @@
       <c r="H132" s="3" t="n"/>
       <c r="I132" s="3" t="n"/>
       <c r="J132" s="3" t="n"/>
-      <c r="K132" s="5" t="n"/>
-      <c r="L132" s="5" t="n"/>
+      <c r="K132" s="3" t="n"/>
+      <c r="L132" s="3" t="n"/>
       <c r="M132" s="5" t="n"/>
       <c r="N132" s="5" t="n"/>
       <c r="O132" s="5" t="n"/>
@@ -4331,6 +4613,8 @@
       <c r="W132" s="5" t="n"/>
       <c r="X132" s="5" t="n"/>
       <c r="Y132" s="5" t="n"/>
+      <c r="Z132" s="5" t="n"/>
+      <c r="AA132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="6" t="n"/>
@@ -4358,6 +4642,8 @@
       <c r="W133" s="6" t="n"/>
       <c r="X133" s="6" t="n"/>
       <c r="Y133" s="6" t="n"/>
+      <c r="Z133" s="6" t="n"/>
+      <c r="AA133" s="6" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="3" t="n"/>
@@ -4370,8 +4656,8 @@
       <c r="H134" s="3" t="n"/>
       <c r="I134" s="3" t="n"/>
       <c r="J134" s="3" t="n"/>
-      <c r="K134" s="5" t="n"/>
-      <c r="L134" s="5" t="n"/>
+      <c r="K134" s="3" t="n"/>
+      <c r="L134" s="3" t="n"/>
       <c r="M134" s="5" t="n"/>
       <c r="N134" s="5" t="n"/>
       <c r="O134" s="5" t="n"/>
@@ -4385,6 +4671,8 @@
       <c r="W134" s="5" t="n"/>
       <c r="X134" s="5" t="n"/>
       <c r="Y134" s="5" t="n"/>
+      <c r="Z134" s="5" t="n"/>
+      <c r="AA134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="6" t="n"/>
@@ -4412,6 +4700,8 @@
       <c r="W135" s="6" t="n"/>
       <c r="X135" s="6" t="n"/>
       <c r="Y135" s="6" t="n"/>
+      <c r="Z135" s="6" t="n"/>
+      <c r="AA135" s="6" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="3" t="n"/>
@@ -4424,8 +4714,8 @@
       <c r="H136" s="3" t="n"/>
       <c r="I136" s="3" t="n"/>
       <c r="J136" s="3" t="n"/>
-      <c r="K136" s="5" t="n"/>
-      <c r="L136" s="5" t="n"/>
+      <c r="K136" s="3" t="n"/>
+      <c r="L136" s="3" t="n"/>
       <c r="M136" s="5" t="n"/>
       <c r="N136" s="5" t="n"/>
       <c r="O136" s="5" t="n"/>
@@ -4439,6 +4729,8 @@
       <c r="W136" s="5" t="n"/>
       <c r="X136" s="5" t="n"/>
       <c r="Y136" s="5" t="n"/>
+      <c r="Z136" s="5" t="n"/>
+      <c r="AA136" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="6" t="n"/>
@@ -4466,6 +4758,8 @@
       <c r="W137" s="6" t="n"/>
       <c r="X137" s="6" t="n"/>
       <c r="Y137" s="6" t="n"/>
+      <c r="Z137" s="6" t="n"/>
+      <c r="AA137" s="6" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="3" t="n"/>
@@ -4478,8 +4772,8 @@
       <c r="H138" s="3" t="n"/>
       <c r="I138" s="3" t="n"/>
       <c r="J138" s="3" t="n"/>
-      <c r="K138" s="5" t="n"/>
-      <c r="L138" s="5" t="n"/>
+      <c r="K138" s="3" t="n"/>
+      <c r="L138" s="3" t="n"/>
       <c r="M138" s="5" t="n"/>
       <c r="N138" s="5" t="n"/>
       <c r="O138" s="5" t="n"/>
@@ -4493,6 +4787,8 @@
       <c r="W138" s="5" t="n"/>
       <c r="X138" s="5" t="n"/>
       <c r="Y138" s="5" t="n"/>
+      <c r="Z138" s="5" t="n"/>
+      <c r="AA138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="6" t="n"/>
@@ -4520,6 +4816,8 @@
       <c r="W139" s="6" t="n"/>
       <c r="X139" s="6" t="n"/>
       <c r="Y139" s="6" t="n"/>
+      <c r="Z139" s="6" t="n"/>
+      <c r="AA139" s="6" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="3" t="n"/>
@@ -4532,8 +4830,8 @@
       <c r="H140" s="3" t="n"/>
       <c r="I140" s="3" t="n"/>
       <c r="J140" s="3" t="n"/>
-      <c r="K140" s="5" t="n"/>
-      <c r="L140" s="5" t="n"/>
+      <c r="K140" s="3" t="n"/>
+      <c r="L140" s="3" t="n"/>
       <c r="M140" s="5" t="n"/>
       <c r="N140" s="5" t="n"/>
       <c r="O140" s="5" t="n"/>
@@ -4547,6 +4845,8 @@
       <c r="W140" s="5" t="n"/>
       <c r="X140" s="5" t="n"/>
       <c r="Y140" s="5" t="n"/>
+      <c r="Z140" s="5" t="n"/>
+      <c r="AA140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="6" t="n"/>
@@ -4574,6 +4874,8 @@
       <c r="W141" s="6" t="n"/>
       <c r="X141" s="6" t="n"/>
       <c r="Y141" s="6" t="n"/>
+      <c r="Z141" s="6" t="n"/>
+      <c r="AA141" s="6" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="3" t="n"/>
@@ -4586,8 +4888,8 @@
       <c r="H142" s="3" t="n"/>
       <c r="I142" s="3" t="n"/>
       <c r="J142" s="3" t="n"/>
-      <c r="K142" s="5" t="n"/>
-      <c r="L142" s="5" t="n"/>
+      <c r="K142" s="3" t="n"/>
+      <c r="L142" s="3" t="n"/>
       <c r="M142" s="5" t="n"/>
       <c r="N142" s="5" t="n"/>
       <c r="O142" s="5" t="n"/>
@@ -4601,6 +4903,8 @@
       <c r="W142" s="5" t="n"/>
       <c r="X142" s="5" t="n"/>
       <c r="Y142" s="5" t="n"/>
+      <c r="Z142" s="5" t="n"/>
+      <c r="AA142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="6" t="n"/>
@@ -4628,6 +4932,8 @@
       <c r="W143" s="6" t="n"/>
       <c r="X143" s="6" t="n"/>
       <c r="Y143" s="6" t="n"/>
+      <c r="Z143" s="6" t="n"/>
+      <c r="AA143" s="6" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="3" t="n"/>
@@ -4640,8 +4946,8 @@
       <c r="H144" s="3" t="n"/>
       <c r="I144" s="3" t="n"/>
       <c r="J144" s="3" t="n"/>
-      <c r="K144" s="5" t="n"/>
-      <c r="L144" s="5" t="n"/>
+      <c r="K144" s="3" t="n"/>
+      <c r="L144" s="3" t="n"/>
       <c r="M144" s="5" t="n"/>
       <c r="N144" s="5" t="n"/>
       <c r="O144" s="5" t="n"/>
@@ -4655,6 +4961,8 @@
       <c r="W144" s="5" t="n"/>
       <c r="X144" s="5" t="n"/>
       <c r="Y144" s="5" t="n"/>
+      <c r="Z144" s="5" t="n"/>
+      <c r="AA144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="6" t="n"/>
@@ -4682,6 +4990,8 @@
       <c r="W145" s="6" t="n"/>
       <c r="X145" s="6" t="n"/>
       <c r="Y145" s="6" t="n"/>
+      <c r="Z145" s="6" t="n"/>
+      <c r="AA145" s="6" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="3" t="n"/>
@@ -4694,8 +5004,8 @@
       <c r="H146" s="3" t="n"/>
       <c r="I146" s="3" t="n"/>
       <c r="J146" s="3" t="n"/>
-      <c r="K146" s="5" t="n"/>
-      <c r="L146" s="5" t="n"/>
+      <c r="K146" s="3" t="n"/>
+      <c r="L146" s="3" t="n"/>
       <c r="M146" s="5" t="n"/>
       <c r="N146" s="5" t="n"/>
       <c r="O146" s="5" t="n"/>
@@ -4709,6 +5019,8 @@
       <c r="W146" s="5" t="n"/>
       <c r="X146" s="5" t="n"/>
       <c r="Y146" s="5" t="n"/>
+      <c r="Z146" s="5" t="n"/>
+      <c r="AA146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="6" t="n"/>
@@ -4736,6 +5048,8 @@
       <c r="W147" s="6" t="n"/>
       <c r="X147" s="6" t="n"/>
       <c r="Y147" s="6" t="n"/>
+      <c r="Z147" s="6" t="n"/>
+      <c r="AA147" s="6" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="3" t="n"/>
@@ -4748,8 +5062,8 @@
       <c r="H148" s="3" t="n"/>
       <c r="I148" s="3" t="n"/>
       <c r="J148" s="3" t="n"/>
-      <c r="K148" s="5" t="n"/>
-      <c r="L148" s="5" t="n"/>
+      <c r="K148" s="3" t="n"/>
+      <c r="L148" s="3" t="n"/>
       <c r="M148" s="5" t="n"/>
       <c r="N148" s="5" t="n"/>
       <c r="O148" s="5" t="n"/>
@@ -4763,6 +5077,8 @@
       <c r="W148" s="5" t="n"/>
       <c r="X148" s="5" t="n"/>
       <c r="Y148" s="5" t="n"/>
+      <c r="Z148" s="5" t="n"/>
+      <c r="AA148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="6" t="n"/>
@@ -4790,6 +5106,8 @@
       <c r="W149" s="6" t="n"/>
       <c r="X149" s="6" t="n"/>
       <c r="Y149" s="6" t="n"/>
+      <c r="Z149" s="6" t="n"/>
+      <c r="AA149" s="6" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="3" t="n"/>
@@ -4802,8 +5120,8 @@
       <c r="H150" s="3" t="n"/>
       <c r="I150" s="3" t="n"/>
       <c r="J150" s="3" t="n"/>
-      <c r="K150" s="5" t="n"/>
-      <c r="L150" s="5" t="n"/>
+      <c r="K150" s="3" t="n"/>
+      <c r="L150" s="3" t="n"/>
       <c r="M150" s="5" t="n"/>
       <c r="N150" s="5" t="n"/>
       <c r="O150" s="5" t="n"/>
@@ -4817,6 +5135,8 @@
       <c r="W150" s="5" t="n"/>
       <c r="X150" s="5" t="n"/>
       <c r="Y150" s="5" t="n"/>
+      <c r="Z150" s="5" t="n"/>
+      <c r="AA150" s="5" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="6" t="n"/>
@@ -4844,6 +5164,8 @@
       <c r="W151" s="6" t="n"/>
       <c r="X151" s="6" t="n"/>
       <c r="Y151" s="6" t="n"/>
+      <c r="Z151" s="6" t="n"/>
+      <c r="AA151" s="6" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="3" t="n"/>
@@ -4856,8 +5178,8 @@
       <c r="H152" s="3" t="n"/>
       <c r="I152" s="3" t="n"/>
       <c r="J152" s="3" t="n"/>
-      <c r="K152" s="5" t="n"/>
-      <c r="L152" s="5" t="n"/>
+      <c r="K152" s="3" t="n"/>
+      <c r="L152" s="3" t="n"/>
       <c r="M152" s="5" t="n"/>
       <c r="N152" s="5" t="n"/>
       <c r="O152" s="5" t="n"/>
@@ -4871,6 +5193,8 @@
       <c r="W152" s="5" t="n"/>
       <c r="X152" s="5" t="n"/>
       <c r="Y152" s="5" t="n"/>
+      <c r="Z152" s="5" t="n"/>
+      <c r="AA152" s="5" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="6" t="n"/>
@@ -4898,6 +5222,8 @@
       <c r="W153" s="6" t="n"/>
       <c r="X153" s="6" t="n"/>
       <c r="Y153" s="6" t="n"/>
+      <c r="Z153" s="6" t="n"/>
+      <c r="AA153" s="6" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="3" t="n"/>
@@ -4910,8 +5236,8 @@
       <c r="H154" s="3" t="n"/>
       <c r="I154" s="3" t="n"/>
       <c r="J154" s="3" t="n"/>
-      <c r="K154" s="5" t="n"/>
-      <c r="L154" s="5" t="n"/>
+      <c r="K154" s="3" t="n"/>
+      <c r="L154" s="3" t="n"/>
       <c r="M154" s="5" t="n"/>
       <c r="N154" s="5" t="n"/>
       <c r="O154" s="5" t="n"/>
@@ -4925,6 +5251,8 @@
       <c r="W154" s="5" t="n"/>
       <c r="X154" s="5" t="n"/>
       <c r="Y154" s="5" t="n"/>
+      <c r="Z154" s="5" t="n"/>
+      <c r="AA154" s="5" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="6" t="n"/>
@@ -4952,6 +5280,8 @@
       <c r="W155" s="6" t="n"/>
       <c r="X155" s="6" t="n"/>
       <c r="Y155" s="6" t="n"/>
+      <c r="Z155" s="6" t="n"/>
+      <c r="AA155" s="6" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="3" t="n"/>
@@ -4964,8 +5294,8 @@
       <c r="H156" s="3" t="n"/>
       <c r="I156" s="3" t="n"/>
       <c r="J156" s="3" t="n"/>
-      <c r="K156" s="5" t="n"/>
-      <c r="L156" s="5" t="n"/>
+      <c r="K156" s="3" t="n"/>
+      <c r="L156" s="3" t="n"/>
       <c r="M156" s="5" t="n"/>
       <c r="N156" s="5" t="n"/>
       <c r="O156" s="5" t="n"/>
@@ -4979,6 +5309,8 @@
       <c r="W156" s="5" t="n"/>
       <c r="X156" s="5" t="n"/>
       <c r="Y156" s="5" t="n"/>
+      <c r="Z156" s="5" t="n"/>
+      <c r="AA156" s="5" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="6" t="n"/>
@@ -5006,6 +5338,8 @@
       <c r="W157" s="6" t="n"/>
       <c r="X157" s="6" t="n"/>
       <c r="Y157" s="6" t="n"/>
+      <c r="Z157" s="6" t="n"/>
+      <c r="AA157" s="6" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="3" t="n"/>
@@ -5018,8 +5352,8 @@
       <c r="H158" s="3" t="n"/>
       <c r="I158" s="3" t="n"/>
       <c r="J158" s="3" t="n"/>
-      <c r="K158" s="5" t="n"/>
-      <c r="L158" s="5" t="n"/>
+      <c r="K158" s="3" t="n"/>
+      <c r="L158" s="3" t="n"/>
       <c r="M158" s="5" t="n"/>
       <c r="N158" s="5" t="n"/>
       <c r="O158" s="5" t="n"/>
@@ -5033,6 +5367,8 @@
       <c r="W158" s="5" t="n"/>
       <c r="X158" s="5" t="n"/>
       <c r="Y158" s="5" t="n"/>
+      <c r="Z158" s="5" t="n"/>
+      <c r="AA158" s="5" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="6" t="n"/>
@@ -5060,6 +5396,8 @@
       <c r="W159" s="6" t="n"/>
       <c r="X159" s="6" t="n"/>
       <c r="Y159" s="6" t="n"/>
+      <c r="Z159" s="6" t="n"/>
+      <c r="AA159" s="6" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="3" t="n"/>
@@ -5072,8 +5410,8 @@
       <c r="H160" s="3" t="n"/>
       <c r="I160" s="3" t="n"/>
       <c r="J160" s="3" t="n"/>
-      <c r="K160" s="5" t="n"/>
-      <c r="L160" s="5" t="n"/>
+      <c r="K160" s="3" t="n"/>
+      <c r="L160" s="3" t="n"/>
       <c r="M160" s="5" t="n"/>
       <c r="N160" s="5" t="n"/>
       <c r="O160" s="5" t="n"/>
@@ -5087,6 +5425,8 @@
       <c r="W160" s="5" t="n"/>
       <c r="X160" s="5" t="n"/>
       <c r="Y160" s="5" t="n"/>
+      <c r="Z160" s="5" t="n"/>
+      <c r="AA160" s="5" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="6" t="n"/>
@@ -5114,6 +5454,8 @@
       <c r="W161" s="6" t="n"/>
       <c r="X161" s="6" t="n"/>
       <c r="Y161" s="6" t="n"/>
+      <c r="Z161" s="6" t="n"/>
+      <c r="AA161" s="6" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="3" t="n"/>
@@ -5126,8 +5468,8 @@
       <c r="H162" s="3" t="n"/>
       <c r="I162" s="3" t="n"/>
       <c r="J162" s="3" t="n"/>
-      <c r="K162" s="5" t="n"/>
-      <c r="L162" s="5" t="n"/>
+      <c r="K162" s="3" t="n"/>
+      <c r="L162" s="3" t="n"/>
       <c r="M162" s="5" t="n"/>
       <c r="N162" s="5" t="n"/>
       <c r="O162" s="5" t="n"/>
@@ -5141,6 +5483,8 @@
       <c r="W162" s="5" t="n"/>
       <c r="X162" s="5" t="n"/>
       <c r="Y162" s="5" t="n"/>
+      <c r="Z162" s="5" t="n"/>
+      <c r="AA162" s="5" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="6" t="n"/>
@@ -5168,6 +5512,8 @@
       <c r="W163" s="6" t="n"/>
       <c r="X163" s="6" t="n"/>
       <c r="Y163" s="6" t="n"/>
+      <c r="Z163" s="6" t="n"/>
+      <c r="AA163" s="6" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="3" t="n"/>
@@ -5180,8 +5526,8 @@
       <c r="H164" s="3" t="n"/>
       <c r="I164" s="3" t="n"/>
       <c r="J164" s="3" t="n"/>
-      <c r="K164" s="5" t="n"/>
-      <c r="L164" s="5" t="n"/>
+      <c r="K164" s="3" t="n"/>
+      <c r="L164" s="3" t="n"/>
       <c r="M164" s="5" t="n"/>
       <c r="N164" s="5" t="n"/>
       <c r="O164" s="5" t="n"/>
@@ -5195,6 +5541,8 @@
       <c r="W164" s="5" t="n"/>
       <c r="X164" s="5" t="n"/>
       <c r="Y164" s="5" t="n"/>
+      <c r="Z164" s="5" t="n"/>
+      <c r="AA164" s="5" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="6" t="n"/>
@@ -5222,6 +5570,8 @@
       <c r="W165" s="6" t="n"/>
       <c r="X165" s="6" t="n"/>
       <c r="Y165" s="6" t="n"/>
+      <c r="Z165" s="6" t="n"/>
+      <c r="AA165" s="6" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="3" t="n"/>
@@ -5234,8 +5584,8 @@
       <c r="H166" s="3" t="n"/>
       <c r="I166" s="3" t="n"/>
       <c r="J166" s="3" t="n"/>
-      <c r="K166" s="5" t="n"/>
-      <c r="L166" s="5" t="n"/>
+      <c r="K166" s="3" t="n"/>
+      <c r="L166" s="3" t="n"/>
       <c r="M166" s="5" t="n"/>
       <c r="N166" s="5" t="n"/>
       <c r="O166" s="5" t="n"/>
@@ -5249,6 +5599,8 @@
       <c r="W166" s="5" t="n"/>
       <c r="X166" s="5" t="n"/>
       <c r="Y166" s="5" t="n"/>
+      <c r="Z166" s="5" t="n"/>
+      <c r="AA166" s="5" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="6" t="n"/>
@@ -5276,6 +5628,8 @@
       <c r="W167" s="6" t="n"/>
       <c r="X167" s="6" t="n"/>
       <c r="Y167" s="6" t="n"/>
+      <c r="Z167" s="6" t="n"/>
+      <c r="AA167" s="6" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="3" t="n"/>
@@ -5288,8 +5642,8 @@
       <c r="H168" s="3" t="n"/>
       <c r="I168" s="3" t="n"/>
       <c r="J168" s="3" t="n"/>
-      <c r="K168" s="5" t="n"/>
-      <c r="L168" s="5" t="n"/>
+      <c r="K168" s="3" t="n"/>
+      <c r="L168" s="3" t="n"/>
       <c r="M168" s="5" t="n"/>
       <c r="N168" s="5" t="n"/>
       <c r="O168" s="5" t="n"/>
@@ -5303,6 +5657,8 @@
       <c r="W168" s="5" t="n"/>
       <c r="X168" s="5" t="n"/>
       <c r="Y168" s="5" t="n"/>
+      <c r="Z168" s="5" t="n"/>
+      <c r="AA168" s="5" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="6" t="n"/>
@@ -5330,6 +5686,8 @@
       <c r="W169" s="6" t="n"/>
       <c r="X169" s="6" t="n"/>
       <c r="Y169" s="6" t="n"/>
+      <c r="Z169" s="6" t="n"/>
+      <c r="AA169" s="6" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="3" t="n"/>
@@ -5342,8 +5700,8 @@
       <c r="H170" s="3" t="n"/>
       <c r="I170" s="3" t="n"/>
       <c r="J170" s="3" t="n"/>
-      <c r="K170" s="5" t="n"/>
-      <c r="L170" s="5" t="n"/>
+      <c r="K170" s="3" t="n"/>
+      <c r="L170" s="3" t="n"/>
       <c r="M170" s="5" t="n"/>
       <c r="N170" s="5" t="n"/>
       <c r="O170" s="5" t="n"/>
@@ -5357,6 +5715,8 @@
       <c r="W170" s="5" t="n"/>
       <c r="X170" s="5" t="n"/>
       <c r="Y170" s="5" t="n"/>
+      <c r="Z170" s="5" t="n"/>
+      <c r="AA170" s="5" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="6" t="n"/>
@@ -5384,6 +5744,8 @@
       <c r="W171" s="6" t="n"/>
       <c r="X171" s="6" t="n"/>
       <c r="Y171" s="6" t="n"/>
+      <c r="Z171" s="6" t="n"/>
+      <c r="AA171" s="6" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="3" t="n"/>
@@ -5396,8 +5758,8 @@
       <c r="H172" s="3" t="n"/>
       <c r="I172" s="3" t="n"/>
       <c r="J172" s="3" t="n"/>
-      <c r="K172" s="5" t="n"/>
-      <c r="L172" s="5" t="n"/>
+      <c r="K172" s="3" t="n"/>
+      <c r="L172" s="3" t="n"/>
       <c r="M172" s="5" t="n"/>
       <c r="N172" s="5" t="n"/>
       <c r="O172" s="5" t="n"/>
@@ -5411,6 +5773,8 @@
       <c r="W172" s="5" t="n"/>
       <c r="X172" s="5" t="n"/>
       <c r="Y172" s="5" t="n"/>
+      <c r="Z172" s="5" t="n"/>
+      <c r="AA172" s="5" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="6" t="n"/>
@@ -5438,6 +5802,8 @@
       <c r="W173" s="6" t="n"/>
       <c r="X173" s="6" t="n"/>
       <c r="Y173" s="6" t="n"/>
+      <c r="Z173" s="6" t="n"/>
+      <c r="AA173" s="6" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="3" t="n"/>
@@ -5450,8 +5816,8 @@
       <c r="H174" s="3" t="n"/>
       <c r="I174" s="3" t="n"/>
       <c r="J174" s="3" t="n"/>
-      <c r="K174" s="5" t="n"/>
-      <c r="L174" s="5" t="n"/>
+      <c r="K174" s="3" t="n"/>
+      <c r="L174" s="3" t="n"/>
       <c r="M174" s="5" t="n"/>
       <c r="N174" s="5" t="n"/>
       <c r="O174" s="5" t="n"/>
@@ -5465,6 +5831,8 @@
       <c r="W174" s="5" t="n"/>
       <c r="X174" s="5" t="n"/>
       <c r="Y174" s="5" t="n"/>
+      <c r="Z174" s="5" t="n"/>
+      <c r="AA174" s="5" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="6" t="n"/>
@@ -5492,6 +5860,8 @@
       <c r="W175" s="6" t="n"/>
       <c r="X175" s="6" t="n"/>
       <c r="Y175" s="6" t="n"/>
+      <c r="Z175" s="6" t="n"/>
+      <c r="AA175" s="6" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="3" t="n"/>
@@ -5504,8 +5874,8 @@
       <c r="H176" s="3" t="n"/>
       <c r="I176" s="3" t="n"/>
       <c r="J176" s="3" t="n"/>
-      <c r="K176" s="5" t="n"/>
-      <c r="L176" s="5" t="n"/>
+      <c r="K176" s="3" t="n"/>
+      <c r="L176" s="3" t="n"/>
       <c r="M176" s="5" t="n"/>
       <c r="N176" s="5" t="n"/>
       <c r="O176" s="5" t="n"/>
@@ -5519,6 +5889,8 @@
       <c r="W176" s="5" t="n"/>
       <c r="X176" s="5" t="n"/>
       <c r="Y176" s="5" t="n"/>
+      <c r="Z176" s="5" t="n"/>
+      <c r="AA176" s="5" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="6" t="n"/>
@@ -5546,6 +5918,8 @@
       <c r="W177" s="6" t="n"/>
       <c r="X177" s="6" t="n"/>
       <c r="Y177" s="6" t="n"/>
+      <c r="Z177" s="6" t="n"/>
+      <c r="AA177" s="6" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="3" t="n"/>
@@ -5558,8 +5932,8 @@
       <c r="H178" s="3" t="n"/>
       <c r="I178" s="3" t="n"/>
       <c r="J178" s="3" t="n"/>
-      <c r="K178" s="5" t="n"/>
-      <c r="L178" s="5" t="n"/>
+      <c r="K178" s="3" t="n"/>
+      <c r="L178" s="3" t="n"/>
       <c r="M178" s="5" t="n"/>
       <c r="N178" s="5" t="n"/>
       <c r="O178" s="5" t="n"/>
@@ -5573,6 +5947,8 @@
       <c r="W178" s="5" t="n"/>
       <c r="X178" s="5" t="n"/>
       <c r="Y178" s="5" t="n"/>
+      <c r="Z178" s="5" t="n"/>
+      <c r="AA178" s="5" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="6" t="n"/>
@@ -5600,6 +5976,8 @@
       <c r="W179" s="6" t="n"/>
       <c r="X179" s="6" t="n"/>
       <c r="Y179" s="6" t="n"/>
+      <c r="Z179" s="6" t="n"/>
+      <c r="AA179" s="6" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="3" t="n"/>
@@ -5612,8 +5990,8 @@
       <c r="H180" s="3" t="n"/>
       <c r="I180" s="3" t="n"/>
       <c r="J180" s="3" t="n"/>
-      <c r="K180" s="5" t="n"/>
-      <c r="L180" s="5" t="n"/>
+      <c r="K180" s="3" t="n"/>
+      <c r="L180" s="3" t="n"/>
       <c r="M180" s="5" t="n"/>
       <c r="N180" s="5" t="n"/>
       <c r="O180" s="5" t="n"/>
@@ -5627,6 +6005,8 @@
       <c r="W180" s="5" t="n"/>
       <c r="X180" s="5" t="n"/>
       <c r="Y180" s="5" t="n"/>
+      <c r="Z180" s="5" t="n"/>
+      <c r="AA180" s="5" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="6" t="n"/>
@@ -5654,6 +6034,8 @@
       <c r="W181" s="6" t="n"/>
       <c r="X181" s="6" t="n"/>
       <c r="Y181" s="6" t="n"/>
+      <c r="Z181" s="6" t="n"/>
+      <c r="AA181" s="6" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="3" t="n"/>
@@ -5666,8 +6048,8 @@
       <c r="H182" s="3" t="n"/>
       <c r="I182" s="3" t="n"/>
       <c r="J182" s="3" t="n"/>
-      <c r="K182" s="5" t="n"/>
-      <c r="L182" s="5" t="n"/>
+      <c r="K182" s="3" t="n"/>
+      <c r="L182" s="3" t="n"/>
       <c r="M182" s="5" t="n"/>
       <c r="N182" s="5" t="n"/>
       <c r="O182" s="5" t="n"/>
@@ -5681,6 +6063,8 @@
       <c r="W182" s="5" t="n"/>
       <c r="X182" s="5" t="n"/>
       <c r="Y182" s="5" t="n"/>
+      <c r="Z182" s="5" t="n"/>
+      <c r="AA182" s="5" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="6" t="n"/>
@@ -5708,6 +6092,8 @@
       <c r="W183" s="6" t="n"/>
       <c r="X183" s="6" t="n"/>
       <c r="Y183" s="6" t="n"/>
+      <c r="Z183" s="6" t="n"/>
+      <c r="AA183" s="6" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="3" t="n"/>
@@ -5720,8 +6106,8 @@
       <c r="H184" s="3" t="n"/>
       <c r="I184" s="3" t="n"/>
       <c r="J184" s="3" t="n"/>
-      <c r="K184" s="5" t="n"/>
-      <c r="L184" s="5" t="n"/>
+      <c r="K184" s="3" t="n"/>
+      <c r="L184" s="3" t="n"/>
       <c r="M184" s="5" t="n"/>
       <c r="N184" s="5" t="n"/>
       <c r="O184" s="5" t="n"/>
@@ -5735,6 +6121,8 @@
       <c r="W184" s="5" t="n"/>
       <c r="X184" s="5" t="n"/>
       <c r="Y184" s="5" t="n"/>
+      <c r="Z184" s="5" t="n"/>
+      <c r="AA184" s="5" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="6" t="n"/>
@@ -5762,6 +6150,8 @@
       <c r="W185" s="6" t="n"/>
       <c r="X185" s="6" t="n"/>
       <c r="Y185" s="6" t="n"/>
+      <c r="Z185" s="6" t="n"/>
+      <c r="AA185" s="6" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="3" t="n"/>
@@ -5774,8 +6164,8 @@
       <c r="H186" s="3" t="n"/>
       <c r="I186" s="3" t="n"/>
       <c r="J186" s="3" t="n"/>
-      <c r="K186" s="5" t="n"/>
-      <c r="L186" s="5" t="n"/>
+      <c r="K186" s="3" t="n"/>
+      <c r="L186" s="3" t="n"/>
       <c r="M186" s="5" t="n"/>
       <c r="N186" s="5" t="n"/>
       <c r="O186" s="5" t="n"/>
@@ -5789,6 +6179,8 @@
       <c r="W186" s="5" t="n"/>
       <c r="X186" s="5" t="n"/>
       <c r="Y186" s="5" t="n"/>
+      <c r="Z186" s="5" t="n"/>
+      <c r="AA186" s="5" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="6" t="n"/>
@@ -5816,6 +6208,8 @@
       <c r="W187" s="6" t="n"/>
       <c r="X187" s="6" t="n"/>
       <c r="Y187" s="6" t="n"/>
+      <c r="Z187" s="6" t="n"/>
+      <c r="AA187" s="6" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="3" t="n"/>
@@ -5828,8 +6222,8 @@
       <c r="H188" s="3" t="n"/>
       <c r="I188" s="3" t="n"/>
       <c r="J188" s="3" t="n"/>
-      <c r="K188" s="5" t="n"/>
-      <c r="L188" s="5" t="n"/>
+      <c r="K188" s="3" t="n"/>
+      <c r="L188" s="3" t="n"/>
       <c r="M188" s="5" t="n"/>
       <c r="N188" s="5" t="n"/>
       <c r="O188" s="5" t="n"/>
@@ -5843,6 +6237,8 @@
       <c r="W188" s="5" t="n"/>
       <c r="X188" s="5" t="n"/>
       <c r="Y188" s="5" t="n"/>
+      <c r="Z188" s="5" t="n"/>
+      <c r="AA188" s="5" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="6" t="n"/>
@@ -5870,6 +6266,8 @@
       <c r="W189" s="6" t="n"/>
       <c r="X189" s="6" t="n"/>
       <c r="Y189" s="6" t="n"/>
+      <c r="Z189" s="6" t="n"/>
+      <c r="AA189" s="6" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="3" t="n"/>
@@ -5882,8 +6280,8 @@
       <c r="H190" s="3" t="n"/>
       <c r="I190" s="3" t="n"/>
       <c r="J190" s="3" t="n"/>
-      <c r="K190" s="5" t="n"/>
-      <c r="L190" s="5" t="n"/>
+      <c r="K190" s="3" t="n"/>
+      <c r="L190" s="3" t="n"/>
       <c r="M190" s="5" t="n"/>
       <c r="N190" s="5" t="n"/>
       <c r="O190" s="5" t="n"/>
@@ -5897,6 +6295,8 @@
       <c r="W190" s="5" t="n"/>
       <c r="X190" s="5" t="n"/>
       <c r="Y190" s="5" t="n"/>
+      <c r="Z190" s="5" t="n"/>
+      <c r="AA190" s="5" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="6" t="n"/>
@@ -5924,6 +6324,8 @@
       <c r="W191" s="6" t="n"/>
       <c r="X191" s="6" t="n"/>
       <c r="Y191" s="6" t="n"/>
+      <c r="Z191" s="6" t="n"/>
+      <c r="AA191" s="6" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="3" t="n"/>
@@ -5936,8 +6338,8 @@
       <c r="H192" s="3" t="n"/>
       <c r="I192" s="3" t="n"/>
       <c r="J192" s="3" t="n"/>
-      <c r="K192" s="5" t="n"/>
-      <c r="L192" s="5" t="n"/>
+      <c r="K192" s="3" t="n"/>
+      <c r="L192" s="3" t="n"/>
       <c r="M192" s="5" t="n"/>
       <c r="N192" s="5" t="n"/>
       <c r="O192" s="5" t="n"/>
@@ -5951,6 +6353,8 @@
       <c r="W192" s="5" t="n"/>
       <c r="X192" s="5" t="n"/>
       <c r="Y192" s="5" t="n"/>
+      <c r="Z192" s="5" t="n"/>
+      <c r="AA192" s="5" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="6" t="n"/>
@@ -5978,6 +6382,8 @@
       <c r="W193" s="6" t="n"/>
       <c r="X193" s="6" t="n"/>
       <c r="Y193" s="6" t="n"/>
+      <c r="Z193" s="6" t="n"/>
+      <c r="AA193" s="6" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="3" t="n"/>
@@ -5990,8 +6396,8 @@
       <c r="H194" s="3" t="n"/>
       <c r="I194" s="3" t="n"/>
       <c r="J194" s="3" t="n"/>
-      <c r="K194" s="5" t="n"/>
-      <c r="L194" s="5" t="n"/>
+      <c r="K194" s="3" t="n"/>
+      <c r="L194" s="3" t="n"/>
       <c r="M194" s="5" t="n"/>
       <c r="N194" s="5" t="n"/>
       <c r="O194" s="5" t="n"/>
@@ -6005,6 +6411,8 @@
       <c r="W194" s="5" t="n"/>
       <c r="X194" s="5" t="n"/>
       <c r="Y194" s="5" t="n"/>
+      <c r="Z194" s="5" t="n"/>
+      <c r="AA194" s="5" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="6" t="n"/>
@@ -6032,6 +6440,8 @@
       <c r="W195" s="6" t="n"/>
       <c r="X195" s="6" t="n"/>
       <c r="Y195" s="6" t="n"/>
+      <c r="Z195" s="6" t="n"/>
+      <c r="AA195" s="6" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="3" t="n"/>
@@ -6044,8 +6454,8 @@
       <c r="H196" s="3" t="n"/>
       <c r="I196" s="3" t="n"/>
       <c r="J196" s="3" t="n"/>
-      <c r="K196" s="5" t="n"/>
-      <c r="L196" s="5" t="n"/>
+      <c r="K196" s="3" t="n"/>
+      <c r="L196" s="3" t="n"/>
       <c r="M196" s="5" t="n"/>
       <c r="N196" s="5" t="n"/>
       <c r="O196" s="5" t="n"/>
@@ -6059,6 +6469,8 @@
       <c r="W196" s="5" t="n"/>
       <c r="X196" s="5" t="n"/>
       <c r="Y196" s="5" t="n"/>
+      <c r="Z196" s="5" t="n"/>
+      <c r="AA196" s="5" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="6" t="n"/>
@@ -6086,6 +6498,8 @@
       <c r="W197" s="6" t="n"/>
       <c r="X197" s="6" t="n"/>
       <c r="Y197" s="6" t="n"/>
+      <c r="Z197" s="6" t="n"/>
+      <c r="AA197" s="6" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="3" t="n"/>
@@ -6098,8 +6512,8 @@
       <c r="H198" s="3" t="n"/>
       <c r="I198" s="3" t="n"/>
       <c r="J198" s="3" t="n"/>
-      <c r="K198" s="5" t="n"/>
-      <c r="L198" s="5" t="n"/>
+      <c r="K198" s="3" t="n"/>
+      <c r="L198" s="3" t="n"/>
       <c r="M198" s="5" t="n"/>
       <c r="N198" s="5" t="n"/>
       <c r="O198" s="5" t="n"/>
@@ -6113,6 +6527,8 @@
       <c r="W198" s="5" t="n"/>
       <c r="X198" s="5" t="n"/>
       <c r="Y198" s="5" t="n"/>
+      <c r="Z198" s="5" t="n"/>
+      <c r="AA198" s="5" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="6" t="n"/>
@@ -6140,6 +6556,8 @@
       <c r="W199" s="6" t="n"/>
       <c r="X199" s="6" t="n"/>
       <c r="Y199" s="6" t="n"/>
+      <c r="Z199" s="6" t="n"/>
+      <c r="AA199" s="6" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="3" t="n"/>
@@ -6152,8 +6570,8 @@
       <c r="H200" s="3" t="n"/>
       <c r="I200" s="3" t="n"/>
       <c r="J200" s="3" t="n"/>
-      <c r="K200" s="5" t="n"/>
-      <c r="L200" s="5" t="n"/>
+      <c r="K200" s="3" t="n"/>
+      <c r="L200" s="3" t="n"/>
       <c r="M200" s="5" t="n"/>
       <c r="N200" s="5" t="n"/>
       <c r="O200" s="5" t="n"/>
@@ -6167,6 +6585,8 @@
       <c r="W200" s="5" t="n"/>
       <c r="X200" s="5" t="n"/>
       <c r="Y200" s="5" t="n"/>
+      <c r="Z200" s="5" t="n"/>
+      <c r="AA200" s="5" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="6" t="n"/>
@@ -6194,6 +6614,8 @@
       <c r="W201" s="6" t="n"/>
       <c r="X201" s="6" t="n"/>
       <c r="Y201" s="6" t="n"/>
+      <c r="Z201" s="6" t="n"/>
+      <c r="AA201" s="6" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="3" t="n"/>
@@ -6206,8 +6628,8 @@
       <c r="H202" s="3" t="n"/>
       <c r="I202" s="3" t="n"/>
       <c r="J202" s="3" t="n"/>
-      <c r="K202" s="5" t="n"/>
-      <c r="L202" s="5" t="n"/>
+      <c r="K202" s="3" t="n"/>
+      <c r="L202" s="3" t="n"/>
       <c r="M202" s="5" t="n"/>
       <c r="N202" s="5" t="n"/>
       <c r="O202" s="5" t="n"/>
@@ -6221,6 +6643,8 @@
       <c r="W202" s="5" t="n"/>
       <c r="X202" s="5" t="n"/>
       <c r="Y202" s="5" t="n"/>
+      <c r="Z202" s="5" t="n"/>
+      <c r="AA202" s="5" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="6" t="n"/>
@@ -6248,6 +6672,8 @@
       <c r="W203" s="6" t="n"/>
       <c r="X203" s="6" t="n"/>
       <c r="Y203" s="6" t="n"/>
+      <c r="Z203" s="6" t="n"/>
+      <c r="AA203" s="6" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="3" t="n"/>
@@ -6260,8 +6686,8 @@
       <c r="H204" s="3" t="n"/>
       <c r="I204" s="3" t="n"/>
       <c r="J204" s="3" t="n"/>
-      <c r="K204" s="5" t="n"/>
-      <c r="L204" s="5" t="n"/>
+      <c r="K204" s="3" t="n"/>
+      <c r="L204" s="3" t="n"/>
       <c r="M204" s="5" t="n"/>
       <c r="N204" s="5" t="n"/>
       <c r="O204" s="5" t="n"/>
@@ -6275,6 +6701,8 @@
       <c r="W204" s="5" t="n"/>
       <c r="X204" s="5" t="n"/>
       <c r="Y204" s="5" t="n"/>
+      <c r="Z204" s="5" t="n"/>
+      <c r="AA204" s="5" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="6" t="n"/>
@@ -6302,6 +6730,8 @@
       <c r="W205" s="6" t="n"/>
       <c r="X205" s="6" t="n"/>
       <c r="Y205" s="6" t="n"/>
+      <c r="Z205" s="6" t="n"/>
+      <c r="AA205" s="6" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="3" t="n"/>
@@ -6314,8 +6744,8 @@
       <c r="H206" s="3" t="n"/>
       <c r="I206" s="3" t="n"/>
       <c r="J206" s="3" t="n"/>
-      <c r="K206" s="5" t="n"/>
-      <c r="L206" s="5" t="n"/>
+      <c r="K206" s="3" t="n"/>
+      <c r="L206" s="3" t="n"/>
       <c r="M206" s="5" t="n"/>
       <c r="N206" s="5" t="n"/>
       <c r="O206" s="5" t="n"/>
@@ -6329,6 +6759,8 @@
       <c r="W206" s="5" t="n"/>
       <c r="X206" s="5" t="n"/>
       <c r="Y206" s="5" t="n"/>
+      <c r="Z206" s="5" t="n"/>
+      <c r="AA206" s="5" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="6" t="n"/>
@@ -6356,6 +6788,8 @@
       <c r="W207" s="6" t="n"/>
       <c r="X207" s="6" t="n"/>
       <c r="Y207" s="6" t="n"/>
+      <c r="Z207" s="6" t="n"/>
+      <c r="AA207" s="6" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="3" t="n"/>
@@ -6368,8 +6802,8 @@
       <c r="H208" s="3" t="n"/>
       <c r="I208" s="3" t="n"/>
       <c r="J208" s="3" t="n"/>
-      <c r="K208" s="5" t="n"/>
-      <c r="L208" s="5" t="n"/>
+      <c r="K208" s="3" t="n"/>
+      <c r="L208" s="3" t="n"/>
       <c r="M208" s="5" t="n"/>
       <c r="N208" s="5" t="n"/>
       <c r="O208" s="5" t="n"/>
@@ -6383,6 +6817,8 @@
       <c r="W208" s="5" t="n"/>
       <c r="X208" s="5" t="n"/>
       <c r="Y208" s="5" t="n"/>
+      <c r="Z208" s="5" t="n"/>
+      <c r="AA208" s="5" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="6" t="n"/>
@@ -6410,6 +6846,8 @@
       <c r="W209" s="6" t="n"/>
       <c r="X209" s="6" t="n"/>
       <c r="Y209" s="6" t="n"/>
+      <c r="Z209" s="6" t="n"/>
+      <c r="AA209" s="6" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="3" t="n"/>
@@ -6422,8 +6860,8 @@
       <c r="H210" s="3" t="n"/>
       <c r="I210" s="3" t="n"/>
       <c r="J210" s="3" t="n"/>
-      <c r="K210" s="5" t="n"/>
-      <c r="L210" s="5" t="n"/>
+      <c r="K210" s="3" t="n"/>
+      <c r="L210" s="3" t="n"/>
       <c r="M210" s="5" t="n"/>
       <c r="N210" s="5" t="n"/>
       <c r="O210" s="5" t="n"/>
@@ -6437,6 +6875,8 @@
       <c r="W210" s="5" t="n"/>
       <c r="X210" s="5" t="n"/>
       <c r="Y210" s="5" t="n"/>
+      <c r="Z210" s="5" t="n"/>
+      <c r="AA210" s="5" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="6" t="n"/>
@@ -6464,6 +6904,8 @@
       <c r="W211" s="6" t="n"/>
       <c r="X211" s="6" t="n"/>
       <c r="Y211" s="6" t="n"/>
+      <c r="Z211" s="6" t="n"/>
+      <c r="AA211" s="6" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="3" t="n"/>
@@ -6476,8 +6918,8 @@
       <c r="H212" s="3" t="n"/>
       <c r="I212" s="3" t="n"/>
       <c r="J212" s="3" t="n"/>
-      <c r="K212" s="5" t="n"/>
-      <c r="L212" s="5" t="n"/>
+      <c r="K212" s="3" t="n"/>
+      <c r="L212" s="3" t="n"/>
       <c r="M212" s="5" t="n"/>
       <c r="N212" s="5" t="n"/>
       <c r="O212" s="5" t="n"/>
@@ -6491,6 +6933,8 @@
       <c r="W212" s="5" t="n"/>
       <c r="X212" s="5" t="n"/>
       <c r="Y212" s="5" t="n"/>
+      <c r="Z212" s="5" t="n"/>
+      <c r="AA212" s="5" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="6" t="n"/>
@@ -6518,6 +6962,8 @@
       <c r="W213" s="6" t="n"/>
       <c r="X213" s="6" t="n"/>
       <c r="Y213" s="6" t="n"/>
+      <c r="Z213" s="6" t="n"/>
+      <c r="AA213" s="6" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="3" t="n"/>
@@ -6530,8 +6976,8 @@
       <c r="H214" s="3" t="n"/>
       <c r="I214" s="3" t="n"/>
       <c r="J214" s="3" t="n"/>
-      <c r="K214" s="5" t="n"/>
-      <c r="L214" s="5" t="n"/>
+      <c r="K214" s="3" t="n"/>
+      <c r="L214" s="3" t="n"/>
       <c r="M214" s="5" t="n"/>
       <c r="N214" s="5" t="n"/>
       <c r="O214" s="5" t="n"/>
@@ -6545,6 +6991,8 @@
       <c r="W214" s="5" t="n"/>
       <c r="X214" s="5" t="n"/>
       <c r="Y214" s="5" t="n"/>
+      <c r="Z214" s="5" t="n"/>
+      <c r="AA214" s="5" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="6" t="n"/>
@@ -6572,6 +7020,8 @@
       <c r="W215" s="6" t="n"/>
       <c r="X215" s="6" t="n"/>
       <c r="Y215" s="6" t="n"/>
+      <c r="Z215" s="6" t="n"/>
+      <c r="AA215" s="6" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="3" t="n"/>
@@ -6584,8 +7034,8 @@
       <c r="H216" s="3" t="n"/>
       <c r="I216" s="3" t="n"/>
       <c r="J216" s="3" t="n"/>
-      <c r="K216" s="5" t="n"/>
-      <c r="L216" s="5" t="n"/>
+      <c r="K216" s="3" t="n"/>
+      <c r="L216" s="3" t="n"/>
       <c r="M216" s="5" t="n"/>
       <c r="N216" s="5" t="n"/>
       <c r="O216" s="5" t="n"/>
@@ -6599,6 +7049,8 @@
       <c r="W216" s="5" t="n"/>
       <c r="X216" s="5" t="n"/>
       <c r="Y216" s="5" t="n"/>
+      <c r="Z216" s="5" t="n"/>
+      <c r="AA216" s="5" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="6" t="n"/>
@@ -6626,6 +7078,8 @@
       <c r="W217" s="6" t="n"/>
       <c r="X217" s="6" t="n"/>
       <c r="Y217" s="6" t="n"/>
+      <c r="Z217" s="6" t="n"/>
+      <c r="AA217" s="6" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="3" t="n"/>
@@ -6638,8 +7092,8 @@
       <c r="H218" s="3" t="n"/>
       <c r="I218" s="3" t="n"/>
       <c r="J218" s="3" t="n"/>
-      <c r="K218" s="5" t="n"/>
-      <c r="L218" s="5" t="n"/>
+      <c r="K218" s="3" t="n"/>
+      <c r="L218" s="3" t="n"/>
       <c r="M218" s="5" t="n"/>
       <c r="N218" s="5" t="n"/>
       <c r="O218" s="5" t="n"/>
@@ -6653,6 +7107,8 @@
       <c r="W218" s="5" t="n"/>
       <c r="X218" s="5" t="n"/>
       <c r="Y218" s="5" t="n"/>
+      <c r="Z218" s="5" t="n"/>
+      <c r="AA218" s="5" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="6" t="n"/>
@@ -6680,6 +7136,8 @@
       <c r="W219" s="6" t="n"/>
       <c r="X219" s="6" t="n"/>
       <c r="Y219" s="6" t="n"/>
+      <c r="Z219" s="6" t="n"/>
+      <c r="AA219" s="6" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="3" t="n"/>
@@ -6692,8 +7150,8 @@
       <c r="H220" s="3" t="n"/>
       <c r="I220" s="3" t="n"/>
       <c r="J220" s="3" t="n"/>
-      <c r="K220" s="5" t="n"/>
-      <c r="L220" s="5" t="n"/>
+      <c r="K220" s="3" t="n"/>
+      <c r="L220" s="3" t="n"/>
       <c r="M220" s="5" t="n"/>
       <c r="N220" s="5" t="n"/>
       <c r="O220" s="5" t="n"/>
@@ -6707,6 +7165,8 @@
       <c r="W220" s="5" t="n"/>
       <c r="X220" s="5" t="n"/>
       <c r="Y220" s="5" t="n"/>
+      <c r="Z220" s="5" t="n"/>
+      <c r="AA220" s="5" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="6" t="n"/>
@@ -6734,6 +7194,8 @@
       <c r="W221" s="6" t="n"/>
       <c r="X221" s="6" t="n"/>
       <c r="Y221" s="6" t="n"/>
+      <c r="Z221" s="6" t="n"/>
+      <c r="AA221" s="6" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="3" t="n"/>
@@ -6746,8 +7208,8 @@
       <c r="H222" s="3" t="n"/>
       <c r="I222" s="3" t="n"/>
       <c r="J222" s="3" t="n"/>
-      <c r="K222" s="5" t="n"/>
-      <c r="L222" s="5" t="n"/>
+      <c r="K222" s="3" t="n"/>
+      <c r="L222" s="3" t="n"/>
       <c r="M222" s="5" t="n"/>
       <c r="N222" s="5" t="n"/>
       <c r="O222" s="5" t="n"/>
@@ -6761,6 +7223,8 @@
       <c r="W222" s="5" t="n"/>
       <c r="X222" s="5" t="n"/>
       <c r="Y222" s="5" t="n"/>
+      <c r="Z222" s="5" t="n"/>
+      <c r="AA222" s="5" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="6" t="n"/>
@@ -6788,6 +7252,8 @@
       <c r="W223" s="6" t="n"/>
       <c r="X223" s="6" t="n"/>
       <c r="Y223" s="6" t="n"/>
+      <c r="Z223" s="6" t="n"/>
+      <c r="AA223" s="6" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="3" t="n"/>
@@ -6800,8 +7266,8 @@
       <c r="H224" s="3" t="n"/>
       <c r="I224" s="3" t="n"/>
       <c r="J224" s="3" t="n"/>
-      <c r="K224" s="5" t="n"/>
-      <c r="L224" s="5" t="n"/>
+      <c r="K224" s="3" t="n"/>
+      <c r="L224" s="3" t="n"/>
       <c r="M224" s="5" t="n"/>
       <c r="N224" s="5" t="n"/>
       <c r="O224" s="5" t="n"/>
@@ -6815,6 +7281,8 @@
       <c r="W224" s="5" t="n"/>
       <c r="X224" s="5" t="n"/>
       <c r="Y224" s="5" t="n"/>
+      <c r="Z224" s="5" t="n"/>
+      <c r="AA224" s="5" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="6" t="n"/>
@@ -6842,6 +7310,8 @@
       <c r="W225" s="6" t="n"/>
       <c r="X225" s="6" t="n"/>
       <c r="Y225" s="6" t="n"/>
+      <c r="Z225" s="6" t="n"/>
+      <c r="AA225" s="6" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="3" t="n"/>
@@ -6854,8 +7324,8 @@
       <c r="H226" s="3" t="n"/>
       <c r="I226" s="3" t="n"/>
       <c r="J226" s="3" t="n"/>
-      <c r="K226" s="5" t="n"/>
-      <c r="L226" s="5" t="n"/>
+      <c r="K226" s="3" t="n"/>
+      <c r="L226" s="3" t="n"/>
       <c r="M226" s="5" t="n"/>
       <c r="N226" s="5" t="n"/>
       <c r="O226" s="5" t="n"/>
@@ -6869,6 +7339,8 @@
       <c r="W226" s="5" t="n"/>
       <c r="X226" s="5" t="n"/>
       <c r="Y226" s="5" t="n"/>
+      <c r="Z226" s="5" t="n"/>
+      <c r="AA226" s="5" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="6" t="n"/>
@@ -6896,6 +7368,8 @@
       <c r="W227" s="6" t="n"/>
       <c r="X227" s="6" t="n"/>
       <c r="Y227" s="6" t="n"/>
+      <c r="Z227" s="6" t="n"/>
+      <c r="AA227" s="6" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="3" t="n"/>
@@ -6908,8 +7382,8 @@
       <c r="H228" s="3" t="n"/>
       <c r="I228" s="3" t="n"/>
       <c r="J228" s="3" t="n"/>
-      <c r="K228" s="5" t="n"/>
-      <c r="L228" s="5" t="n"/>
+      <c r="K228" s="3" t="n"/>
+      <c r="L228" s="3" t="n"/>
       <c r="M228" s="5" t="n"/>
       <c r="N228" s="5" t="n"/>
       <c r="O228" s="5" t="n"/>
@@ -6923,6 +7397,8 @@
       <c r="W228" s="5" t="n"/>
       <c r="X228" s="5" t="n"/>
       <c r="Y228" s="5" t="n"/>
+      <c r="Z228" s="5" t="n"/>
+      <c r="AA228" s="5" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="6" t="n"/>
@@ -6950,6 +7426,8 @@
       <c r="W229" s="6" t="n"/>
       <c r="X229" s="6" t="n"/>
       <c r="Y229" s="6" t="n"/>
+      <c r="Z229" s="6" t="n"/>
+      <c r="AA229" s="6" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="3" t="n"/>
@@ -6962,8 +7440,8 @@
       <c r="H230" s="3" t="n"/>
       <c r="I230" s="3" t="n"/>
       <c r="J230" s="3" t="n"/>
-      <c r="K230" s="5" t="n"/>
-      <c r="L230" s="5" t="n"/>
+      <c r="K230" s="3" t="n"/>
+      <c r="L230" s="3" t="n"/>
       <c r="M230" s="5" t="n"/>
       <c r="N230" s="5" t="n"/>
       <c r="O230" s="5" t="n"/>
@@ -6977,6 +7455,8 @@
       <c r="W230" s="5" t="n"/>
       <c r="X230" s="5" t="n"/>
       <c r="Y230" s="5" t="n"/>
+      <c r="Z230" s="5" t="n"/>
+      <c r="AA230" s="5" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="6" t="n"/>
@@ -7004,6 +7484,8 @@
       <c r="W231" s="6" t="n"/>
       <c r="X231" s="6" t="n"/>
       <c r="Y231" s="6" t="n"/>
+      <c r="Z231" s="6" t="n"/>
+      <c r="AA231" s="6" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="3" t="n"/>
@@ -7016,8 +7498,8 @@
       <c r="H232" s="3" t="n"/>
       <c r="I232" s="3" t="n"/>
       <c r="J232" s="3" t="n"/>
-      <c r="K232" s="5" t="n"/>
-      <c r="L232" s="5" t="n"/>
+      <c r="K232" s="3" t="n"/>
+      <c r="L232" s="3" t="n"/>
       <c r="M232" s="5" t="n"/>
       <c r="N232" s="5" t="n"/>
       <c r="O232" s="5" t="n"/>
@@ -7031,6 +7513,8 @@
       <c r="W232" s="5" t="n"/>
       <c r="X232" s="5" t="n"/>
       <c r="Y232" s="5" t="n"/>
+      <c r="Z232" s="5" t="n"/>
+      <c r="AA232" s="5" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="6" t="n"/>
@@ -7058,6 +7542,8 @@
       <c r="W233" s="6" t="n"/>
       <c r="X233" s="6" t="n"/>
       <c r="Y233" s="6" t="n"/>
+      <c r="Z233" s="6" t="n"/>
+      <c r="AA233" s="6" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="3" t="n"/>
@@ -7070,8 +7556,8 @@
       <c r="H234" s="3" t="n"/>
       <c r="I234" s="3" t="n"/>
       <c r="J234" s="3" t="n"/>
-      <c r="K234" s="5" t="n"/>
-      <c r="L234" s="5" t="n"/>
+      <c r="K234" s="3" t="n"/>
+      <c r="L234" s="3" t="n"/>
       <c r="M234" s="5" t="n"/>
       <c r="N234" s="5" t="n"/>
       <c r="O234" s="5" t="n"/>
@@ -7085,6 +7571,8 @@
       <c r="W234" s="5" t="n"/>
       <c r="X234" s="5" t="n"/>
       <c r="Y234" s="5" t="n"/>
+      <c r="Z234" s="5" t="n"/>
+      <c r="AA234" s="5" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="6" t="n"/>
@@ -7112,6 +7600,8 @@
       <c r="W235" s="6" t="n"/>
       <c r="X235" s="6" t="n"/>
       <c r="Y235" s="6" t="n"/>
+      <c r="Z235" s="6" t="n"/>
+      <c r="AA235" s="6" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="3" t="n"/>
@@ -7124,8 +7614,8 @@
       <c r="H236" s="3" t="n"/>
       <c r="I236" s="3" t="n"/>
       <c r="J236" s="3" t="n"/>
-      <c r="K236" s="5" t="n"/>
-      <c r="L236" s="5" t="n"/>
+      <c r="K236" s="3" t="n"/>
+      <c r="L236" s="3" t="n"/>
       <c r="M236" s="5" t="n"/>
       <c r="N236" s="5" t="n"/>
       <c r="O236" s="5" t="n"/>
@@ -7139,6 +7629,8 @@
       <c r="W236" s="5" t="n"/>
       <c r="X236" s="5" t="n"/>
       <c r="Y236" s="5" t="n"/>
+      <c r="Z236" s="5" t="n"/>
+      <c r="AA236" s="5" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="6" t="n"/>
@@ -7166,6 +7658,8 @@
       <c r="W237" s="6" t="n"/>
       <c r="X237" s="6" t="n"/>
       <c r="Y237" s="6" t="n"/>
+      <c r="Z237" s="6" t="n"/>
+      <c r="AA237" s="6" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="3" t="n"/>
@@ -7178,8 +7672,8 @@
       <c r="H238" s="3" t="n"/>
       <c r="I238" s="3" t="n"/>
       <c r="J238" s="3" t="n"/>
-      <c r="K238" s="5" t="n"/>
-      <c r="L238" s="5" t="n"/>
+      <c r="K238" s="3" t="n"/>
+      <c r="L238" s="3" t="n"/>
       <c r="M238" s="5" t="n"/>
       <c r="N238" s="5" t="n"/>
       <c r="O238" s="5" t="n"/>
@@ -7193,6 +7687,8 @@
       <c r="W238" s="5" t="n"/>
       <c r="X238" s="5" t="n"/>
       <c r="Y238" s="5" t="n"/>
+      <c r="Z238" s="5" t="n"/>
+      <c r="AA238" s="5" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="6" t="n"/>
@@ -7220,6 +7716,8 @@
       <c r="W239" s="6" t="n"/>
       <c r="X239" s="6" t="n"/>
       <c r="Y239" s="6" t="n"/>
+      <c r="Z239" s="6" t="n"/>
+      <c r="AA239" s="6" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="3" t="n"/>
@@ -7232,8 +7730,8 @@
       <c r="H240" s="3" t="n"/>
       <c r="I240" s="3" t="n"/>
       <c r="J240" s="3" t="n"/>
-      <c r="K240" s="5" t="n"/>
-      <c r="L240" s="5" t="n"/>
+      <c r="K240" s="3" t="n"/>
+      <c r="L240" s="3" t="n"/>
       <c r="M240" s="5" t="n"/>
       <c r="N240" s="5" t="n"/>
       <c r="O240" s="5" t="n"/>
@@ -7247,6 +7745,8 @@
       <c r="W240" s="5" t="n"/>
       <c r="X240" s="5" t="n"/>
       <c r="Y240" s="5" t="n"/>
+      <c r="Z240" s="5" t="n"/>
+      <c r="AA240" s="5" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="6" t="n"/>
@@ -7274,6 +7774,8 @@
       <c r="W241" s="6" t="n"/>
       <c r="X241" s="6" t="n"/>
       <c r="Y241" s="6" t="n"/>
+      <c r="Z241" s="6" t="n"/>
+      <c r="AA241" s="6" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="3" t="n"/>
@@ -7286,8 +7788,8 @@
       <c r="H242" s="3" t="n"/>
       <c r="I242" s="3" t="n"/>
       <c r="J242" s="3" t="n"/>
-      <c r="K242" s="5" t="n"/>
-      <c r="L242" s="5" t="n"/>
+      <c r="K242" s="3" t="n"/>
+      <c r="L242" s="3" t="n"/>
       <c r="M242" s="5" t="n"/>
       <c r="N242" s="5" t="n"/>
       <c r="O242" s="5" t="n"/>
@@ -7301,6 +7803,8 @@
       <c r="W242" s="5" t="n"/>
       <c r="X242" s="5" t="n"/>
       <c r="Y242" s="5" t="n"/>
+      <c r="Z242" s="5" t="n"/>
+      <c r="AA242" s="5" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="6" t="n"/>
@@ -7328,6 +7832,8 @@
       <c r="W243" s="6" t="n"/>
       <c r="X243" s="6" t="n"/>
       <c r="Y243" s="6" t="n"/>
+      <c r="Z243" s="6" t="n"/>
+      <c r="AA243" s="6" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="3" t="n"/>
@@ -7340,8 +7846,8 @@
       <c r="H244" s="3" t="n"/>
       <c r="I244" s="3" t="n"/>
       <c r="J244" s="3" t="n"/>
-      <c r="K244" s="5" t="n"/>
-      <c r="L244" s="5" t="n"/>
+      <c r="K244" s="3" t="n"/>
+      <c r="L244" s="3" t="n"/>
       <c r="M244" s="5" t="n"/>
       <c r="N244" s="5" t="n"/>
       <c r="O244" s="5" t="n"/>
@@ -7355,6 +7861,8 @@
       <c r="W244" s="5" t="n"/>
       <c r="X244" s="5" t="n"/>
       <c r="Y244" s="5" t="n"/>
+      <c r="Z244" s="5" t="n"/>
+      <c r="AA244" s="5" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="6" t="n"/>
@@ -7382,6 +7890,8 @@
       <c r="W245" s="6" t="n"/>
       <c r="X245" s="6" t="n"/>
       <c r="Y245" s="6" t="n"/>
+      <c r="Z245" s="6" t="n"/>
+      <c r="AA245" s="6" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="3" t="n"/>
@@ -7394,8 +7904,8 @@
       <c r="H246" s="3" t="n"/>
       <c r="I246" s="3" t="n"/>
       <c r="J246" s="3" t="n"/>
-      <c r="K246" s="5" t="n"/>
-      <c r="L246" s="5" t="n"/>
+      <c r="K246" s="3" t="n"/>
+      <c r="L246" s="3" t="n"/>
       <c r="M246" s="5" t="n"/>
       <c r="N246" s="5" t="n"/>
       <c r="O246" s="5" t="n"/>
@@ -7409,6 +7919,8 @@
       <c r="W246" s="5" t="n"/>
       <c r="X246" s="5" t="n"/>
       <c r="Y246" s="5" t="n"/>
+      <c r="Z246" s="5" t="n"/>
+      <c r="AA246" s="5" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="6" t="n"/>
@@ -7436,6 +7948,8 @@
       <c r="W247" s="6" t="n"/>
       <c r="X247" s="6" t="n"/>
       <c r="Y247" s="6" t="n"/>
+      <c r="Z247" s="6" t="n"/>
+      <c r="AA247" s="6" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="3" t="n"/>
@@ -7448,8 +7962,8 @@
       <c r="H248" s="3" t="n"/>
       <c r="I248" s="3" t="n"/>
       <c r="J248" s="3" t="n"/>
-      <c r="K248" s="5" t="n"/>
-      <c r="L248" s="5" t="n"/>
+      <c r="K248" s="3" t="n"/>
+      <c r="L248" s="3" t="n"/>
       <c r="M248" s="5" t="n"/>
       <c r="N248" s="5" t="n"/>
       <c r="O248" s="5" t="n"/>
@@ -7463,6 +7977,8 @@
       <c r="W248" s="5" t="n"/>
       <c r="X248" s="5" t="n"/>
       <c r="Y248" s="5" t="n"/>
+      <c r="Z248" s="5" t="n"/>
+      <c r="AA248" s="5" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="6" t="n"/>
@@ -7490,6 +8006,8 @@
       <c r="W249" s="6" t="n"/>
       <c r="X249" s="6" t="n"/>
       <c r="Y249" s="6" t="n"/>
+      <c r="Z249" s="6" t="n"/>
+      <c r="AA249" s="6" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="3" t="n"/>
@@ -7502,8 +8020,8 @@
       <c r="H250" s="3" t="n"/>
       <c r="I250" s="3" t="n"/>
       <c r="J250" s="3" t="n"/>
-      <c r="K250" s="5" t="n"/>
-      <c r="L250" s="5" t="n"/>
+      <c r="K250" s="3" t="n"/>
+      <c r="L250" s="3" t="n"/>
       <c r="M250" s="5" t="n"/>
       <c r="N250" s="5" t="n"/>
       <c r="O250" s="5" t="n"/>
@@ -7517,6 +8035,8 @@
       <c r="W250" s="5" t="n"/>
       <c r="X250" s="5" t="n"/>
       <c r="Y250" s="5" t="n"/>
+      <c r="Z250" s="5" t="n"/>
+      <c r="AA250" s="5" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="6" t="n"/>
@@ -7544,6 +8064,8 @@
       <c r="W251" s="6" t="n"/>
       <c r="X251" s="6" t="n"/>
       <c r="Y251" s="6" t="n"/>
+      <c r="Z251" s="6" t="n"/>
+      <c r="AA251" s="6" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="3" t="n"/>
@@ -7556,8 +8078,8 @@
       <c r="H252" s="3" t="n"/>
       <c r="I252" s="3" t="n"/>
       <c r="J252" s="3" t="n"/>
-      <c r="K252" s="5" t="n"/>
-      <c r="L252" s="5" t="n"/>
+      <c r="K252" s="3" t="n"/>
+      <c r="L252" s="3" t="n"/>
       <c r="M252" s="5" t="n"/>
       <c r="N252" s="5" t="n"/>
       <c r="O252" s="5" t="n"/>
@@ -7571,6 +8093,8 @@
       <c r="W252" s="5" t="n"/>
       <c r="X252" s="5" t="n"/>
       <c r="Y252" s="5" t="n"/>
+      <c r="Z252" s="5" t="n"/>
+      <c r="AA252" s="5" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="6" t="n"/>
@@ -7598,6 +8122,8 @@
       <c r="W253" s="6" t="n"/>
       <c r="X253" s="6" t="n"/>
       <c r="Y253" s="6" t="n"/>
+      <c r="Z253" s="6" t="n"/>
+      <c r="AA253" s="6" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="3" t="n"/>
@@ -7610,8 +8136,8 @@
       <c r="H254" s="3" t="n"/>
       <c r="I254" s="3" t="n"/>
       <c r="J254" s="3" t="n"/>
-      <c r="K254" s="5" t="n"/>
-      <c r="L254" s="5" t="n"/>
+      <c r="K254" s="3" t="n"/>
+      <c r="L254" s="3" t="n"/>
       <c r="M254" s="5" t="n"/>
       <c r="N254" s="5" t="n"/>
       <c r="O254" s="5" t="n"/>
@@ -7625,6 +8151,8 @@
       <c r="W254" s="5" t="n"/>
       <c r="X254" s="5" t="n"/>
       <c r="Y254" s="5" t="n"/>
+      <c r="Z254" s="5" t="n"/>
+      <c r="AA254" s="5" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="6" t="n"/>
@@ -7652,6 +8180,8 @@
       <c r="W255" s="6" t="n"/>
       <c r="X255" s="6" t="n"/>
       <c r="Y255" s="6" t="n"/>
+      <c r="Z255" s="6" t="n"/>
+      <c r="AA255" s="6" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="3" t="n"/>
@@ -7664,8 +8194,8 @@
       <c r="H256" s="3" t="n"/>
       <c r="I256" s="3" t="n"/>
       <c r="J256" s="3" t="n"/>
-      <c r="K256" s="5" t="n"/>
-      <c r="L256" s="5" t="n"/>
+      <c r="K256" s="3" t="n"/>
+      <c r="L256" s="3" t="n"/>
       <c r="M256" s="5" t="n"/>
       <c r="N256" s="5" t="n"/>
       <c r="O256" s="5" t="n"/>
@@ -7679,6 +8209,8 @@
       <c r="W256" s="5" t="n"/>
       <c r="X256" s="5" t="n"/>
       <c r="Y256" s="5" t="n"/>
+      <c r="Z256" s="5" t="n"/>
+      <c r="AA256" s="5" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="6" t="n"/>
@@ -7706,6 +8238,8 @@
       <c r="W257" s="6" t="n"/>
       <c r="X257" s="6" t="n"/>
       <c r="Y257" s="6" t="n"/>
+      <c r="Z257" s="6" t="n"/>
+      <c r="AA257" s="6" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="3" t="n"/>
@@ -7718,8 +8252,8 @@
       <c r="H258" s="3" t="n"/>
       <c r="I258" s="3" t="n"/>
       <c r="J258" s="3" t="n"/>
-      <c r="K258" s="5" t="n"/>
-      <c r="L258" s="5" t="n"/>
+      <c r="K258" s="3" t="n"/>
+      <c r="L258" s="3" t="n"/>
       <c r="M258" s="5" t="n"/>
       <c r="N258" s="5" t="n"/>
       <c r="O258" s="5" t="n"/>
@@ -7733,6 +8267,8 @@
       <c r="W258" s="5" t="n"/>
       <c r="X258" s="5" t="n"/>
       <c r="Y258" s="5" t="n"/>
+      <c r="Z258" s="5" t="n"/>
+      <c r="AA258" s="5" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="6" t="n"/>
@@ -7760,6 +8296,8 @@
       <c r="W259" s="6" t="n"/>
       <c r="X259" s="6" t="n"/>
       <c r="Y259" s="6" t="n"/>
+      <c r="Z259" s="6" t="n"/>
+      <c r="AA259" s="6" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="3" t="n"/>
@@ -7772,8 +8310,8 @@
       <c r="H260" s="3" t="n"/>
       <c r="I260" s="3" t="n"/>
       <c r="J260" s="3" t="n"/>
-      <c r="K260" s="5" t="n"/>
-      <c r="L260" s="5" t="n"/>
+      <c r="K260" s="3" t="n"/>
+      <c r="L260" s="3" t="n"/>
       <c r="M260" s="5" t="n"/>
       <c r="N260" s="5" t="n"/>
       <c r="O260" s="5" t="n"/>
@@ -7787,6 +8325,8 @@
       <c r="W260" s="5" t="n"/>
       <c r="X260" s="5" t="n"/>
       <c r="Y260" s="5" t="n"/>
+      <c r="Z260" s="5" t="n"/>
+      <c r="AA260" s="5" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="6" t="n"/>
@@ -7814,6 +8354,8 @@
       <c r="W261" s="6" t="n"/>
       <c r="X261" s="6" t="n"/>
       <c r="Y261" s="6" t="n"/>
+      <c r="Z261" s="6" t="n"/>
+      <c r="AA261" s="6" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="3" t="n"/>
@@ -7826,8 +8368,8 @@
       <c r="H262" s="3" t="n"/>
       <c r="I262" s="3" t="n"/>
       <c r="J262" s="3" t="n"/>
-      <c r="K262" s="5" t="n"/>
-      <c r="L262" s="5" t="n"/>
+      <c r="K262" s="3" t="n"/>
+      <c r="L262" s="3" t="n"/>
       <c r="M262" s="5" t="n"/>
       <c r="N262" s="5" t="n"/>
       <c r="O262" s="5" t="n"/>
@@ -7841,6 +8383,8 @@
       <c r="W262" s="5" t="n"/>
       <c r="X262" s="5" t="n"/>
       <c r="Y262" s="5" t="n"/>
+      <c r="Z262" s="5" t="n"/>
+      <c r="AA262" s="5" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="6" t="n"/>
@@ -7868,6 +8412,8 @@
       <c r="W263" s="6" t="n"/>
       <c r="X263" s="6" t="n"/>
       <c r="Y263" s="6" t="n"/>
+      <c r="Z263" s="6" t="n"/>
+      <c r="AA263" s="6" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="3" t="n"/>
@@ -7880,8 +8426,8 @@
       <c r="H264" s="3" t="n"/>
       <c r="I264" s="3" t="n"/>
       <c r="J264" s="3" t="n"/>
-      <c r="K264" s="5" t="n"/>
-      <c r="L264" s="5" t="n"/>
+      <c r="K264" s="3" t="n"/>
+      <c r="L264" s="3" t="n"/>
       <c r="M264" s="5" t="n"/>
       <c r="N264" s="5" t="n"/>
       <c r="O264" s="5" t="n"/>
@@ -7895,6 +8441,8 @@
       <c r="W264" s="5" t="n"/>
       <c r="X264" s="5" t="n"/>
       <c r="Y264" s="5" t="n"/>
+      <c r="Z264" s="5" t="n"/>
+      <c r="AA264" s="5" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="6" t="n"/>
@@ -7922,6 +8470,8 @@
       <c r="W265" s="6" t="n"/>
       <c r="X265" s="6" t="n"/>
       <c r="Y265" s="6" t="n"/>
+      <c r="Z265" s="6" t="n"/>
+      <c r="AA265" s="6" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="3" t="n"/>
@@ -7934,8 +8484,8 @@
       <c r="H266" s="3" t="n"/>
       <c r="I266" s="3" t="n"/>
       <c r="J266" s="3" t="n"/>
-      <c r="K266" s="5" t="n"/>
-      <c r="L266" s="5" t="n"/>
+      <c r="K266" s="3" t="n"/>
+      <c r="L266" s="3" t="n"/>
       <c r="M266" s="5" t="n"/>
       <c r="N266" s="5" t="n"/>
       <c r="O266" s="5" t="n"/>
@@ -7949,6 +8499,8 @@
       <c r="W266" s="5" t="n"/>
       <c r="X266" s="5" t="n"/>
       <c r="Y266" s="5" t="n"/>
+      <c r="Z266" s="5" t="n"/>
+      <c r="AA266" s="5" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="6" t="n"/>
@@ -7976,6 +8528,8 @@
       <c r="W267" s="6" t="n"/>
       <c r="X267" s="6" t="n"/>
       <c r="Y267" s="6" t="n"/>
+      <c r="Z267" s="6" t="n"/>
+      <c r="AA267" s="6" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="3" t="n"/>
@@ -7988,8 +8542,8 @@
       <c r="H268" s="3" t="n"/>
       <c r="I268" s="3" t="n"/>
       <c r="J268" s="3" t="n"/>
-      <c r="K268" s="5" t="n"/>
-      <c r="L268" s="5" t="n"/>
+      <c r="K268" s="3" t="n"/>
+      <c r="L268" s="3" t="n"/>
       <c r="M268" s="5" t="n"/>
       <c r="N268" s="5" t="n"/>
       <c r="O268" s="5" t="n"/>
@@ -8003,6 +8557,8 @@
       <c r="W268" s="5" t="n"/>
       <c r="X268" s="5" t="n"/>
       <c r="Y268" s="5" t="n"/>
+      <c r="Z268" s="5" t="n"/>
+      <c r="AA268" s="5" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="6" t="n"/>
@@ -8030,6 +8586,8 @@
       <c r="W269" s="6" t="n"/>
       <c r="X269" s="6" t="n"/>
       <c r="Y269" s="6" t="n"/>
+      <c r="Z269" s="6" t="n"/>
+      <c r="AA269" s="6" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="3" t="n"/>
@@ -8042,8 +8600,8 @@
       <c r="H270" s="3" t="n"/>
       <c r="I270" s="3" t="n"/>
       <c r="J270" s="3" t="n"/>
-      <c r="K270" s="5" t="n"/>
-      <c r="L270" s="5" t="n"/>
+      <c r="K270" s="3" t="n"/>
+      <c r="L270" s="3" t="n"/>
       <c r="M270" s="5" t="n"/>
       <c r="N270" s="5" t="n"/>
       <c r="O270" s="5" t="n"/>
@@ -8057,6 +8615,8 @@
       <c r="W270" s="5" t="n"/>
       <c r="X270" s="5" t="n"/>
       <c r="Y270" s="5" t="n"/>
+      <c r="Z270" s="5" t="n"/>
+      <c r="AA270" s="5" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="6" t="n"/>
@@ -8084,6 +8644,8 @@
       <c r="W271" s="6" t="n"/>
       <c r="X271" s="6" t="n"/>
       <c r="Y271" s="6" t="n"/>
+      <c r="Z271" s="6" t="n"/>
+      <c r="AA271" s="6" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="3" t="n"/>
@@ -8096,8 +8658,8 @@
       <c r="H272" s="3" t="n"/>
       <c r="I272" s="3" t="n"/>
       <c r="J272" s="3" t="n"/>
-      <c r="K272" s="5" t="n"/>
-      <c r="L272" s="5" t="n"/>
+      <c r="K272" s="3" t="n"/>
+      <c r="L272" s="3" t="n"/>
       <c r="M272" s="5" t="n"/>
       <c r="N272" s="5" t="n"/>
       <c r="O272" s="5" t="n"/>
@@ -8111,6 +8673,8 @@
       <c r="W272" s="5" t="n"/>
       <c r="X272" s="5" t="n"/>
       <c r="Y272" s="5" t="n"/>
+      <c r="Z272" s="5" t="n"/>
+      <c r="AA272" s="5" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="6" t="n"/>
@@ -8138,6 +8702,8 @@
       <c r="W273" s="6" t="n"/>
       <c r="X273" s="6" t="n"/>
       <c r="Y273" s="6" t="n"/>
+      <c r="Z273" s="6" t="n"/>
+      <c r="AA273" s="6" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="3" t="n"/>
@@ -8150,8 +8716,8 @@
       <c r="H274" s="3" t="n"/>
       <c r="I274" s="3" t="n"/>
       <c r="J274" s="3" t="n"/>
-      <c r="K274" s="5" t="n"/>
-      <c r="L274" s="5" t="n"/>
+      <c r="K274" s="3" t="n"/>
+      <c r="L274" s="3" t="n"/>
       <c r="M274" s="5" t="n"/>
       <c r="N274" s="5" t="n"/>
       <c r="O274" s="5" t="n"/>
@@ -8165,6 +8731,8 @@
       <c r="W274" s="5" t="n"/>
       <c r="X274" s="5" t="n"/>
       <c r="Y274" s="5" t="n"/>
+      <c r="Z274" s="5" t="n"/>
+      <c r="AA274" s="5" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="6" t="n"/>
@@ -8192,6 +8760,8 @@
       <c r="W275" s="6" t="n"/>
       <c r="X275" s="6" t="n"/>
       <c r="Y275" s="6" t="n"/>
+      <c r="Z275" s="6" t="n"/>
+      <c r="AA275" s="6" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="3" t="n"/>
@@ -8204,8 +8774,8 @@
       <c r="H276" s="3" t="n"/>
       <c r="I276" s="3" t="n"/>
       <c r="J276" s="3" t="n"/>
-      <c r="K276" s="5" t="n"/>
-      <c r="L276" s="5" t="n"/>
+      <c r="K276" s="3" t="n"/>
+      <c r="L276" s="3" t="n"/>
       <c r="M276" s="5" t="n"/>
       <c r="N276" s="5" t="n"/>
       <c r="O276" s="5" t="n"/>
@@ -8219,6 +8789,8 @@
       <c r="W276" s="5" t="n"/>
       <c r="X276" s="5" t="n"/>
       <c r="Y276" s="5" t="n"/>
+      <c r="Z276" s="5" t="n"/>
+      <c r="AA276" s="5" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="6" t="n"/>
@@ -8246,6 +8818,8 @@
       <c r="W277" s="6" t="n"/>
       <c r="X277" s="6" t="n"/>
       <c r="Y277" s="6" t="n"/>
+      <c r="Z277" s="6" t="n"/>
+      <c r="AA277" s="6" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="3" t="n"/>
@@ -8258,8 +8832,8 @@
       <c r="H278" s="3" t="n"/>
       <c r="I278" s="3" t="n"/>
       <c r="J278" s="3" t="n"/>
-      <c r="K278" s="5" t="n"/>
-      <c r="L278" s="5" t="n"/>
+      <c r="K278" s="3" t="n"/>
+      <c r="L278" s="3" t="n"/>
       <c r="M278" s="5" t="n"/>
       <c r="N278" s="5" t="n"/>
       <c r="O278" s="5" t="n"/>
@@ -8273,6 +8847,8 @@
       <c r="W278" s="5" t="n"/>
       <c r="X278" s="5" t="n"/>
       <c r="Y278" s="5" t="n"/>
+      <c r="Z278" s="5" t="n"/>
+      <c r="AA278" s="5" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="6" t="n"/>
@@ -8300,6 +8876,8 @@
       <c r="W279" s="6" t="n"/>
       <c r="X279" s="6" t="n"/>
       <c r="Y279" s="6" t="n"/>
+      <c r="Z279" s="6" t="n"/>
+      <c r="AA279" s="6" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="3" t="n"/>
@@ -8312,8 +8890,8 @@
       <c r="H280" s="3" t="n"/>
       <c r="I280" s="3" t="n"/>
       <c r="J280" s="3" t="n"/>
-      <c r="K280" s="5" t="n"/>
-      <c r="L280" s="5" t="n"/>
+      <c r="K280" s="3" t="n"/>
+      <c r="L280" s="3" t="n"/>
       <c r="M280" s="5" t="n"/>
       <c r="N280" s="5" t="n"/>
       <c r="O280" s="5" t="n"/>
@@ -8327,6 +8905,8 @@
       <c r="W280" s="5" t="n"/>
       <c r="X280" s="5" t="n"/>
       <c r="Y280" s="5" t="n"/>
+      <c r="Z280" s="5" t="n"/>
+      <c r="AA280" s="5" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="6" t="n"/>
@@ -8354,6 +8934,8 @@
       <c r="W281" s="6" t="n"/>
       <c r="X281" s="6" t="n"/>
       <c r="Y281" s="6" t="n"/>
+      <c r="Z281" s="6" t="n"/>
+      <c r="AA281" s="6" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="3" t="n"/>
@@ -8366,8 +8948,8 @@
       <c r="H282" s="3" t="n"/>
       <c r="I282" s="3" t="n"/>
       <c r="J282" s="3" t="n"/>
-      <c r="K282" s="5" t="n"/>
-      <c r="L282" s="5" t="n"/>
+      <c r="K282" s="3" t="n"/>
+      <c r="L282" s="3" t="n"/>
       <c r="M282" s="5" t="n"/>
       <c r="N282" s="5" t="n"/>
       <c r="O282" s="5" t="n"/>
@@ -8381,6 +8963,8 @@
       <c r="W282" s="5" t="n"/>
       <c r="X282" s="5" t="n"/>
       <c r="Y282" s="5" t="n"/>
+      <c r="Z282" s="5" t="n"/>
+      <c r="AA282" s="5" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="6" t="n"/>
@@ -8408,6 +8992,8 @@
       <c r="W283" s="6" t="n"/>
       <c r="X283" s="6" t="n"/>
       <c r="Y283" s="6" t="n"/>
+      <c r="Z283" s="6" t="n"/>
+      <c r="AA283" s="6" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="3" t="n"/>
@@ -8420,8 +9006,8 @@
       <c r="H284" s="3" t="n"/>
       <c r="I284" s="3" t="n"/>
       <c r="J284" s="3" t="n"/>
-      <c r="K284" s="5" t="n"/>
-      <c r="L284" s="5" t="n"/>
+      <c r="K284" s="3" t="n"/>
+      <c r="L284" s="3" t="n"/>
       <c r="M284" s="5" t="n"/>
       <c r="N284" s="5" t="n"/>
       <c r="O284" s="5" t="n"/>
@@ -8435,6 +9021,8 @@
       <c r="W284" s="5" t="n"/>
       <c r="X284" s="5" t="n"/>
       <c r="Y284" s="5" t="n"/>
+      <c r="Z284" s="5" t="n"/>
+      <c r="AA284" s="5" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="6" t="n"/>
@@ -8462,6 +9050,8 @@
       <c r="W285" s="6" t="n"/>
       <c r="X285" s="6" t="n"/>
       <c r="Y285" s="6" t="n"/>
+      <c r="Z285" s="6" t="n"/>
+      <c r="AA285" s="6" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="3" t="n"/>
@@ -8474,8 +9064,8 @@
       <c r="H286" s="3" t="n"/>
       <c r="I286" s="3" t="n"/>
       <c r="J286" s="3" t="n"/>
-      <c r="K286" s="5" t="n"/>
-      <c r="L286" s="5" t="n"/>
+      <c r="K286" s="3" t="n"/>
+      <c r="L286" s="3" t="n"/>
       <c r="M286" s="5" t="n"/>
       <c r="N286" s="5" t="n"/>
       <c r="O286" s="5" t="n"/>
@@ -8489,6 +9079,8 @@
       <c r="W286" s="5" t="n"/>
       <c r="X286" s="5" t="n"/>
       <c r="Y286" s="5" t="n"/>
+      <c r="Z286" s="5" t="n"/>
+      <c r="AA286" s="5" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="6" t="n"/>
@@ -8516,6 +9108,8 @@
       <c r="W287" s="6" t="n"/>
       <c r="X287" s="6" t="n"/>
       <c r="Y287" s="6" t="n"/>
+      <c r="Z287" s="6" t="n"/>
+      <c r="AA287" s="6" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="3" t="n"/>
@@ -8528,8 +9122,8 @@
       <c r="H288" s="3" t="n"/>
       <c r="I288" s="3" t="n"/>
       <c r="J288" s="3" t="n"/>
-      <c r="K288" s="5" t="n"/>
-      <c r="L288" s="5" t="n"/>
+      <c r="K288" s="3" t="n"/>
+      <c r="L288" s="3" t="n"/>
       <c r="M288" s="5" t="n"/>
       <c r="N288" s="5" t="n"/>
       <c r="O288" s="5" t="n"/>
@@ -8543,6 +9137,8 @@
       <c r="W288" s="5" t="n"/>
       <c r="X288" s="5" t="n"/>
       <c r="Y288" s="5" t="n"/>
+      <c r="Z288" s="5" t="n"/>
+      <c r="AA288" s="5" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="6" t="n"/>
@@ -8570,6 +9166,8 @@
       <c r="W289" s="6" t="n"/>
       <c r="X289" s="6" t="n"/>
       <c r="Y289" s="6" t="n"/>
+      <c r="Z289" s="6" t="n"/>
+      <c r="AA289" s="6" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="3" t="n"/>
@@ -8582,8 +9180,8 @@
       <c r="H290" s="3" t="n"/>
       <c r="I290" s="3" t="n"/>
       <c r="J290" s="3" t="n"/>
-      <c r="K290" s="5" t="n"/>
-      <c r="L290" s="5" t="n"/>
+      <c r="K290" s="3" t="n"/>
+      <c r="L290" s="3" t="n"/>
       <c r="M290" s="5" t="n"/>
       <c r="N290" s="5" t="n"/>
       <c r="O290" s="5" t="n"/>
@@ -8597,6 +9195,8 @@
       <c r="W290" s="5" t="n"/>
       <c r="X290" s="5" t="n"/>
       <c r="Y290" s="5" t="n"/>
+      <c r="Z290" s="5" t="n"/>
+      <c r="AA290" s="5" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="6" t="n"/>
@@ -8624,6 +9224,8 @@
       <c r="W291" s="6" t="n"/>
       <c r="X291" s="6" t="n"/>
       <c r="Y291" s="6" t="n"/>
+      <c r="Z291" s="6" t="n"/>
+      <c r="AA291" s="6" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="3" t="n"/>
@@ -8636,8 +9238,8 @@
       <c r="H292" s="3" t="n"/>
       <c r="I292" s="3" t="n"/>
       <c r="J292" s="3" t="n"/>
-      <c r="K292" s="5" t="n"/>
-      <c r="L292" s="5" t="n"/>
+      <c r="K292" s="3" t="n"/>
+      <c r="L292" s="3" t="n"/>
       <c r="M292" s="5" t="n"/>
       <c r="N292" s="5" t="n"/>
       <c r="O292" s="5" t="n"/>
@@ -8651,6 +9253,8 @@
       <c r="W292" s="5" t="n"/>
       <c r="X292" s="5" t="n"/>
       <c r="Y292" s="5" t="n"/>
+      <c r="Z292" s="5" t="n"/>
+      <c r="AA292" s="5" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="6" t="n"/>
@@ -8678,6 +9282,8 @@
       <c r="W293" s="6" t="n"/>
       <c r="X293" s="6" t="n"/>
       <c r="Y293" s="6" t="n"/>
+      <c r="Z293" s="6" t="n"/>
+      <c r="AA293" s="6" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="3" t="n"/>
@@ -8690,8 +9296,8 @@
       <c r="H294" s="3" t="n"/>
       <c r="I294" s="3" t="n"/>
       <c r="J294" s="3" t="n"/>
-      <c r="K294" s="5" t="n"/>
-      <c r="L294" s="5" t="n"/>
+      <c r="K294" s="3" t="n"/>
+      <c r="L294" s="3" t="n"/>
       <c r="M294" s="5" t="n"/>
       <c r="N294" s="5" t="n"/>
       <c r="O294" s="5" t="n"/>
@@ -8705,6 +9311,8 @@
       <c r="W294" s="5" t="n"/>
       <c r="X294" s="5" t="n"/>
       <c r="Y294" s="5" t="n"/>
+      <c r="Z294" s="5" t="n"/>
+      <c r="AA294" s="5" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="6" t="n"/>
@@ -8732,6 +9340,8 @@
       <c r="W295" s="6" t="n"/>
       <c r="X295" s="6" t="n"/>
       <c r="Y295" s="6" t="n"/>
+      <c r="Z295" s="6" t="n"/>
+      <c r="AA295" s="6" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="3" t="n"/>
@@ -8744,8 +9354,8 @@
       <c r="H296" s="3" t="n"/>
       <c r="I296" s="3" t="n"/>
       <c r="J296" s="3" t="n"/>
-      <c r="K296" s="5" t="n"/>
-      <c r="L296" s="5" t="n"/>
+      <c r="K296" s="3" t="n"/>
+      <c r="L296" s="3" t="n"/>
       <c r="M296" s="5" t="n"/>
       <c r="N296" s="5" t="n"/>
       <c r="O296" s="5" t="n"/>
@@ -8759,6 +9369,8 @@
       <c r="W296" s="5" t="n"/>
       <c r="X296" s="5" t="n"/>
       <c r="Y296" s="5" t="n"/>
+      <c r="Z296" s="5" t="n"/>
+      <c r="AA296" s="5" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="6" t="n"/>
@@ -8786,6 +9398,8 @@
       <c r="W297" s="6" t="n"/>
       <c r="X297" s="6" t="n"/>
       <c r="Y297" s="6" t="n"/>
+      <c r="Z297" s="6" t="n"/>
+      <c r="AA297" s="6" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="3" t="n"/>
@@ -8798,8 +9412,8 @@
       <c r="H298" s="3" t="n"/>
       <c r="I298" s="3" t="n"/>
       <c r="J298" s="3" t="n"/>
-      <c r="K298" s="5" t="n"/>
-      <c r="L298" s="5" t="n"/>
+      <c r="K298" s="3" t="n"/>
+      <c r="L298" s="3" t="n"/>
       <c r="M298" s="5" t="n"/>
       <c r="N298" s="5" t="n"/>
       <c r="O298" s="5" t="n"/>
@@ -8813,6 +9427,8 @@
       <c r="W298" s="5" t="n"/>
       <c r="X298" s="5" t="n"/>
       <c r="Y298" s="5" t="n"/>
+      <c r="Z298" s="5" t="n"/>
+      <c r="AA298" s="5" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="6" t="n"/>
@@ -8840,6 +9456,8 @@
       <c r="W299" s="6" t="n"/>
       <c r="X299" s="6" t="n"/>
       <c r="Y299" s="6" t="n"/>
+      <c r="Z299" s="6" t="n"/>
+      <c r="AA299" s="6" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="3" t="n"/>
@@ -8852,8 +9470,8 @@
       <c r="H300" s="3" t="n"/>
       <c r="I300" s="3" t="n"/>
       <c r="J300" s="3" t="n"/>
-      <c r="K300" s="5" t="n"/>
-      <c r="L300" s="5" t="n"/>
+      <c r="K300" s="3" t="n"/>
+      <c r="L300" s="3" t="n"/>
       <c r="M300" s="5" t="n"/>
       <c r="N300" s="5" t="n"/>
       <c r="O300" s="5" t="n"/>
@@ -8867,6 +9485,8 @@
       <c r="W300" s="5" t="n"/>
       <c r="X300" s="5" t="n"/>
       <c r="Y300" s="5" t="n"/>
+      <c r="Z300" s="5" t="n"/>
+      <c r="AA300" s="5" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="6" t="n"/>
@@ -8894,6 +9514,8 @@
       <c r="W301" s="6" t="n"/>
       <c r="X301" s="6" t="n"/>
       <c r="Y301" s="6" t="n"/>
+      <c r="Z301" s="6" t="n"/>
+      <c r="AA301" s="6" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="11">
@@ -8912,22 +9534,22 @@
     <dataValidation sqref="E2:E301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر اليوم" type="list">
       <formula1>"الأحد,الاثنين,الثلاثاء,الأربعاء,الخميس,الجمعة,السبت"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
+    <dataValidation sqref="O2:O301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
       <formula1>"مشرفاً ومقرراً,مشرفاً,مشرفاً مشاركاً,مناقشاً,مناقشاً خارجياً,مشرفةً ومقررةً,مناقِشةً"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
+    <dataValidation sqref="R2:R301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
       <formula1>"مشرفاً ومقرراً,مشرفاً,مشرفاً مشاركاً,مناقشاً,مناقشاً خارجياً,مشرفةً ومقررةً,مناقِشةً"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
+    <dataValidation sqref="U2:U301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
       <formula1>"مشرفاً ومقرراً,مشرفاً,مشرفاً مشاركاً,مناقشاً,مناقشاً خارجياً,مشرفةً ومقررةً,مناقِشةً"</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
+    <dataValidation sqref="X2:X301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
       <formula1>"مشرفاً ومقرراً,مشرفاً,مشرفاً مشاركاً,مناقشاً,مناقشاً خارجياً,مشرفةً ومقررةً,مناقِشةً"</formula1>
     </dataValidation>
-    <dataValidation sqref="Y2:Y301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
+    <dataValidation sqref="AA2:AA301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
       <formula1>"مشرفاً ومقرراً,مشرفاً,مشرفاً مشاركاً,مناقشاً,مناقشاً خارجياً,مشرفةً ومقررةً,مناقِشةً"</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر أو اكتب الصفة" type="list">
+    <dataValidation sqref="N2:N301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر أو اكتب الصفة" type="list">
       <formula1>"الأستاذ في قسم الفقه,الأستاذ المشارك في قسم الفقه,الأستاذ المساعد في قسم الفقه"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8993,7 +9615,7 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>6) رابط البث: الافتراضي قناة اليوتيوب (اختره من القائمة أو اتركه فاضي). تقدر تلصق رابط زوم أو بلاك بورد أو أي منصة. يظهر كرمز QR إذا فعّلته في الموقع.</t>
+          <t>6) رابط اللجنة (زوم) اختياري، ورابط التسجيل يُضاف بعد المناقشة. رابط البث: الافتراضي قناة اليوتيوب (اختره من القائمة أو اتركه فاضي). تقدر تلصق رابط زوم أو بلاك بورد أو أي منصة. يظهر كرمز QR إذا فعّلته في الموقع.</t>
         </is>
       </c>
     </row>
@@ -9111,63 +9733,63 @@
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>عضو1 الاسم:   أ.د. عمر بن علي السديس</t>
+          <t>رابط اللجنة:   أ.د. عمر بن علي السديس</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>عضو1 الصفة:   الأستاذ في قسم الفقه</t>
+          <t>رابط التسجيل:   الأستاذ في قسم الفقه</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>عضو1 الدور:   مشرفاً ومقرراً</t>
+          <t>عضو1 الاسم:   مشرفاً ومقرراً</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>عضو2 الاسم:   أ.د. فهد بن صالح الحمود</t>
+          <t>عضو1 الصفة:   أ.د. فهد بن صالح الحمود</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>عضو2 الصفة:   الأستاذ في قسم الفقه</t>
+          <t>عضو1 الدور:   الأستاذ في قسم الفقه</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>عضو2 الدور:   مناقشاً</t>
+          <t>عضو2 الاسم:   مناقشاً</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>عضو3 الاسم:   د. أحمد بن سليمان العودة</t>
+          <t>عضو2 الصفة:   د. أحمد بن سليمان العودة</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>عضو3 الصفة:   الأستاذ المساعد في قسم الفقه</t>
+          <t>عضو2 الدور:   الأستاذ المساعد في قسم الفقه</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>عضو3 الدور:   مناقشاً</t>
+          <t>عضو3 الاسم:   مناقشاً</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Notes and booking-coordinator columns, weekly break separators
- New grid columns الملاحظات and منسق الحجز (pick lists that learn;
  the coordinator a user last picked auto-fills new rows); grid data
  migrated to the new layout; booking import reads both columns
- Shared booking data regenerated with notes/coordinator; existing rows
  get only their blank cells filled
- Weekly break separators (Fri/Sat) between weeks, on by default and
  remembered per user, exported as rows and skipped on re-import
- Excel template gains the two columns

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqjysm6ZxBaYZPctG6chPQ
</commit_message>
<xml_diff>
--- a/assets/templates/template.xlsx
+++ b/assets/templates/template.xlsx
@@ -282,75 +282,85 @@
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
-        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+        <t>مثال: انتهت المناقشة / تم التأجيل</t>
       </text>
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: الأستاذ في قسم الفقه</t>
+        <t>اسم الموظف المنسق للحجز، مثال: محمد الحربي</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
+        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
       </text>
     </comment>
     <comment ref="P1" authorId="0" shapeId="0">
       <text>
-        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+        <t>مثال: الأستاذ في قسم الفقه</t>
       </text>
     </comment>
     <comment ref="Q1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: الأستاذ في قسم الفقه</t>
+        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
       </text>
     </comment>
     <comment ref="R1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
+        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
       </text>
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
       <text>
-        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+        <t>مثال: الأستاذ في قسم الفقه</t>
       </text>
     </comment>
     <comment ref="T1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: الأستاذ في قسم الفقه</t>
+        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
       </text>
     </comment>
     <comment ref="U1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
+        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
       </text>
     </comment>
     <comment ref="V1" authorId="0" shapeId="0">
       <text>
-        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+        <t>مثال: الأستاذ في قسم الفقه</t>
       </text>
     </comment>
     <comment ref="W1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: الأستاذ في قسم الفقه</t>
+        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
       </text>
     </comment>
     <comment ref="X1" authorId="0" shapeId="0">
       <text>
-        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
+        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
       </text>
     </comment>
     <comment ref="Y1" authorId="0" shapeId="0">
       <text>
-        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+        <t>مثال: الأستاذ في قسم الفقه</t>
       </text>
     </comment>
     <comment ref="Z1" authorId="0" shapeId="0">
       <text>
+        <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <t>اسم العضو مع اللقب، مثال: أ.د. عمر بن علي السديس</t>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="0" shapeId="0">
+      <text>
         <t>مثال: الأستاذ في قسم الفقه</t>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
+    <comment ref="AC1" authorId="0" shapeId="0">
       <text>
         <t>مثال: مشرفاً ومقرراً / مناقشاً</t>
       </text>
@@ -648,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA301"/>
+  <dimension ref="A1:AC301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -678,6 +688,8 @@
     <col width="24" customWidth="1" min="25" max="25"/>
     <col width="24" customWidth="1" min="26" max="26"/>
     <col width="24" customWidth="1" min="27" max="27"/>
+    <col width="24" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -741,77 +753,87 @@
           <t>رابط التسجيل</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>الملاحظات</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>منسق الحجز</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>عضو1 الاسم</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>عضو1 الصفة</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>عضو1 الدور</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>عضو2 الاسم</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>عضو2 الصفة</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>عضو2 الدور</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>عضو3 الاسم</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>عضو3 الصفة</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>عضو3 الدور</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>عضو4 الاسم</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>عضو4 الصفة</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>عضو4 الدور</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>عضو5 الاسم</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>عضو5 الصفة</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>عضو5 الدور</t>
         </is>
@@ -830,8 +852,8 @@
       <c r="J2" s="3" t="n"/>
       <c r="K2" s="3" t="n"/>
       <c r="L2" s="3" t="n"/>
-      <c r="M2" s="5" t="n"/>
-      <c r="N2" s="5" t="n"/>
+      <c r="M2" s="3" t="n"/>
+      <c r="N2" s="3" t="n"/>
       <c r="O2" s="5" t="n"/>
       <c r="P2" s="5" t="n"/>
       <c r="Q2" s="5" t="n"/>
@@ -845,6 +867,8 @@
       <c r="Y2" s="5" t="n"/>
       <c r="Z2" s="5" t="n"/>
       <c r="AA2" s="5" t="n"/>
+      <c r="AB2" s="5" t="n"/>
+      <c r="AC2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="n"/>
@@ -874,6 +898,8 @@
       <c r="Y3" s="6" t="n"/>
       <c r="Z3" s="6" t="n"/>
       <c r="AA3" s="6" t="n"/>
+      <c r="AB3" s="6" t="n"/>
+      <c r="AC3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -888,8 +914,8 @@
       <c r="J4" s="3" t="n"/>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="n"/>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="n"/>
+      <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="n"/>
       <c r="O4" s="5" t="n"/>
       <c r="P4" s="5" t="n"/>
       <c r="Q4" s="5" t="n"/>
@@ -903,6 +929,8 @@
       <c r="Y4" s="5" t="n"/>
       <c r="Z4" s="5" t="n"/>
       <c r="AA4" s="5" t="n"/>
+      <c r="AB4" s="5" t="n"/>
+      <c r="AC4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n"/>
@@ -932,6 +960,8 @@
       <c r="Y5" s="6" t="n"/>
       <c r="Z5" s="6" t="n"/>
       <c r="AA5" s="6" t="n"/>
+      <c r="AB5" s="6" t="n"/>
+      <c r="AC5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -946,8 +976,8 @@
       <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="n"/>
       <c r="L6" s="3" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
+      <c r="M6" s="3" t="n"/>
+      <c r="N6" s="3" t="n"/>
       <c r="O6" s="5" t="n"/>
       <c r="P6" s="5" t="n"/>
       <c r="Q6" s="5" t="n"/>
@@ -961,6 +991,8 @@
       <c r="Y6" s="5" t="n"/>
       <c r="Z6" s="5" t="n"/>
       <c r="AA6" s="5" t="n"/>
+      <c r="AB6" s="5" t="n"/>
+      <c r="AC6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n"/>
@@ -990,6 +1022,8 @@
       <c r="Y7" s="6" t="n"/>
       <c r="Z7" s="6" t="n"/>
       <c r="AA7" s="6" t="n"/>
+      <c r="AB7" s="6" t="n"/>
+      <c r="AC7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -1004,8 +1038,8 @@
       <c r="J8" s="3" t="n"/>
       <c r="K8" s="3" t="n"/>
       <c r="L8" s="3" t="n"/>
-      <c r="M8" s="5" t="n"/>
-      <c r="N8" s="5" t="n"/>
+      <c r="M8" s="3" t="n"/>
+      <c r="N8" s="3" t="n"/>
       <c r="O8" s="5" t="n"/>
       <c r="P8" s="5" t="n"/>
       <c r="Q8" s="5" t="n"/>
@@ -1019,6 +1053,8 @@
       <c r="Y8" s="5" t="n"/>
       <c r="Z8" s="5" t="n"/>
       <c r="AA8" s="5" t="n"/>
+      <c r="AB8" s="5" t="n"/>
+      <c r="AC8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
@@ -1048,6 +1084,8 @@
       <c r="Y9" s="6" t="n"/>
       <c r="Z9" s="6" t="n"/>
       <c r="AA9" s="6" t="n"/>
+      <c r="AB9" s="6" t="n"/>
+      <c r="AC9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -1062,8 +1100,8 @@
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="n"/>
       <c r="L10" s="3" t="n"/>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="5" t="n"/>
+      <c r="M10" s="3" t="n"/>
+      <c r="N10" s="3" t="n"/>
       <c r="O10" s="5" t="n"/>
       <c r="P10" s="5" t="n"/>
       <c r="Q10" s="5" t="n"/>
@@ -1077,6 +1115,8 @@
       <c r="Y10" s="5" t="n"/>
       <c r="Z10" s="5" t="n"/>
       <c r="AA10" s="5" t="n"/>
+      <c r="AB10" s="5" t="n"/>
+      <c r="AC10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
@@ -1106,6 +1146,8 @@
       <c r="Y11" s="6" t="n"/>
       <c r="Z11" s="6" t="n"/>
       <c r="AA11" s="6" t="n"/>
+      <c r="AB11" s="6" t="n"/>
+      <c r="AC11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -1120,8 +1162,8 @@
       <c r="J12" s="3" t="n"/>
       <c r="K12" s="3" t="n"/>
       <c r="L12" s="3" t="n"/>
-      <c r="M12" s="5" t="n"/>
-      <c r="N12" s="5" t="n"/>
+      <c r="M12" s="3" t="n"/>
+      <c r="N12" s="3" t="n"/>
       <c r="O12" s="5" t="n"/>
       <c r="P12" s="5" t="n"/>
       <c r="Q12" s="5" t="n"/>
@@ -1135,6 +1177,8 @@
       <c r="Y12" s="5" t="n"/>
       <c r="Z12" s="5" t="n"/>
       <c r="AA12" s="5" t="n"/>
+      <c r="AB12" s="5" t="n"/>
+      <c r="AC12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
@@ -1164,6 +1208,8 @@
       <c r="Y13" s="6" t="n"/>
       <c r="Z13" s="6" t="n"/>
       <c r="AA13" s="6" t="n"/>
+      <c r="AB13" s="6" t="n"/>
+      <c r="AC13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -1178,8 +1224,8 @@
       <c r="J14" s="3" t="n"/>
       <c r="K14" s="3" t="n"/>
       <c r="L14" s="3" t="n"/>
-      <c r="M14" s="5" t="n"/>
-      <c r="N14" s="5" t="n"/>
+      <c r="M14" s="3" t="n"/>
+      <c r="N14" s="3" t="n"/>
       <c r="O14" s="5" t="n"/>
       <c r="P14" s="5" t="n"/>
       <c r="Q14" s="5" t="n"/>
@@ -1193,6 +1239,8 @@
       <c r="Y14" s="5" t="n"/>
       <c r="Z14" s="5" t="n"/>
       <c r="AA14" s="5" t="n"/>
+      <c r="AB14" s="5" t="n"/>
+      <c r="AC14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
@@ -1222,6 +1270,8 @@
       <c r="Y15" s="6" t="n"/>
       <c r="Z15" s="6" t="n"/>
       <c r="AA15" s="6" t="n"/>
+      <c r="AB15" s="6" t="n"/>
+      <c r="AC15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -1236,8 +1286,8 @@
       <c r="J16" s="3" t="n"/>
       <c r="K16" s="3" t="n"/>
       <c r="L16" s="3" t="n"/>
-      <c r="M16" s="5" t="n"/>
-      <c r="N16" s="5" t="n"/>
+      <c r="M16" s="3" t="n"/>
+      <c r="N16" s="3" t="n"/>
       <c r="O16" s="5" t="n"/>
       <c r="P16" s="5" t="n"/>
       <c r="Q16" s="5" t="n"/>
@@ -1251,6 +1301,8 @@
       <c r="Y16" s="5" t="n"/>
       <c r="Z16" s="5" t="n"/>
       <c r="AA16" s="5" t="n"/>
+      <c r="AB16" s="5" t="n"/>
+      <c r="AC16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
@@ -1280,6 +1332,8 @@
       <c r="Y17" s="6" t="n"/>
       <c r="Z17" s="6" t="n"/>
       <c r="AA17" s="6" t="n"/>
+      <c r="AB17" s="6" t="n"/>
+      <c r="AC17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -1294,8 +1348,8 @@
       <c r="J18" s="3" t="n"/>
       <c r="K18" s="3" t="n"/>
       <c r="L18" s="3" t="n"/>
-      <c r="M18" s="5" t="n"/>
-      <c r="N18" s="5" t="n"/>
+      <c r="M18" s="3" t="n"/>
+      <c r="N18" s="3" t="n"/>
       <c r="O18" s="5" t="n"/>
       <c r="P18" s="5" t="n"/>
       <c r="Q18" s="5" t="n"/>
@@ -1309,6 +1363,8 @@
       <c r="Y18" s="5" t="n"/>
       <c r="Z18" s="5" t="n"/>
       <c r="AA18" s="5" t="n"/>
+      <c r="AB18" s="5" t="n"/>
+      <c r="AC18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
@@ -1338,6 +1394,8 @@
       <c r="Y19" s="6" t="n"/>
       <c r="Z19" s="6" t="n"/>
       <c r="AA19" s="6" t="n"/>
+      <c r="AB19" s="6" t="n"/>
+      <c r="AC19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -1352,8 +1410,8 @@
       <c r="J20" s="3" t="n"/>
       <c r="K20" s="3" t="n"/>
       <c r="L20" s="3" t="n"/>
-      <c r="M20" s="5" t="n"/>
-      <c r="N20" s="5" t="n"/>
+      <c r="M20" s="3" t="n"/>
+      <c r="N20" s="3" t="n"/>
       <c r="O20" s="5" t="n"/>
       <c r="P20" s="5" t="n"/>
       <c r="Q20" s="5" t="n"/>
@@ -1367,6 +1425,8 @@
       <c r="Y20" s="5" t="n"/>
       <c r="Z20" s="5" t="n"/>
       <c r="AA20" s="5" t="n"/>
+      <c r="AB20" s="5" t="n"/>
+      <c r="AC20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n"/>
@@ -1396,6 +1456,8 @@
       <c r="Y21" s="6" t="n"/>
       <c r="Z21" s="6" t="n"/>
       <c r="AA21" s="6" t="n"/>
+      <c r="AB21" s="6" t="n"/>
+      <c r="AC21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -1410,8 +1472,8 @@
       <c r="J22" s="3" t="n"/>
       <c r="K22" s="3" t="n"/>
       <c r="L22" s="3" t="n"/>
-      <c r="M22" s="5" t="n"/>
-      <c r="N22" s="5" t="n"/>
+      <c r="M22" s="3" t="n"/>
+      <c r="N22" s="3" t="n"/>
       <c r="O22" s="5" t="n"/>
       <c r="P22" s="5" t="n"/>
       <c r="Q22" s="5" t="n"/>
@@ -1425,6 +1487,8 @@
       <c r="Y22" s="5" t="n"/>
       <c r="Z22" s="5" t="n"/>
       <c r="AA22" s="5" t="n"/>
+      <c r="AB22" s="5" t="n"/>
+      <c r="AC22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
@@ -1454,6 +1518,8 @@
       <c r="Y23" s="6" t="n"/>
       <c r="Z23" s="6" t="n"/>
       <c r="AA23" s="6" t="n"/>
+      <c r="AB23" s="6" t="n"/>
+      <c r="AC23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -1468,8 +1534,8 @@
       <c r="J24" s="3" t="n"/>
       <c r="K24" s="3" t="n"/>
       <c r="L24" s="3" t="n"/>
-      <c r="M24" s="5" t="n"/>
-      <c r="N24" s="5" t="n"/>
+      <c r="M24" s="3" t="n"/>
+      <c r="N24" s="3" t="n"/>
       <c r="O24" s="5" t="n"/>
       <c r="P24" s="5" t="n"/>
       <c r="Q24" s="5" t="n"/>
@@ -1483,6 +1549,8 @@
       <c r="Y24" s="5" t="n"/>
       <c r="Z24" s="5" t="n"/>
       <c r="AA24" s="5" t="n"/>
+      <c r="AB24" s="5" t="n"/>
+      <c r="AC24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n"/>
@@ -1512,6 +1580,8 @@
       <c r="Y25" s="6" t="n"/>
       <c r="Z25" s="6" t="n"/>
       <c r="AA25" s="6" t="n"/>
+      <c r="AB25" s="6" t="n"/>
+      <c r="AC25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -1526,8 +1596,8 @@
       <c r="J26" s="3" t="n"/>
       <c r="K26" s="3" t="n"/>
       <c r="L26" s="3" t="n"/>
-      <c r="M26" s="5" t="n"/>
-      <c r="N26" s="5" t="n"/>
+      <c r="M26" s="3" t="n"/>
+      <c r="N26" s="3" t="n"/>
       <c r="O26" s="5" t="n"/>
       <c r="P26" s="5" t="n"/>
       <c r="Q26" s="5" t="n"/>
@@ -1541,6 +1611,8 @@
       <c r="Y26" s="5" t="n"/>
       <c r="Z26" s="5" t="n"/>
       <c r="AA26" s="5" t="n"/>
+      <c r="AB26" s="5" t="n"/>
+      <c r="AC26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n"/>
@@ -1570,6 +1642,8 @@
       <c r="Y27" s="6" t="n"/>
       <c r="Z27" s="6" t="n"/>
       <c r="AA27" s="6" t="n"/>
+      <c r="AB27" s="6" t="n"/>
+      <c r="AC27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -1584,8 +1658,8 @@
       <c r="J28" s="3" t="n"/>
       <c r="K28" s="3" t="n"/>
       <c r="L28" s="3" t="n"/>
-      <c r="M28" s="5" t="n"/>
-      <c r="N28" s="5" t="n"/>
+      <c r="M28" s="3" t="n"/>
+      <c r="N28" s="3" t="n"/>
       <c r="O28" s="5" t="n"/>
       <c r="P28" s="5" t="n"/>
       <c r="Q28" s="5" t="n"/>
@@ -1599,6 +1673,8 @@
       <c r="Y28" s="5" t="n"/>
       <c r="Z28" s="5" t="n"/>
       <c r="AA28" s="5" t="n"/>
+      <c r="AB28" s="5" t="n"/>
+      <c r="AC28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n"/>
@@ -1628,6 +1704,8 @@
       <c r="Y29" s="6" t="n"/>
       <c r="Z29" s="6" t="n"/>
       <c r="AA29" s="6" t="n"/>
+      <c r="AB29" s="6" t="n"/>
+      <c r="AC29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -1642,8 +1720,8 @@
       <c r="J30" s="3" t="n"/>
       <c r="K30" s="3" t="n"/>
       <c r="L30" s="3" t="n"/>
-      <c r="M30" s="5" t="n"/>
-      <c r="N30" s="5" t="n"/>
+      <c r="M30" s="3" t="n"/>
+      <c r="N30" s="3" t="n"/>
       <c r="O30" s="5" t="n"/>
       <c r="P30" s="5" t="n"/>
       <c r="Q30" s="5" t="n"/>
@@ -1657,6 +1735,8 @@
       <c r="Y30" s="5" t="n"/>
       <c r="Z30" s="5" t="n"/>
       <c r="AA30" s="5" t="n"/>
+      <c r="AB30" s="5" t="n"/>
+      <c r="AC30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n"/>
@@ -1686,6 +1766,8 @@
       <c r="Y31" s="6" t="n"/>
       <c r="Z31" s="6" t="n"/>
       <c r="AA31" s="6" t="n"/>
+      <c r="AB31" s="6" t="n"/>
+      <c r="AC31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -1700,8 +1782,8 @@
       <c r="J32" s="3" t="n"/>
       <c r="K32" s="3" t="n"/>
       <c r="L32" s="3" t="n"/>
-      <c r="M32" s="5" t="n"/>
-      <c r="N32" s="5" t="n"/>
+      <c r="M32" s="3" t="n"/>
+      <c r="N32" s="3" t="n"/>
       <c r="O32" s="5" t="n"/>
       <c r="P32" s="5" t="n"/>
       <c r="Q32" s="5" t="n"/>
@@ -1715,6 +1797,8 @@
       <c r="Y32" s="5" t="n"/>
       <c r="Z32" s="5" t="n"/>
       <c r="AA32" s="5" t="n"/>
+      <c r="AB32" s="5" t="n"/>
+      <c r="AC32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
@@ -1744,6 +1828,8 @@
       <c r="Y33" s="6" t="n"/>
       <c r="Z33" s="6" t="n"/>
       <c r="AA33" s="6" t="n"/>
+      <c r="AB33" s="6" t="n"/>
+      <c r="AC33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -1758,8 +1844,8 @@
       <c r="J34" s="3" t="n"/>
       <c r="K34" s="3" t="n"/>
       <c r="L34" s="3" t="n"/>
-      <c r="M34" s="5" t="n"/>
-      <c r="N34" s="5" t="n"/>
+      <c r="M34" s="3" t="n"/>
+      <c r="N34" s="3" t="n"/>
       <c r="O34" s="5" t="n"/>
       <c r="P34" s="5" t="n"/>
       <c r="Q34" s="5" t="n"/>
@@ -1773,6 +1859,8 @@
       <c r="Y34" s="5" t="n"/>
       <c r="Z34" s="5" t="n"/>
       <c r="AA34" s="5" t="n"/>
+      <c r="AB34" s="5" t="n"/>
+      <c r="AC34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
@@ -1802,6 +1890,8 @@
       <c r="Y35" s="6" t="n"/>
       <c r="Z35" s="6" t="n"/>
       <c r="AA35" s="6" t="n"/>
+      <c r="AB35" s="6" t="n"/>
+      <c r="AC35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -1816,8 +1906,8 @@
       <c r="J36" s="3" t="n"/>
       <c r="K36" s="3" t="n"/>
       <c r="L36" s="3" t="n"/>
-      <c r="M36" s="5" t="n"/>
-      <c r="N36" s="5" t="n"/>
+      <c r="M36" s="3" t="n"/>
+      <c r="N36" s="3" t="n"/>
       <c r="O36" s="5" t="n"/>
       <c r="P36" s="5" t="n"/>
       <c r="Q36" s="5" t="n"/>
@@ -1831,6 +1921,8 @@
       <c r="Y36" s="5" t="n"/>
       <c r="Z36" s="5" t="n"/>
       <c r="AA36" s="5" t="n"/>
+      <c r="AB36" s="5" t="n"/>
+      <c r="AC36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n"/>
@@ -1860,6 +1952,8 @@
       <c r="Y37" s="6" t="n"/>
       <c r="Z37" s="6" t="n"/>
       <c r="AA37" s="6" t="n"/>
+      <c r="AB37" s="6" t="n"/>
+      <c r="AC37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -1874,8 +1968,8 @@
       <c r="J38" s="3" t="n"/>
       <c r="K38" s="3" t="n"/>
       <c r="L38" s="3" t="n"/>
-      <c r="M38" s="5" t="n"/>
-      <c r="N38" s="5" t="n"/>
+      <c r="M38" s="3" t="n"/>
+      <c r="N38" s="3" t="n"/>
       <c r="O38" s="5" t="n"/>
       <c r="P38" s="5" t="n"/>
       <c r="Q38" s="5" t="n"/>
@@ -1889,6 +1983,8 @@
       <c r="Y38" s="5" t="n"/>
       <c r="Z38" s="5" t="n"/>
       <c r="AA38" s="5" t="n"/>
+      <c r="AB38" s="5" t="n"/>
+      <c r="AC38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
@@ -1918,6 +2014,8 @@
       <c r="Y39" s="6" t="n"/>
       <c r="Z39" s="6" t="n"/>
       <c r="AA39" s="6" t="n"/>
+      <c r="AB39" s="6" t="n"/>
+      <c r="AC39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -1932,8 +2030,8 @@
       <c r="J40" s="3" t="n"/>
       <c r="K40" s="3" t="n"/>
       <c r="L40" s="3" t="n"/>
-      <c r="M40" s="5" t="n"/>
-      <c r="N40" s="5" t="n"/>
+      <c r="M40" s="3" t="n"/>
+      <c r="N40" s="3" t="n"/>
       <c r="O40" s="5" t="n"/>
       <c r="P40" s="5" t="n"/>
       <c r="Q40" s="5" t="n"/>
@@ -1947,6 +2045,8 @@
       <c r="Y40" s="5" t="n"/>
       <c r="Z40" s="5" t="n"/>
       <c r="AA40" s="5" t="n"/>
+      <c r="AB40" s="5" t="n"/>
+      <c r="AC40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n"/>
@@ -1976,6 +2076,8 @@
       <c r="Y41" s="6" t="n"/>
       <c r="Z41" s="6" t="n"/>
       <c r="AA41" s="6" t="n"/>
+      <c r="AB41" s="6" t="n"/>
+      <c r="AC41" s="6" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -1990,8 +2092,8 @@
       <c r="J42" s="3" t="n"/>
       <c r="K42" s="3" t="n"/>
       <c r="L42" s="3" t="n"/>
-      <c r="M42" s="5" t="n"/>
-      <c r="N42" s="5" t="n"/>
+      <c r="M42" s="3" t="n"/>
+      <c r="N42" s="3" t="n"/>
       <c r="O42" s="5" t="n"/>
       <c r="P42" s="5" t="n"/>
       <c r="Q42" s="5" t="n"/>
@@ -2005,6 +2107,8 @@
       <c r="Y42" s="5" t="n"/>
       <c r="Z42" s="5" t="n"/>
       <c r="AA42" s="5" t="n"/>
+      <c r="AB42" s="5" t="n"/>
+      <c r="AC42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n"/>
@@ -2034,6 +2138,8 @@
       <c r="Y43" s="6" t="n"/>
       <c r="Z43" s="6" t="n"/>
       <c r="AA43" s="6" t="n"/>
+      <c r="AB43" s="6" t="n"/>
+      <c r="AC43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
@@ -2048,8 +2154,8 @@
       <c r="J44" s="3" t="n"/>
       <c r="K44" s="3" t="n"/>
       <c r="L44" s="3" t="n"/>
-      <c r="M44" s="5" t="n"/>
-      <c r="N44" s="5" t="n"/>
+      <c r="M44" s="3" t="n"/>
+      <c r="N44" s="3" t="n"/>
       <c r="O44" s="5" t="n"/>
       <c r="P44" s="5" t="n"/>
       <c r="Q44" s="5" t="n"/>
@@ -2063,6 +2169,8 @@
       <c r="Y44" s="5" t="n"/>
       <c r="Z44" s="5" t="n"/>
       <c r="AA44" s="5" t="n"/>
+      <c r="AB44" s="5" t="n"/>
+      <c r="AC44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n"/>
@@ -2092,6 +2200,8 @@
       <c r="Y45" s="6" t="n"/>
       <c r="Z45" s="6" t="n"/>
       <c r="AA45" s="6" t="n"/>
+      <c r="AB45" s="6" t="n"/>
+      <c r="AC45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
@@ -2106,8 +2216,8 @@
       <c r="J46" s="3" t="n"/>
       <c r="K46" s="3" t="n"/>
       <c r="L46" s="3" t="n"/>
-      <c r="M46" s="5" t="n"/>
-      <c r="N46" s="5" t="n"/>
+      <c r="M46" s="3" t="n"/>
+      <c r="N46" s="3" t="n"/>
       <c r="O46" s="5" t="n"/>
       <c r="P46" s="5" t="n"/>
       <c r="Q46" s="5" t="n"/>
@@ -2121,6 +2231,8 @@
       <c r="Y46" s="5" t="n"/>
       <c r="Z46" s="5" t="n"/>
       <c r="AA46" s="5" t="n"/>
+      <c r="AB46" s="5" t="n"/>
+      <c r="AC46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n"/>
@@ -2150,6 +2262,8 @@
       <c r="Y47" s="6" t="n"/>
       <c r="Z47" s="6" t="n"/>
       <c r="AA47" s="6" t="n"/>
+      <c r="AB47" s="6" t="n"/>
+      <c r="AC47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -2164,8 +2278,8 @@
       <c r="J48" s="3" t="n"/>
       <c r="K48" s="3" t="n"/>
       <c r="L48" s="3" t="n"/>
-      <c r="M48" s="5" t="n"/>
-      <c r="N48" s="5" t="n"/>
+      <c r="M48" s="3" t="n"/>
+      <c r="N48" s="3" t="n"/>
       <c r="O48" s="5" t="n"/>
       <c r="P48" s="5" t="n"/>
       <c r="Q48" s="5" t="n"/>
@@ -2179,6 +2293,8 @@
       <c r="Y48" s="5" t="n"/>
       <c r="Z48" s="5" t="n"/>
       <c r="AA48" s="5" t="n"/>
+      <c r="AB48" s="5" t="n"/>
+      <c r="AC48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n"/>
@@ -2208,6 +2324,8 @@
       <c r="Y49" s="6" t="n"/>
       <c r="Z49" s="6" t="n"/>
       <c r="AA49" s="6" t="n"/>
+      <c r="AB49" s="6" t="n"/>
+      <c r="AC49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
@@ -2222,8 +2340,8 @@
       <c r="J50" s="3" t="n"/>
       <c r="K50" s="3" t="n"/>
       <c r="L50" s="3" t="n"/>
-      <c r="M50" s="5" t="n"/>
-      <c r="N50" s="5" t="n"/>
+      <c r="M50" s="3" t="n"/>
+      <c r="N50" s="3" t="n"/>
       <c r="O50" s="5" t="n"/>
       <c r="P50" s="5" t="n"/>
       <c r="Q50" s="5" t="n"/>
@@ -2237,6 +2355,8 @@
       <c r="Y50" s="5" t="n"/>
       <c r="Z50" s="5" t="n"/>
       <c r="AA50" s="5" t="n"/>
+      <c r="AB50" s="5" t="n"/>
+      <c r="AC50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n"/>
@@ -2266,6 +2386,8 @@
       <c r="Y51" s="6" t="n"/>
       <c r="Z51" s="6" t="n"/>
       <c r="AA51" s="6" t="n"/>
+      <c r="AB51" s="6" t="n"/>
+      <c r="AC51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -2280,8 +2402,8 @@
       <c r="J52" s="3" t="n"/>
       <c r="K52" s="3" t="n"/>
       <c r="L52" s="3" t="n"/>
-      <c r="M52" s="5" t="n"/>
-      <c r="N52" s="5" t="n"/>
+      <c r="M52" s="3" t="n"/>
+      <c r="N52" s="3" t="n"/>
       <c r="O52" s="5" t="n"/>
       <c r="P52" s="5" t="n"/>
       <c r="Q52" s="5" t="n"/>
@@ -2295,6 +2417,8 @@
       <c r="Y52" s="5" t="n"/>
       <c r="Z52" s="5" t="n"/>
       <c r="AA52" s="5" t="n"/>
+      <c r="AB52" s="5" t="n"/>
+      <c r="AC52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n"/>
@@ -2324,6 +2448,8 @@
       <c r="Y53" s="6" t="n"/>
       <c r="Z53" s="6" t="n"/>
       <c r="AA53" s="6" t="n"/>
+      <c r="AB53" s="6" t="n"/>
+      <c r="AC53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
@@ -2338,8 +2464,8 @@
       <c r="J54" s="3" t="n"/>
       <c r="K54" s="3" t="n"/>
       <c r="L54" s="3" t="n"/>
-      <c r="M54" s="5" t="n"/>
-      <c r="N54" s="5" t="n"/>
+      <c r="M54" s="3" t="n"/>
+      <c r="N54" s="3" t="n"/>
       <c r="O54" s="5" t="n"/>
       <c r="P54" s="5" t="n"/>
       <c r="Q54" s="5" t="n"/>
@@ -2353,6 +2479,8 @@
       <c r="Y54" s="5" t="n"/>
       <c r="Z54" s="5" t="n"/>
       <c r="AA54" s="5" t="n"/>
+      <c r="AB54" s="5" t="n"/>
+      <c r="AC54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n"/>
@@ -2382,6 +2510,8 @@
       <c r="Y55" s="6" t="n"/>
       <c r="Z55" s="6" t="n"/>
       <c r="AA55" s="6" t="n"/>
+      <c r="AB55" s="6" t="n"/>
+      <c r="AC55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
@@ -2396,8 +2526,8 @@
       <c r="J56" s="3" t="n"/>
       <c r="K56" s="3" t="n"/>
       <c r="L56" s="3" t="n"/>
-      <c r="M56" s="5" t="n"/>
-      <c r="N56" s="5" t="n"/>
+      <c r="M56" s="3" t="n"/>
+      <c r="N56" s="3" t="n"/>
       <c r="O56" s="5" t="n"/>
       <c r="P56" s="5" t="n"/>
       <c r="Q56" s="5" t="n"/>
@@ -2411,6 +2541,8 @@
       <c r="Y56" s="5" t="n"/>
       <c r="Z56" s="5" t="n"/>
       <c r="AA56" s="5" t="n"/>
+      <c r="AB56" s="5" t="n"/>
+      <c r="AC56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="n"/>
@@ -2440,6 +2572,8 @@
       <c r="Y57" s="6" t="n"/>
       <c r="Z57" s="6" t="n"/>
       <c r="AA57" s="6" t="n"/>
+      <c r="AB57" s="6" t="n"/>
+      <c r="AC57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
@@ -2454,8 +2588,8 @@
       <c r="J58" s="3" t="n"/>
       <c r="K58" s="3" t="n"/>
       <c r="L58" s="3" t="n"/>
-      <c r="M58" s="5" t="n"/>
-      <c r="N58" s="5" t="n"/>
+      <c r="M58" s="3" t="n"/>
+      <c r="N58" s="3" t="n"/>
       <c r="O58" s="5" t="n"/>
       <c r="P58" s="5" t="n"/>
       <c r="Q58" s="5" t="n"/>
@@ -2469,6 +2603,8 @@
       <c r="Y58" s="5" t="n"/>
       <c r="Z58" s="5" t="n"/>
       <c r="AA58" s="5" t="n"/>
+      <c r="AB58" s="5" t="n"/>
+      <c r="AC58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="6" t="n"/>
@@ -2498,6 +2634,8 @@
       <c r="Y59" s="6" t="n"/>
       <c r="Z59" s="6" t="n"/>
       <c r="AA59" s="6" t="n"/>
+      <c r="AB59" s="6" t="n"/>
+      <c r="AC59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
@@ -2512,8 +2650,8 @@
       <c r="J60" s="3" t="n"/>
       <c r="K60" s="3" t="n"/>
       <c r="L60" s="3" t="n"/>
-      <c r="M60" s="5" t="n"/>
-      <c r="N60" s="5" t="n"/>
+      <c r="M60" s="3" t="n"/>
+      <c r="N60" s="3" t="n"/>
       <c r="O60" s="5" t="n"/>
       <c r="P60" s="5" t="n"/>
       <c r="Q60" s="5" t="n"/>
@@ -2527,6 +2665,8 @@
       <c r="Y60" s="5" t="n"/>
       <c r="Z60" s="5" t="n"/>
       <c r="AA60" s="5" t="n"/>
+      <c r="AB60" s="5" t="n"/>
+      <c r="AC60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="6" t="n"/>
@@ -2556,6 +2696,8 @@
       <c r="Y61" s="6" t="n"/>
       <c r="Z61" s="6" t="n"/>
       <c r="AA61" s="6" t="n"/>
+      <c r="AB61" s="6" t="n"/>
+      <c r="AC61" s="6" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
@@ -2570,8 +2712,8 @@
       <c r="J62" s="3" t="n"/>
       <c r="K62" s="3" t="n"/>
       <c r="L62" s="3" t="n"/>
-      <c r="M62" s="5" t="n"/>
-      <c r="N62" s="5" t="n"/>
+      <c r="M62" s="3" t="n"/>
+      <c r="N62" s="3" t="n"/>
       <c r="O62" s="5" t="n"/>
       <c r="P62" s="5" t="n"/>
       <c r="Q62" s="5" t="n"/>
@@ -2585,6 +2727,8 @@
       <c r="Y62" s="5" t="n"/>
       <c r="Z62" s="5" t="n"/>
       <c r="AA62" s="5" t="n"/>
+      <c r="AB62" s="5" t="n"/>
+      <c r="AC62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="6" t="n"/>
@@ -2614,6 +2758,8 @@
       <c r="Y63" s="6" t="n"/>
       <c r="Z63" s="6" t="n"/>
       <c r="AA63" s="6" t="n"/>
+      <c r="AB63" s="6" t="n"/>
+      <c r="AC63" s="6" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
@@ -2628,8 +2774,8 @@
       <c r="J64" s="3" t="n"/>
       <c r="K64" s="3" t="n"/>
       <c r="L64" s="3" t="n"/>
-      <c r="M64" s="5" t="n"/>
-      <c r="N64" s="5" t="n"/>
+      <c r="M64" s="3" t="n"/>
+      <c r="N64" s="3" t="n"/>
       <c r="O64" s="5" t="n"/>
       <c r="P64" s="5" t="n"/>
       <c r="Q64" s="5" t="n"/>
@@ -2643,6 +2789,8 @@
       <c r="Y64" s="5" t="n"/>
       <c r="Z64" s="5" t="n"/>
       <c r="AA64" s="5" t="n"/>
+      <c r="AB64" s="5" t="n"/>
+      <c r="AC64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="n"/>
@@ -2672,6 +2820,8 @@
       <c r="Y65" s="6" t="n"/>
       <c r="Z65" s="6" t="n"/>
       <c r="AA65" s="6" t="n"/>
+      <c r="AB65" s="6" t="n"/>
+      <c r="AC65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -2686,8 +2836,8 @@
       <c r="J66" s="3" t="n"/>
       <c r="K66" s="3" t="n"/>
       <c r="L66" s="3" t="n"/>
-      <c r="M66" s="5" t="n"/>
-      <c r="N66" s="5" t="n"/>
+      <c r="M66" s="3" t="n"/>
+      <c r="N66" s="3" t="n"/>
       <c r="O66" s="5" t="n"/>
       <c r="P66" s="5" t="n"/>
       <c r="Q66" s="5" t="n"/>
@@ -2701,6 +2851,8 @@
       <c r="Y66" s="5" t="n"/>
       <c r="Z66" s="5" t="n"/>
       <c r="AA66" s="5" t="n"/>
+      <c r="AB66" s="5" t="n"/>
+      <c r="AC66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="6" t="n"/>
@@ -2730,6 +2882,8 @@
       <c r="Y67" s="6" t="n"/>
       <c r="Z67" s="6" t="n"/>
       <c r="AA67" s="6" t="n"/>
+      <c r="AB67" s="6" t="n"/>
+      <c r="AC67" s="6" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
@@ -2744,8 +2898,8 @@
       <c r="J68" s="3" t="n"/>
       <c r="K68" s="3" t="n"/>
       <c r="L68" s="3" t="n"/>
-      <c r="M68" s="5" t="n"/>
-      <c r="N68" s="5" t="n"/>
+      <c r="M68" s="3" t="n"/>
+      <c r="N68" s="3" t="n"/>
       <c r="O68" s="5" t="n"/>
       <c r="P68" s="5" t="n"/>
       <c r="Q68" s="5" t="n"/>
@@ -2759,6 +2913,8 @@
       <c r="Y68" s="5" t="n"/>
       <c r="Z68" s="5" t="n"/>
       <c r="AA68" s="5" t="n"/>
+      <c r="AB68" s="5" t="n"/>
+      <c r="AC68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="n"/>
@@ -2788,6 +2944,8 @@
       <c r="Y69" s="6" t="n"/>
       <c r="Z69" s="6" t="n"/>
       <c r="AA69" s="6" t="n"/>
+      <c r="AB69" s="6" t="n"/>
+      <c r="AC69" s="6" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n"/>
@@ -2802,8 +2960,8 @@
       <c r="J70" s="3" t="n"/>
       <c r="K70" s="3" t="n"/>
       <c r="L70" s="3" t="n"/>
-      <c r="M70" s="5" t="n"/>
-      <c r="N70" s="5" t="n"/>
+      <c r="M70" s="3" t="n"/>
+      <c r="N70" s="3" t="n"/>
       <c r="O70" s="5" t="n"/>
       <c r="P70" s="5" t="n"/>
       <c r="Q70" s="5" t="n"/>
@@ -2817,6 +2975,8 @@
       <c r="Y70" s="5" t="n"/>
       <c r="Z70" s="5" t="n"/>
       <c r="AA70" s="5" t="n"/>
+      <c r="AB70" s="5" t="n"/>
+      <c r="AC70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n"/>
@@ -2846,6 +3006,8 @@
       <c r="Y71" s="6" t="n"/>
       <c r="Z71" s="6" t="n"/>
       <c r="AA71" s="6" t="n"/>
+      <c r="AB71" s="6" t="n"/>
+      <c r="AC71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n"/>
@@ -2860,8 +3022,8 @@
       <c r="J72" s="3" t="n"/>
       <c r="K72" s="3" t="n"/>
       <c r="L72" s="3" t="n"/>
-      <c r="M72" s="5" t="n"/>
-      <c r="N72" s="5" t="n"/>
+      <c r="M72" s="3" t="n"/>
+      <c r="N72" s="3" t="n"/>
       <c r="O72" s="5" t="n"/>
       <c r="P72" s="5" t="n"/>
       <c r="Q72" s="5" t="n"/>
@@ -2875,6 +3037,8 @@
       <c r="Y72" s="5" t="n"/>
       <c r="Z72" s="5" t="n"/>
       <c r="AA72" s="5" t="n"/>
+      <c r="AB72" s="5" t="n"/>
+      <c r="AC72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="n"/>
@@ -2904,6 +3068,8 @@
       <c r="Y73" s="6" t="n"/>
       <c r="Z73" s="6" t="n"/>
       <c r="AA73" s="6" t="n"/>
+      <c r="AB73" s="6" t="n"/>
+      <c r="AC73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n"/>
@@ -2918,8 +3084,8 @@
       <c r="J74" s="3" t="n"/>
       <c r="K74" s="3" t="n"/>
       <c r="L74" s="3" t="n"/>
-      <c r="M74" s="5" t="n"/>
-      <c r="N74" s="5" t="n"/>
+      <c r="M74" s="3" t="n"/>
+      <c r="N74" s="3" t="n"/>
       <c r="O74" s="5" t="n"/>
       <c r="P74" s="5" t="n"/>
       <c r="Q74" s="5" t="n"/>
@@ -2933,6 +3099,8 @@
       <c r="Y74" s="5" t="n"/>
       <c r="Z74" s="5" t="n"/>
       <c r="AA74" s="5" t="n"/>
+      <c r="AB74" s="5" t="n"/>
+      <c r="AC74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n"/>
@@ -2962,6 +3130,8 @@
       <c r="Y75" s="6" t="n"/>
       <c r="Z75" s="6" t="n"/>
       <c r="AA75" s="6" t="n"/>
+      <c r="AB75" s="6" t="n"/>
+      <c r="AC75" s="6" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n"/>
@@ -2976,8 +3146,8 @@
       <c r="J76" s="3" t="n"/>
       <c r="K76" s="3" t="n"/>
       <c r="L76" s="3" t="n"/>
-      <c r="M76" s="5" t="n"/>
-      <c r="N76" s="5" t="n"/>
+      <c r="M76" s="3" t="n"/>
+      <c r="N76" s="3" t="n"/>
       <c r="O76" s="5" t="n"/>
       <c r="P76" s="5" t="n"/>
       <c r="Q76" s="5" t="n"/>
@@ -2991,6 +3161,8 @@
       <c r="Y76" s="5" t="n"/>
       <c r="Z76" s="5" t="n"/>
       <c r="AA76" s="5" t="n"/>
+      <c r="AB76" s="5" t="n"/>
+      <c r="AC76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="6" t="n"/>
@@ -3020,6 +3192,8 @@
       <c r="Y77" s="6" t="n"/>
       <c r="Z77" s="6" t="n"/>
       <c r="AA77" s="6" t="n"/>
+      <c r="AB77" s="6" t="n"/>
+      <c r="AC77" s="6" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n"/>
@@ -3034,8 +3208,8 @@
       <c r="J78" s="3" t="n"/>
       <c r="K78" s="3" t="n"/>
       <c r="L78" s="3" t="n"/>
-      <c r="M78" s="5" t="n"/>
-      <c r="N78" s="5" t="n"/>
+      <c r="M78" s="3" t="n"/>
+      <c r="N78" s="3" t="n"/>
       <c r="O78" s="5" t="n"/>
       <c r="P78" s="5" t="n"/>
       <c r="Q78" s="5" t="n"/>
@@ -3049,6 +3223,8 @@
       <c r="Y78" s="5" t="n"/>
       <c r="Z78" s="5" t="n"/>
       <c r="AA78" s="5" t="n"/>
+      <c r="AB78" s="5" t="n"/>
+      <c r="AC78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="n"/>
@@ -3078,6 +3254,8 @@
       <c r="Y79" s="6" t="n"/>
       <c r="Z79" s="6" t="n"/>
       <c r="AA79" s="6" t="n"/>
+      <c r="AB79" s="6" t="n"/>
+      <c r="AC79" s="6" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n"/>
@@ -3092,8 +3270,8 @@
       <c r="J80" s="3" t="n"/>
       <c r="K80" s="3" t="n"/>
       <c r="L80" s="3" t="n"/>
-      <c r="M80" s="5" t="n"/>
-      <c r="N80" s="5" t="n"/>
+      <c r="M80" s="3" t="n"/>
+      <c r="N80" s="3" t="n"/>
       <c r="O80" s="5" t="n"/>
       <c r="P80" s="5" t="n"/>
       <c r="Q80" s="5" t="n"/>
@@ -3107,6 +3285,8 @@
       <c r="Y80" s="5" t="n"/>
       <c r="Z80" s="5" t="n"/>
       <c r="AA80" s="5" t="n"/>
+      <c r="AB80" s="5" t="n"/>
+      <c r="AC80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="n"/>
@@ -3136,6 +3316,8 @@
       <c r="Y81" s="6" t="n"/>
       <c r="Z81" s="6" t="n"/>
       <c r="AA81" s="6" t="n"/>
+      <c r="AB81" s="6" t="n"/>
+      <c r="AC81" s="6" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n"/>
@@ -3150,8 +3332,8 @@
       <c r="J82" s="3" t="n"/>
       <c r="K82" s="3" t="n"/>
       <c r="L82" s="3" t="n"/>
-      <c r="M82" s="5" t="n"/>
-      <c r="N82" s="5" t="n"/>
+      <c r="M82" s="3" t="n"/>
+      <c r="N82" s="3" t="n"/>
       <c r="O82" s="5" t="n"/>
       <c r="P82" s="5" t="n"/>
       <c r="Q82" s="5" t="n"/>
@@ -3165,6 +3347,8 @@
       <c r="Y82" s="5" t="n"/>
       <c r="Z82" s="5" t="n"/>
       <c r="AA82" s="5" t="n"/>
+      <c r="AB82" s="5" t="n"/>
+      <c r="AC82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="6" t="n"/>
@@ -3194,6 +3378,8 @@
       <c r="Y83" s="6" t="n"/>
       <c r="Z83" s="6" t="n"/>
       <c r="AA83" s="6" t="n"/>
+      <c r="AB83" s="6" t="n"/>
+      <c r="AC83" s="6" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n"/>
@@ -3208,8 +3394,8 @@
       <c r="J84" s="3" t="n"/>
       <c r="K84" s="3" t="n"/>
       <c r="L84" s="3" t="n"/>
-      <c r="M84" s="5" t="n"/>
-      <c r="N84" s="5" t="n"/>
+      <c r="M84" s="3" t="n"/>
+      <c r="N84" s="3" t="n"/>
       <c r="O84" s="5" t="n"/>
       <c r="P84" s="5" t="n"/>
       <c r="Q84" s="5" t="n"/>
@@ -3223,6 +3409,8 @@
       <c r="Y84" s="5" t="n"/>
       <c r="Z84" s="5" t="n"/>
       <c r="AA84" s="5" t="n"/>
+      <c r="AB84" s="5" t="n"/>
+      <c r="AC84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="n"/>
@@ -3252,6 +3440,8 @@
       <c r="Y85" s="6" t="n"/>
       <c r="Z85" s="6" t="n"/>
       <c r="AA85" s="6" t="n"/>
+      <c r="AB85" s="6" t="n"/>
+      <c r="AC85" s="6" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n"/>
@@ -3266,8 +3456,8 @@
       <c r="J86" s="3" t="n"/>
       <c r="K86" s="3" t="n"/>
       <c r="L86" s="3" t="n"/>
-      <c r="M86" s="5" t="n"/>
-      <c r="N86" s="5" t="n"/>
+      <c r="M86" s="3" t="n"/>
+      <c r="N86" s="3" t="n"/>
       <c r="O86" s="5" t="n"/>
       <c r="P86" s="5" t="n"/>
       <c r="Q86" s="5" t="n"/>
@@ -3281,6 +3471,8 @@
       <c r="Y86" s="5" t="n"/>
       <c r="Z86" s="5" t="n"/>
       <c r="AA86" s="5" t="n"/>
+      <c r="AB86" s="5" t="n"/>
+      <c r="AC86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="6" t="n"/>
@@ -3310,6 +3502,8 @@
       <c r="Y87" s="6" t="n"/>
       <c r="Z87" s="6" t="n"/>
       <c r="AA87" s="6" t="n"/>
+      <c r="AB87" s="6" t="n"/>
+      <c r="AC87" s="6" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n"/>
@@ -3324,8 +3518,8 @@
       <c r="J88" s="3" t="n"/>
       <c r="K88" s="3" t="n"/>
       <c r="L88" s="3" t="n"/>
-      <c r="M88" s="5" t="n"/>
-      <c r="N88" s="5" t="n"/>
+      <c r="M88" s="3" t="n"/>
+      <c r="N88" s="3" t="n"/>
       <c r="O88" s="5" t="n"/>
       <c r="P88" s="5" t="n"/>
       <c r="Q88" s="5" t="n"/>
@@ -3339,6 +3533,8 @@
       <c r="Y88" s="5" t="n"/>
       <c r="Z88" s="5" t="n"/>
       <c r="AA88" s="5" t="n"/>
+      <c r="AB88" s="5" t="n"/>
+      <c r="AC88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="n"/>
@@ -3368,6 +3564,8 @@
       <c r="Y89" s="6" t="n"/>
       <c r="Z89" s="6" t="n"/>
       <c r="AA89" s="6" t="n"/>
+      <c r="AB89" s="6" t="n"/>
+      <c r="AC89" s="6" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n"/>
@@ -3382,8 +3580,8 @@
       <c r="J90" s="3" t="n"/>
       <c r="K90" s="3" t="n"/>
       <c r="L90" s="3" t="n"/>
-      <c r="M90" s="5" t="n"/>
-      <c r="N90" s="5" t="n"/>
+      <c r="M90" s="3" t="n"/>
+      <c r="N90" s="3" t="n"/>
       <c r="O90" s="5" t="n"/>
       <c r="P90" s="5" t="n"/>
       <c r="Q90" s="5" t="n"/>
@@ -3397,6 +3595,8 @@
       <c r="Y90" s="5" t="n"/>
       <c r="Z90" s="5" t="n"/>
       <c r="AA90" s="5" t="n"/>
+      <c r="AB90" s="5" t="n"/>
+      <c r="AC90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="6" t="n"/>
@@ -3426,6 +3626,8 @@
       <c r="Y91" s="6" t="n"/>
       <c r="Z91" s="6" t="n"/>
       <c r="AA91" s="6" t="n"/>
+      <c r="AB91" s="6" t="n"/>
+      <c r="AC91" s="6" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n"/>
@@ -3440,8 +3642,8 @@
       <c r="J92" s="3" t="n"/>
       <c r="K92" s="3" t="n"/>
       <c r="L92" s="3" t="n"/>
-      <c r="M92" s="5" t="n"/>
-      <c r="N92" s="5" t="n"/>
+      <c r="M92" s="3" t="n"/>
+      <c r="N92" s="3" t="n"/>
       <c r="O92" s="5" t="n"/>
       <c r="P92" s="5" t="n"/>
       <c r="Q92" s="5" t="n"/>
@@ -3455,6 +3657,8 @@
       <c r="Y92" s="5" t="n"/>
       <c r="Z92" s="5" t="n"/>
       <c r="AA92" s="5" t="n"/>
+      <c r="AB92" s="5" t="n"/>
+      <c r="AC92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="6" t="n"/>
@@ -3484,6 +3688,8 @@
       <c r="Y93" s="6" t="n"/>
       <c r="Z93" s="6" t="n"/>
       <c r="AA93" s="6" t="n"/>
+      <c r="AB93" s="6" t="n"/>
+      <c r="AC93" s="6" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n"/>
@@ -3498,8 +3704,8 @@
       <c r="J94" s="3" t="n"/>
       <c r="K94" s="3" t="n"/>
       <c r="L94" s="3" t="n"/>
-      <c r="M94" s="5" t="n"/>
-      <c r="N94" s="5" t="n"/>
+      <c r="M94" s="3" t="n"/>
+      <c r="N94" s="3" t="n"/>
       <c r="O94" s="5" t="n"/>
       <c r="P94" s="5" t="n"/>
       <c r="Q94" s="5" t="n"/>
@@ -3513,6 +3719,8 @@
       <c r="Y94" s="5" t="n"/>
       <c r="Z94" s="5" t="n"/>
       <c r="AA94" s="5" t="n"/>
+      <c r="AB94" s="5" t="n"/>
+      <c r="AC94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="6" t="n"/>
@@ -3542,6 +3750,8 @@
       <c r="Y95" s="6" t="n"/>
       <c r="Z95" s="6" t="n"/>
       <c r="AA95" s="6" t="n"/>
+      <c r="AB95" s="6" t="n"/>
+      <c r="AC95" s="6" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n"/>
@@ -3556,8 +3766,8 @@
       <c r="J96" s="3" t="n"/>
       <c r="K96" s="3" t="n"/>
       <c r="L96" s="3" t="n"/>
-      <c r="M96" s="5" t="n"/>
-      <c r="N96" s="5" t="n"/>
+      <c r="M96" s="3" t="n"/>
+      <c r="N96" s="3" t="n"/>
       <c r="O96" s="5" t="n"/>
       <c r="P96" s="5" t="n"/>
       <c r="Q96" s="5" t="n"/>
@@ -3571,6 +3781,8 @@
       <c r="Y96" s="5" t="n"/>
       <c r="Z96" s="5" t="n"/>
       <c r="AA96" s="5" t="n"/>
+      <c r="AB96" s="5" t="n"/>
+      <c r="AC96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="6" t="n"/>
@@ -3600,6 +3812,8 @@
       <c r="Y97" s="6" t="n"/>
       <c r="Z97" s="6" t="n"/>
       <c r="AA97" s="6" t="n"/>
+      <c r="AB97" s="6" t="n"/>
+      <c r="AC97" s="6" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n"/>
@@ -3614,8 +3828,8 @@
       <c r="J98" s="3" t="n"/>
       <c r="K98" s="3" t="n"/>
       <c r="L98" s="3" t="n"/>
-      <c r="M98" s="5" t="n"/>
-      <c r="N98" s="5" t="n"/>
+      <c r="M98" s="3" t="n"/>
+      <c r="N98" s="3" t="n"/>
       <c r="O98" s="5" t="n"/>
       <c r="P98" s="5" t="n"/>
       <c r="Q98" s="5" t="n"/>
@@ -3629,6 +3843,8 @@
       <c r="Y98" s="5" t="n"/>
       <c r="Z98" s="5" t="n"/>
       <c r="AA98" s="5" t="n"/>
+      <c r="AB98" s="5" t="n"/>
+      <c r="AC98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="6" t="n"/>
@@ -3658,6 +3874,8 @@
       <c r="Y99" s="6" t="n"/>
       <c r="Z99" s="6" t="n"/>
       <c r="AA99" s="6" t="n"/>
+      <c r="AB99" s="6" t="n"/>
+      <c r="AC99" s="6" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n"/>
@@ -3672,8 +3890,8 @@
       <c r="J100" s="3" t="n"/>
       <c r="K100" s="3" t="n"/>
       <c r="L100" s="3" t="n"/>
-      <c r="M100" s="5" t="n"/>
-      <c r="N100" s="5" t="n"/>
+      <c r="M100" s="3" t="n"/>
+      <c r="N100" s="3" t="n"/>
       <c r="O100" s="5" t="n"/>
       <c r="P100" s="5" t="n"/>
       <c r="Q100" s="5" t="n"/>
@@ -3687,6 +3905,8 @@
       <c r="Y100" s="5" t="n"/>
       <c r="Z100" s="5" t="n"/>
       <c r="AA100" s="5" t="n"/>
+      <c r="AB100" s="5" t="n"/>
+      <c r="AC100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="6" t="n"/>
@@ -3716,6 +3936,8 @@
       <c r="Y101" s="6" t="n"/>
       <c r="Z101" s="6" t="n"/>
       <c r="AA101" s="6" t="n"/>
+      <c r="AB101" s="6" t="n"/>
+      <c r="AC101" s="6" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n"/>
@@ -3730,8 +3952,8 @@
       <c r="J102" s="3" t="n"/>
       <c r="K102" s="3" t="n"/>
       <c r="L102" s="3" t="n"/>
-      <c r="M102" s="5" t="n"/>
-      <c r="N102" s="5" t="n"/>
+      <c r="M102" s="3" t="n"/>
+      <c r="N102" s="3" t="n"/>
       <c r="O102" s="5" t="n"/>
       <c r="P102" s="5" t="n"/>
       <c r="Q102" s="5" t="n"/>
@@ -3745,6 +3967,8 @@
       <c r="Y102" s="5" t="n"/>
       <c r="Z102" s="5" t="n"/>
       <c r="AA102" s="5" t="n"/>
+      <c r="AB102" s="5" t="n"/>
+      <c r="AC102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="6" t="n"/>
@@ -3774,6 +3998,8 @@
       <c r="Y103" s="6" t="n"/>
       <c r="Z103" s="6" t="n"/>
       <c r="AA103" s="6" t="n"/>
+      <c r="AB103" s="6" t="n"/>
+      <c r="AC103" s="6" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n"/>
@@ -3788,8 +4014,8 @@
       <c r="J104" s="3" t="n"/>
       <c r="K104" s="3" t="n"/>
       <c r="L104" s="3" t="n"/>
-      <c r="M104" s="5" t="n"/>
-      <c r="N104" s="5" t="n"/>
+      <c r="M104" s="3" t="n"/>
+      <c r="N104" s="3" t="n"/>
       <c r="O104" s="5" t="n"/>
       <c r="P104" s="5" t="n"/>
       <c r="Q104" s="5" t="n"/>
@@ -3803,6 +4029,8 @@
       <c r="Y104" s="5" t="n"/>
       <c r="Z104" s="5" t="n"/>
       <c r="AA104" s="5" t="n"/>
+      <c r="AB104" s="5" t="n"/>
+      <c r="AC104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="6" t="n"/>
@@ -3832,6 +4060,8 @@
       <c r="Y105" s="6" t="n"/>
       <c r="Z105" s="6" t="n"/>
       <c r="AA105" s="6" t="n"/>
+      <c r="AB105" s="6" t="n"/>
+      <c r="AC105" s="6" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n"/>
@@ -3846,8 +4076,8 @@
       <c r="J106" s="3" t="n"/>
       <c r="K106" s="3" t="n"/>
       <c r="L106" s="3" t="n"/>
-      <c r="M106" s="5" t="n"/>
-      <c r="N106" s="5" t="n"/>
+      <c r="M106" s="3" t="n"/>
+      <c r="N106" s="3" t="n"/>
       <c r="O106" s="5" t="n"/>
       <c r="P106" s="5" t="n"/>
       <c r="Q106" s="5" t="n"/>
@@ -3861,6 +4091,8 @@
       <c r="Y106" s="5" t="n"/>
       <c r="Z106" s="5" t="n"/>
       <c r="AA106" s="5" t="n"/>
+      <c r="AB106" s="5" t="n"/>
+      <c r="AC106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="6" t="n"/>
@@ -3890,6 +4122,8 @@
       <c r="Y107" s="6" t="n"/>
       <c r="Z107" s="6" t="n"/>
       <c r="AA107" s="6" t="n"/>
+      <c r="AB107" s="6" t="n"/>
+      <c r="AC107" s="6" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n"/>
@@ -3904,8 +4138,8 @@
       <c r="J108" s="3" t="n"/>
       <c r="K108" s="3" t="n"/>
       <c r="L108" s="3" t="n"/>
-      <c r="M108" s="5" t="n"/>
-      <c r="N108" s="5" t="n"/>
+      <c r="M108" s="3" t="n"/>
+      <c r="N108" s="3" t="n"/>
       <c r="O108" s="5" t="n"/>
       <c r="P108" s="5" t="n"/>
       <c r="Q108" s="5" t="n"/>
@@ -3919,6 +4153,8 @@
       <c r="Y108" s="5" t="n"/>
       <c r="Z108" s="5" t="n"/>
       <c r="AA108" s="5" t="n"/>
+      <c r="AB108" s="5" t="n"/>
+      <c r="AC108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="6" t="n"/>
@@ -3948,6 +4184,8 @@
       <c r="Y109" s="6" t="n"/>
       <c r="Z109" s="6" t="n"/>
       <c r="AA109" s="6" t="n"/>
+      <c r="AB109" s="6" t="n"/>
+      <c r="AC109" s="6" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="3" t="n"/>
@@ -3962,8 +4200,8 @@
       <c r="J110" s="3" t="n"/>
       <c r="K110" s="3" t="n"/>
       <c r="L110" s="3" t="n"/>
-      <c r="M110" s="5" t="n"/>
-      <c r="N110" s="5" t="n"/>
+      <c r="M110" s="3" t="n"/>
+      <c r="N110" s="3" t="n"/>
       <c r="O110" s="5" t="n"/>
       <c r="P110" s="5" t="n"/>
       <c r="Q110" s="5" t="n"/>
@@ -3977,6 +4215,8 @@
       <c r="Y110" s="5" t="n"/>
       <c r="Z110" s="5" t="n"/>
       <c r="AA110" s="5" t="n"/>
+      <c r="AB110" s="5" t="n"/>
+      <c r="AC110" s="5" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="6" t="n"/>
@@ -4006,6 +4246,8 @@
       <c r="Y111" s="6" t="n"/>
       <c r="Z111" s="6" t="n"/>
       <c r="AA111" s="6" t="n"/>
+      <c r="AB111" s="6" t="n"/>
+      <c r="AC111" s="6" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="3" t="n"/>
@@ -4020,8 +4262,8 @@
       <c r="J112" s="3" t="n"/>
       <c r="K112" s="3" t="n"/>
       <c r="L112" s="3" t="n"/>
-      <c r="M112" s="5" t="n"/>
-      <c r="N112" s="5" t="n"/>
+      <c r="M112" s="3" t="n"/>
+      <c r="N112" s="3" t="n"/>
       <c r="O112" s="5" t="n"/>
       <c r="P112" s="5" t="n"/>
       <c r="Q112" s="5" t="n"/>
@@ -4035,6 +4277,8 @@
       <c r="Y112" s="5" t="n"/>
       <c r="Z112" s="5" t="n"/>
       <c r="AA112" s="5" t="n"/>
+      <c r="AB112" s="5" t="n"/>
+      <c r="AC112" s="5" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="6" t="n"/>
@@ -4064,6 +4308,8 @@
       <c r="Y113" s="6" t="n"/>
       <c r="Z113" s="6" t="n"/>
       <c r="AA113" s="6" t="n"/>
+      <c r="AB113" s="6" t="n"/>
+      <c r="AC113" s="6" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="n"/>
@@ -4078,8 +4324,8 @@
       <c r="J114" s="3" t="n"/>
       <c r="K114" s="3" t="n"/>
       <c r="L114" s="3" t="n"/>
-      <c r="M114" s="5" t="n"/>
-      <c r="N114" s="5" t="n"/>
+      <c r="M114" s="3" t="n"/>
+      <c r="N114" s="3" t="n"/>
       <c r="O114" s="5" t="n"/>
       <c r="P114" s="5" t="n"/>
       <c r="Q114" s="5" t="n"/>
@@ -4093,6 +4339,8 @@
       <c r="Y114" s="5" t="n"/>
       <c r="Z114" s="5" t="n"/>
       <c r="AA114" s="5" t="n"/>
+      <c r="AB114" s="5" t="n"/>
+      <c r="AC114" s="5" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="6" t="n"/>
@@ -4122,6 +4370,8 @@
       <c r="Y115" s="6" t="n"/>
       <c r="Z115" s="6" t="n"/>
       <c r="AA115" s="6" t="n"/>
+      <c r="AB115" s="6" t="n"/>
+      <c r="AC115" s="6" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="3" t="n"/>
@@ -4136,8 +4386,8 @@
       <c r="J116" s="3" t="n"/>
       <c r="K116" s="3" t="n"/>
       <c r="L116" s="3" t="n"/>
-      <c r="M116" s="5" t="n"/>
-      <c r="N116" s="5" t="n"/>
+      <c r="M116" s="3" t="n"/>
+      <c r="N116" s="3" t="n"/>
       <c r="O116" s="5" t="n"/>
       <c r="P116" s="5" t="n"/>
       <c r="Q116" s="5" t="n"/>
@@ -4151,6 +4401,8 @@
       <c r="Y116" s="5" t="n"/>
       <c r="Z116" s="5" t="n"/>
       <c r="AA116" s="5" t="n"/>
+      <c r="AB116" s="5" t="n"/>
+      <c r="AC116" s="5" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="6" t="n"/>
@@ -4180,6 +4432,8 @@
       <c r="Y117" s="6" t="n"/>
       <c r="Z117" s="6" t="n"/>
       <c r="AA117" s="6" t="n"/>
+      <c r="AB117" s="6" t="n"/>
+      <c r="AC117" s="6" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="3" t="n"/>
@@ -4194,8 +4448,8 @@
       <c r="J118" s="3" t="n"/>
       <c r="K118" s="3" t="n"/>
       <c r="L118" s="3" t="n"/>
-      <c r="M118" s="5" t="n"/>
-      <c r="N118" s="5" t="n"/>
+      <c r="M118" s="3" t="n"/>
+      <c r="N118" s="3" t="n"/>
       <c r="O118" s="5" t="n"/>
       <c r="P118" s="5" t="n"/>
       <c r="Q118" s="5" t="n"/>
@@ -4209,6 +4463,8 @@
       <c r="Y118" s="5" t="n"/>
       <c r="Z118" s="5" t="n"/>
       <c r="AA118" s="5" t="n"/>
+      <c r="AB118" s="5" t="n"/>
+      <c r="AC118" s="5" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="6" t="n"/>
@@ -4238,6 +4494,8 @@
       <c r="Y119" s="6" t="n"/>
       <c r="Z119" s="6" t="n"/>
       <c r="AA119" s="6" t="n"/>
+      <c r="AB119" s="6" t="n"/>
+      <c r="AC119" s="6" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="3" t="n"/>
@@ -4252,8 +4510,8 @@
       <c r="J120" s="3" t="n"/>
       <c r="K120" s="3" t="n"/>
       <c r="L120" s="3" t="n"/>
-      <c r="M120" s="5" t="n"/>
-      <c r="N120" s="5" t="n"/>
+      <c r="M120" s="3" t="n"/>
+      <c r="N120" s="3" t="n"/>
       <c r="O120" s="5" t="n"/>
       <c r="P120" s="5" t="n"/>
       <c r="Q120" s="5" t="n"/>
@@ -4267,6 +4525,8 @@
       <c r="Y120" s="5" t="n"/>
       <c r="Z120" s="5" t="n"/>
       <c r="AA120" s="5" t="n"/>
+      <c r="AB120" s="5" t="n"/>
+      <c r="AC120" s="5" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="6" t="n"/>
@@ -4296,6 +4556,8 @@
       <c r="Y121" s="6" t="n"/>
       <c r="Z121" s="6" t="n"/>
       <c r="AA121" s="6" t="n"/>
+      <c r="AB121" s="6" t="n"/>
+      <c r="AC121" s="6" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="3" t="n"/>
@@ -4310,8 +4572,8 @@
       <c r="J122" s="3" t="n"/>
       <c r="K122" s="3" t="n"/>
       <c r="L122" s="3" t="n"/>
-      <c r="M122" s="5" t="n"/>
-      <c r="N122" s="5" t="n"/>
+      <c r="M122" s="3" t="n"/>
+      <c r="N122" s="3" t="n"/>
       <c r="O122" s="5" t="n"/>
       <c r="P122" s="5" t="n"/>
       <c r="Q122" s="5" t="n"/>
@@ -4325,6 +4587,8 @@
       <c r="Y122" s="5" t="n"/>
       <c r="Z122" s="5" t="n"/>
       <c r="AA122" s="5" t="n"/>
+      <c r="AB122" s="5" t="n"/>
+      <c r="AC122" s="5" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="6" t="n"/>
@@ -4354,6 +4618,8 @@
       <c r="Y123" s="6" t="n"/>
       <c r="Z123" s="6" t="n"/>
       <c r="AA123" s="6" t="n"/>
+      <c r="AB123" s="6" t="n"/>
+      <c r="AC123" s="6" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="3" t="n"/>
@@ -4368,8 +4634,8 @@
       <c r="J124" s="3" t="n"/>
       <c r="K124" s="3" t="n"/>
       <c r="L124" s="3" t="n"/>
-      <c r="M124" s="5" t="n"/>
-      <c r="N124" s="5" t="n"/>
+      <c r="M124" s="3" t="n"/>
+      <c r="N124" s="3" t="n"/>
       <c r="O124" s="5" t="n"/>
       <c r="P124" s="5" t="n"/>
       <c r="Q124" s="5" t="n"/>
@@ -4383,6 +4649,8 @@
       <c r="Y124" s="5" t="n"/>
       <c r="Z124" s="5" t="n"/>
       <c r="AA124" s="5" t="n"/>
+      <c r="AB124" s="5" t="n"/>
+      <c r="AC124" s="5" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="6" t="n"/>
@@ -4412,6 +4680,8 @@
       <c r="Y125" s="6" t="n"/>
       <c r="Z125" s="6" t="n"/>
       <c r="AA125" s="6" t="n"/>
+      <c r="AB125" s="6" t="n"/>
+      <c r="AC125" s="6" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="3" t="n"/>
@@ -4426,8 +4696,8 @@
       <c r="J126" s="3" t="n"/>
       <c r="K126" s="3" t="n"/>
       <c r="L126" s="3" t="n"/>
-      <c r="M126" s="5" t="n"/>
-      <c r="N126" s="5" t="n"/>
+      <c r="M126" s="3" t="n"/>
+      <c r="N126" s="3" t="n"/>
       <c r="O126" s="5" t="n"/>
       <c r="P126" s="5" t="n"/>
       <c r="Q126" s="5" t="n"/>
@@ -4441,6 +4711,8 @@
       <c r="Y126" s="5" t="n"/>
       <c r="Z126" s="5" t="n"/>
       <c r="AA126" s="5" t="n"/>
+      <c r="AB126" s="5" t="n"/>
+      <c r="AC126" s="5" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="6" t="n"/>
@@ -4470,6 +4742,8 @@
       <c r="Y127" s="6" t="n"/>
       <c r="Z127" s="6" t="n"/>
       <c r="AA127" s="6" t="n"/>
+      <c r="AB127" s="6" t="n"/>
+      <c r="AC127" s="6" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="3" t="n"/>
@@ -4484,8 +4758,8 @@
       <c r="J128" s="3" t="n"/>
       <c r="K128" s="3" t="n"/>
       <c r="L128" s="3" t="n"/>
-      <c r="M128" s="5" t="n"/>
-      <c r="N128" s="5" t="n"/>
+      <c r="M128" s="3" t="n"/>
+      <c r="N128" s="3" t="n"/>
       <c r="O128" s="5" t="n"/>
       <c r="P128" s="5" t="n"/>
       <c r="Q128" s="5" t="n"/>
@@ -4499,6 +4773,8 @@
       <c r="Y128" s="5" t="n"/>
       <c r="Z128" s="5" t="n"/>
       <c r="AA128" s="5" t="n"/>
+      <c r="AB128" s="5" t="n"/>
+      <c r="AC128" s="5" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="6" t="n"/>
@@ -4528,6 +4804,8 @@
       <c r="Y129" s="6" t="n"/>
       <c r="Z129" s="6" t="n"/>
       <c r="AA129" s="6" t="n"/>
+      <c r="AB129" s="6" t="n"/>
+      <c r="AC129" s="6" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="3" t="n"/>
@@ -4542,8 +4820,8 @@
       <c r="J130" s="3" t="n"/>
       <c r="K130" s="3" t="n"/>
       <c r="L130" s="3" t="n"/>
-      <c r="M130" s="5" t="n"/>
-      <c r="N130" s="5" t="n"/>
+      <c r="M130" s="3" t="n"/>
+      <c r="N130" s="3" t="n"/>
       <c r="O130" s="5" t="n"/>
       <c r="P130" s="5" t="n"/>
       <c r="Q130" s="5" t="n"/>
@@ -4557,6 +4835,8 @@
       <c r="Y130" s="5" t="n"/>
       <c r="Z130" s="5" t="n"/>
       <c r="AA130" s="5" t="n"/>
+      <c r="AB130" s="5" t="n"/>
+      <c r="AC130" s="5" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="6" t="n"/>
@@ -4586,6 +4866,8 @@
       <c r="Y131" s="6" t="n"/>
       <c r="Z131" s="6" t="n"/>
       <c r="AA131" s="6" t="n"/>
+      <c r="AB131" s="6" t="n"/>
+      <c r="AC131" s="6" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="3" t="n"/>
@@ -4600,8 +4882,8 @@
       <c r="J132" s="3" t="n"/>
       <c r="K132" s="3" t="n"/>
       <c r="L132" s="3" t="n"/>
-      <c r="M132" s="5" t="n"/>
-      <c r="N132" s="5" t="n"/>
+      <c r="M132" s="3" t="n"/>
+      <c r="N132" s="3" t="n"/>
       <c r="O132" s="5" t="n"/>
       <c r="P132" s="5" t="n"/>
       <c r="Q132" s="5" t="n"/>
@@ -4615,6 +4897,8 @@
       <c r="Y132" s="5" t="n"/>
       <c r="Z132" s="5" t="n"/>
       <c r="AA132" s="5" t="n"/>
+      <c r="AB132" s="5" t="n"/>
+      <c r="AC132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="6" t="n"/>
@@ -4644,6 +4928,8 @@
       <c r="Y133" s="6" t="n"/>
       <c r="Z133" s="6" t="n"/>
       <c r="AA133" s="6" t="n"/>
+      <c r="AB133" s="6" t="n"/>
+      <c r="AC133" s="6" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="3" t="n"/>
@@ -4658,8 +4944,8 @@
       <c r="J134" s="3" t="n"/>
       <c r="K134" s="3" t="n"/>
       <c r="L134" s="3" t="n"/>
-      <c r="M134" s="5" t="n"/>
-      <c r="N134" s="5" t="n"/>
+      <c r="M134" s="3" t="n"/>
+      <c r="N134" s="3" t="n"/>
       <c r="O134" s="5" t="n"/>
       <c r="P134" s="5" t="n"/>
       <c r="Q134" s="5" t="n"/>
@@ -4673,6 +4959,8 @@
       <c r="Y134" s="5" t="n"/>
       <c r="Z134" s="5" t="n"/>
       <c r="AA134" s="5" t="n"/>
+      <c r="AB134" s="5" t="n"/>
+      <c r="AC134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="6" t="n"/>
@@ -4702,6 +4990,8 @@
       <c r="Y135" s="6" t="n"/>
       <c r="Z135" s="6" t="n"/>
       <c r="AA135" s="6" t="n"/>
+      <c r="AB135" s="6" t="n"/>
+      <c r="AC135" s="6" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="3" t="n"/>
@@ -4716,8 +5006,8 @@
       <c r="J136" s="3" t="n"/>
       <c r="K136" s="3" t="n"/>
       <c r="L136" s="3" t="n"/>
-      <c r="M136" s="5" t="n"/>
-      <c r="N136" s="5" t="n"/>
+      <c r="M136" s="3" t="n"/>
+      <c r="N136" s="3" t="n"/>
       <c r="O136" s="5" t="n"/>
       <c r="P136" s="5" t="n"/>
       <c r="Q136" s="5" t="n"/>
@@ -4731,6 +5021,8 @@
       <c r="Y136" s="5" t="n"/>
       <c r="Z136" s="5" t="n"/>
       <c r="AA136" s="5" t="n"/>
+      <c r="AB136" s="5" t="n"/>
+      <c r="AC136" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="6" t="n"/>
@@ -4760,6 +5052,8 @@
       <c r="Y137" s="6" t="n"/>
       <c r="Z137" s="6" t="n"/>
       <c r="AA137" s="6" t="n"/>
+      <c r="AB137" s="6" t="n"/>
+      <c r="AC137" s="6" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="3" t="n"/>
@@ -4774,8 +5068,8 @@
       <c r="J138" s="3" t="n"/>
       <c r="K138" s="3" t="n"/>
       <c r="L138" s="3" t="n"/>
-      <c r="M138" s="5" t="n"/>
-      <c r="N138" s="5" t="n"/>
+      <c r="M138" s="3" t="n"/>
+      <c r="N138" s="3" t="n"/>
       <c r="O138" s="5" t="n"/>
       <c r="P138" s="5" t="n"/>
       <c r="Q138" s="5" t="n"/>
@@ -4789,6 +5083,8 @@
       <c r="Y138" s="5" t="n"/>
       <c r="Z138" s="5" t="n"/>
       <c r="AA138" s="5" t="n"/>
+      <c r="AB138" s="5" t="n"/>
+      <c r="AC138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="6" t="n"/>
@@ -4818,6 +5114,8 @@
       <c r="Y139" s="6" t="n"/>
       <c r="Z139" s="6" t="n"/>
       <c r="AA139" s="6" t="n"/>
+      <c r="AB139" s="6" t="n"/>
+      <c r="AC139" s="6" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="3" t="n"/>
@@ -4832,8 +5130,8 @@
       <c r="J140" s="3" t="n"/>
       <c r="K140" s="3" t="n"/>
       <c r="L140" s="3" t="n"/>
-      <c r="M140" s="5" t="n"/>
-      <c r="N140" s="5" t="n"/>
+      <c r="M140" s="3" t="n"/>
+      <c r="N140" s="3" t="n"/>
       <c r="O140" s="5" t="n"/>
       <c r="P140" s="5" t="n"/>
       <c r="Q140" s="5" t="n"/>
@@ -4847,6 +5145,8 @@
       <c r="Y140" s="5" t="n"/>
       <c r="Z140" s="5" t="n"/>
       <c r="AA140" s="5" t="n"/>
+      <c r="AB140" s="5" t="n"/>
+      <c r="AC140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="6" t="n"/>
@@ -4876,6 +5176,8 @@
       <c r="Y141" s="6" t="n"/>
       <c r="Z141" s="6" t="n"/>
       <c r="AA141" s="6" t="n"/>
+      <c r="AB141" s="6" t="n"/>
+      <c r="AC141" s="6" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="3" t="n"/>
@@ -4890,8 +5192,8 @@
       <c r="J142" s="3" t="n"/>
       <c r="K142" s="3" t="n"/>
       <c r="L142" s="3" t="n"/>
-      <c r="M142" s="5" t="n"/>
-      <c r="N142" s="5" t="n"/>
+      <c r="M142" s="3" t="n"/>
+      <c r="N142" s="3" t="n"/>
       <c r="O142" s="5" t="n"/>
       <c r="P142" s="5" t="n"/>
       <c r="Q142" s="5" t="n"/>
@@ -4905,6 +5207,8 @@
       <c r="Y142" s="5" t="n"/>
       <c r="Z142" s="5" t="n"/>
       <c r="AA142" s="5" t="n"/>
+      <c r="AB142" s="5" t="n"/>
+      <c r="AC142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="6" t="n"/>
@@ -4934,6 +5238,8 @@
       <c r="Y143" s="6" t="n"/>
       <c r="Z143" s="6" t="n"/>
       <c r="AA143" s="6" t="n"/>
+      <c r="AB143" s="6" t="n"/>
+      <c r="AC143" s="6" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="3" t="n"/>
@@ -4948,8 +5254,8 @@
       <c r="J144" s="3" t="n"/>
       <c r="K144" s="3" t="n"/>
       <c r="L144" s="3" t="n"/>
-      <c r="M144" s="5" t="n"/>
-      <c r="N144" s="5" t="n"/>
+      <c r="M144" s="3" t="n"/>
+      <c r="N144" s="3" t="n"/>
       <c r="O144" s="5" t="n"/>
       <c r="P144" s="5" t="n"/>
       <c r="Q144" s="5" t="n"/>
@@ -4963,6 +5269,8 @@
       <c r="Y144" s="5" t="n"/>
       <c r="Z144" s="5" t="n"/>
       <c r="AA144" s="5" t="n"/>
+      <c r="AB144" s="5" t="n"/>
+      <c r="AC144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="6" t="n"/>
@@ -4992,6 +5300,8 @@
       <c r="Y145" s="6" t="n"/>
       <c r="Z145" s="6" t="n"/>
       <c r="AA145" s="6" t="n"/>
+      <c r="AB145" s="6" t="n"/>
+      <c r="AC145" s="6" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="3" t="n"/>
@@ -5006,8 +5316,8 @@
       <c r="J146" s="3" t="n"/>
       <c r="K146" s="3" t="n"/>
       <c r="L146" s="3" t="n"/>
-      <c r="M146" s="5" t="n"/>
-      <c r="N146" s="5" t="n"/>
+      <c r="M146" s="3" t="n"/>
+      <c r="N146" s="3" t="n"/>
       <c r="O146" s="5" t="n"/>
       <c r="P146" s="5" t="n"/>
       <c r="Q146" s="5" t="n"/>
@@ -5021,6 +5331,8 @@
       <c r="Y146" s="5" t="n"/>
       <c r="Z146" s="5" t="n"/>
       <c r="AA146" s="5" t="n"/>
+      <c r="AB146" s="5" t="n"/>
+      <c r="AC146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="6" t="n"/>
@@ -5050,6 +5362,8 @@
       <c r="Y147" s="6" t="n"/>
       <c r="Z147" s="6" t="n"/>
       <c r="AA147" s="6" t="n"/>
+      <c r="AB147" s="6" t="n"/>
+      <c r="AC147" s="6" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="3" t="n"/>
@@ -5064,8 +5378,8 @@
       <c r="J148" s="3" t="n"/>
       <c r="K148" s="3" t="n"/>
       <c r="L148" s="3" t="n"/>
-      <c r="M148" s="5" t="n"/>
-      <c r="N148" s="5" t="n"/>
+      <c r="M148" s="3" t="n"/>
+      <c r="N148" s="3" t="n"/>
       <c r="O148" s="5" t="n"/>
       <c r="P148" s="5" t="n"/>
       <c r="Q148" s="5" t="n"/>
@@ -5079,6 +5393,8 @@
       <c r="Y148" s="5" t="n"/>
       <c r="Z148" s="5" t="n"/>
       <c r="AA148" s="5" t="n"/>
+      <c r="AB148" s="5" t="n"/>
+      <c r="AC148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="6" t="n"/>
@@ -5108,6 +5424,8 @@
       <c r="Y149" s="6" t="n"/>
       <c r="Z149" s="6" t="n"/>
       <c r="AA149" s="6" t="n"/>
+      <c r="AB149" s="6" t="n"/>
+      <c r="AC149" s="6" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="3" t="n"/>
@@ -5122,8 +5440,8 @@
       <c r="J150" s="3" t="n"/>
       <c r="K150" s="3" t="n"/>
       <c r="L150" s="3" t="n"/>
-      <c r="M150" s="5" t="n"/>
-      <c r="N150" s="5" t="n"/>
+      <c r="M150" s="3" t="n"/>
+      <c r="N150" s="3" t="n"/>
       <c r="O150" s="5" t="n"/>
       <c r="P150" s="5" t="n"/>
       <c r="Q150" s="5" t="n"/>
@@ -5137,6 +5455,8 @@
       <c r="Y150" s="5" t="n"/>
       <c r="Z150" s="5" t="n"/>
       <c r="AA150" s="5" t="n"/>
+      <c r="AB150" s="5" t="n"/>
+      <c r="AC150" s="5" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="6" t="n"/>
@@ -5166,6 +5486,8 @@
       <c r="Y151" s="6" t="n"/>
       <c r="Z151" s="6" t="n"/>
       <c r="AA151" s="6" t="n"/>
+      <c r="AB151" s="6" t="n"/>
+      <c r="AC151" s="6" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="3" t="n"/>
@@ -5180,8 +5502,8 @@
       <c r="J152" s="3" t="n"/>
       <c r="K152" s="3" t="n"/>
       <c r="L152" s="3" t="n"/>
-      <c r="M152" s="5" t="n"/>
-      <c r="N152" s="5" t="n"/>
+      <c r="M152" s="3" t="n"/>
+      <c r="N152" s="3" t="n"/>
       <c r="O152" s="5" t="n"/>
       <c r="P152" s="5" t="n"/>
       <c r="Q152" s="5" t="n"/>
@@ -5195,6 +5517,8 @@
       <c r="Y152" s="5" t="n"/>
       <c r="Z152" s="5" t="n"/>
       <c r="AA152" s="5" t="n"/>
+      <c r="AB152" s="5" t="n"/>
+      <c r="AC152" s="5" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="6" t="n"/>
@@ -5224,6 +5548,8 @@
       <c r="Y153" s="6" t="n"/>
       <c r="Z153" s="6" t="n"/>
       <c r="AA153" s="6" t="n"/>
+      <c r="AB153" s="6" t="n"/>
+      <c r="AC153" s="6" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="3" t="n"/>
@@ -5238,8 +5564,8 @@
       <c r="J154" s="3" t="n"/>
       <c r="K154" s="3" t="n"/>
       <c r="L154" s="3" t="n"/>
-      <c r="M154" s="5" t="n"/>
-      <c r="N154" s="5" t="n"/>
+      <c r="M154" s="3" t="n"/>
+      <c r="N154" s="3" t="n"/>
       <c r="O154" s="5" t="n"/>
       <c r="P154" s="5" t="n"/>
       <c r="Q154" s="5" t="n"/>
@@ -5253,6 +5579,8 @@
       <c r="Y154" s="5" t="n"/>
       <c r="Z154" s="5" t="n"/>
       <c r="AA154" s="5" t="n"/>
+      <c r="AB154" s="5" t="n"/>
+      <c r="AC154" s="5" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="6" t="n"/>
@@ -5282,6 +5610,8 @@
       <c r="Y155" s="6" t="n"/>
       <c r="Z155" s="6" t="n"/>
       <c r="AA155" s="6" t="n"/>
+      <c r="AB155" s="6" t="n"/>
+      <c r="AC155" s="6" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="3" t="n"/>
@@ -5296,8 +5626,8 @@
       <c r="J156" s="3" t="n"/>
       <c r="K156" s="3" t="n"/>
       <c r="L156" s="3" t="n"/>
-      <c r="M156" s="5" t="n"/>
-      <c r="N156" s="5" t="n"/>
+      <c r="M156" s="3" t="n"/>
+      <c r="N156" s="3" t="n"/>
       <c r="O156" s="5" t="n"/>
       <c r="P156" s="5" t="n"/>
       <c r="Q156" s="5" t="n"/>
@@ -5311,6 +5641,8 @@
       <c r="Y156" s="5" t="n"/>
       <c r="Z156" s="5" t="n"/>
       <c r="AA156" s="5" t="n"/>
+      <c r="AB156" s="5" t="n"/>
+      <c r="AC156" s="5" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="6" t="n"/>
@@ -5340,6 +5672,8 @@
       <c r="Y157" s="6" t="n"/>
       <c r="Z157" s="6" t="n"/>
       <c r="AA157" s="6" t="n"/>
+      <c r="AB157" s="6" t="n"/>
+      <c r="AC157" s="6" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="3" t="n"/>
@@ -5354,8 +5688,8 @@
       <c r="J158" s="3" t="n"/>
       <c r="K158" s="3" t="n"/>
       <c r="L158" s="3" t="n"/>
-      <c r="M158" s="5" t="n"/>
-      <c r="N158" s="5" t="n"/>
+      <c r="M158" s="3" t="n"/>
+      <c r="N158" s="3" t="n"/>
       <c r="O158" s="5" t="n"/>
       <c r="P158" s="5" t="n"/>
       <c r="Q158" s="5" t="n"/>
@@ -5369,6 +5703,8 @@
       <c r="Y158" s="5" t="n"/>
       <c r="Z158" s="5" t="n"/>
       <c r="AA158" s="5" t="n"/>
+      <c r="AB158" s="5" t="n"/>
+      <c r="AC158" s="5" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="6" t="n"/>
@@ -5398,6 +5734,8 @@
       <c r="Y159" s="6" t="n"/>
       <c r="Z159" s="6" t="n"/>
       <c r="AA159" s="6" t="n"/>
+      <c r="AB159" s="6" t="n"/>
+      <c r="AC159" s="6" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="3" t="n"/>
@@ -5412,8 +5750,8 @@
       <c r="J160" s="3" t="n"/>
       <c r="K160" s="3" t="n"/>
       <c r="L160" s="3" t="n"/>
-      <c r="M160" s="5" t="n"/>
-      <c r="N160" s="5" t="n"/>
+      <c r="M160" s="3" t="n"/>
+      <c r="N160" s="3" t="n"/>
       <c r="O160" s="5" t="n"/>
       <c r="P160" s="5" t="n"/>
       <c r="Q160" s="5" t="n"/>
@@ -5427,6 +5765,8 @@
       <c r="Y160" s="5" t="n"/>
       <c r="Z160" s="5" t="n"/>
       <c r="AA160" s="5" t="n"/>
+      <c r="AB160" s="5" t="n"/>
+      <c r="AC160" s="5" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="6" t="n"/>
@@ -5456,6 +5796,8 @@
       <c r="Y161" s="6" t="n"/>
       <c r="Z161" s="6" t="n"/>
       <c r="AA161" s="6" t="n"/>
+      <c r="AB161" s="6" t="n"/>
+      <c r="AC161" s="6" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="3" t="n"/>
@@ -5470,8 +5812,8 @@
       <c r="J162" s="3" t="n"/>
       <c r="K162" s="3" t="n"/>
       <c r="L162" s="3" t="n"/>
-      <c r="M162" s="5" t="n"/>
-      <c r="N162" s="5" t="n"/>
+      <c r="M162" s="3" t="n"/>
+      <c r="N162" s="3" t="n"/>
       <c r="O162" s="5" t="n"/>
       <c r="P162" s="5" t="n"/>
       <c r="Q162" s="5" t="n"/>
@@ -5485,6 +5827,8 @@
       <c r="Y162" s="5" t="n"/>
       <c r="Z162" s="5" t="n"/>
       <c r="AA162" s="5" t="n"/>
+      <c r="AB162" s="5" t="n"/>
+      <c r="AC162" s="5" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="6" t="n"/>
@@ -5514,6 +5858,8 @@
       <c r="Y163" s="6" t="n"/>
       <c r="Z163" s="6" t="n"/>
       <c r="AA163" s="6" t="n"/>
+      <c r="AB163" s="6" t="n"/>
+      <c r="AC163" s="6" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="3" t="n"/>
@@ -5528,8 +5874,8 @@
       <c r="J164" s="3" t="n"/>
       <c r="K164" s="3" t="n"/>
       <c r="L164" s="3" t="n"/>
-      <c r="M164" s="5" t="n"/>
-      <c r="N164" s="5" t="n"/>
+      <c r="M164" s="3" t="n"/>
+      <c r="N164" s="3" t="n"/>
       <c r="O164" s="5" t="n"/>
       <c r="P164" s="5" t="n"/>
       <c r="Q164" s="5" t="n"/>
@@ -5543,6 +5889,8 @@
       <c r="Y164" s="5" t="n"/>
       <c r="Z164" s="5" t="n"/>
       <c r="AA164" s="5" t="n"/>
+      <c r="AB164" s="5" t="n"/>
+      <c r="AC164" s="5" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="6" t="n"/>
@@ -5572,6 +5920,8 @@
       <c r="Y165" s="6" t="n"/>
       <c r="Z165" s="6" t="n"/>
       <c r="AA165" s="6" t="n"/>
+      <c r="AB165" s="6" t="n"/>
+      <c r="AC165" s="6" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="3" t="n"/>
@@ -5586,8 +5936,8 @@
       <c r="J166" s="3" t="n"/>
       <c r="K166" s="3" t="n"/>
       <c r="L166" s="3" t="n"/>
-      <c r="M166" s="5" t="n"/>
-      <c r="N166" s="5" t="n"/>
+      <c r="M166" s="3" t="n"/>
+      <c r="N166" s="3" t="n"/>
       <c r="O166" s="5" t="n"/>
       <c r="P166" s="5" t="n"/>
       <c r="Q166" s="5" t="n"/>
@@ -5601,6 +5951,8 @@
       <c r="Y166" s="5" t="n"/>
       <c r="Z166" s="5" t="n"/>
       <c r="AA166" s="5" t="n"/>
+      <c r="AB166" s="5" t="n"/>
+      <c r="AC166" s="5" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="6" t="n"/>
@@ -5630,6 +5982,8 @@
       <c r="Y167" s="6" t="n"/>
       <c r="Z167" s="6" t="n"/>
       <c r="AA167" s="6" t="n"/>
+      <c r="AB167" s="6" t="n"/>
+      <c r="AC167" s="6" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="3" t="n"/>
@@ -5644,8 +5998,8 @@
       <c r="J168" s="3" t="n"/>
       <c r="K168" s="3" t="n"/>
       <c r="L168" s="3" t="n"/>
-      <c r="M168" s="5" t="n"/>
-      <c r="N168" s="5" t="n"/>
+      <c r="M168" s="3" t="n"/>
+      <c r="N168" s="3" t="n"/>
       <c r="O168" s="5" t="n"/>
       <c r="P168" s="5" t="n"/>
       <c r="Q168" s="5" t="n"/>
@@ -5659,6 +6013,8 @@
       <c r="Y168" s="5" t="n"/>
       <c r="Z168" s="5" t="n"/>
       <c r="AA168" s="5" t="n"/>
+      <c r="AB168" s="5" t="n"/>
+      <c r="AC168" s="5" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="6" t="n"/>
@@ -5688,6 +6044,8 @@
       <c r="Y169" s="6" t="n"/>
       <c r="Z169" s="6" t="n"/>
       <c r="AA169" s="6" t="n"/>
+      <c r="AB169" s="6" t="n"/>
+      <c r="AC169" s="6" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="3" t="n"/>
@@ -5702,8 +6060,8 @@
       <c r="J170" s="3" t="n"/>
       <c r="K170" s="3" t="n"/>
       <c r="L170" s="3" t="n"/>
-      <c r="M170" s="5" t="n"/>
-      <c r="N170" s="5" t="n"/>
+      <c r="M170" s="3" t="n"/>
+      <c r="N170" s="3" t="n"/>
       <c r="O170" s="5" t="n"/>
       <c r="P170" s="5" t="n"/>
       <c r="Q170" s="5" t="n"/>
@@ -5717,6 +6075,8 @@
       <c r="Y170" s="5" t="n"/>
       <c r="Z170" s="5" t="n"/>
       <c r="AA170" s="5" t="n"/>
+      <c r="AB170" s="5" t="n"/>
+      <c r="AC170" s="5" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="6" t="n"/>
@@ -5746,6 +6106,8 @@
       <c r="Y171" s="6" t="n"/>
       <c r="Z171" s="6" t="n"/>
       <c r="AA171" s="6" t="n"/>
+      <c r="AB171" s="6" t="n"/>
+      <c r="AC171" s="6" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="3" t="n"/>
@@ -5760,8 +6122,8 @@
       <c r="J172" s="3" t="n"/>
       <c r="K172" s="3" t="n"/>
       <c r="L172" s="3" t="n"/>
-      <c r="M172" s="5" t="n"/>
-      <c r="N172" s="5" t="n"/>
+      <c r="M172" s="3" t="n"/>
+      <c r="N172" s="3" t="n"/>
       <c r="O172" s="5" t="n"/>
       <c r="P172" s="5" t="n"/>
       <c r="Q172" s="5" t="n"/>
@@ -5775,6 +6137,8 @@
       <c r="Y172" s="5" t="n"/>
       <c r="Z172" s="5" t="n"/>
       <c r="AA172" s="5" t="n"/>
+      <c r="AB172" s="5" t="n"/>
+      <c r="AC172" s="5" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="6" t="n"/>
@@ -5804,6 +6168,8 @@
       <c r="Y173" s="6" t="n"/>
       <c r="Z173" s="6" t="n"/>
       <c r="AA173" s="6" t="n"/>
+      <c r="AB173" s="6" t="n"/>
+      <c r="AC173" s="6" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="3" t="n"/>
@@ -5818,8 +6184,8 @@
       <c r="J174" s="3" t="n"/>
       <c r="K174" s="3" t="n"/>
       <c r="L174" s="3" t="n"/>
-      <c r="M174" s="5" t="n"/>
-      <c r="N174" s="5" t="n"/>
+      <c r="M174" s="3" t="n"/>
+      <c r="N174" s="3" t="n"/>
       <c r="O174" s="5" t="n"/>
       <c r="P174" s="5" t="n"/>
       <c r="Q174" s="5" t="n"/>
@@ -5833,6 +6199,8 @@
       <c r="Y174" s="5" t="n"/>
       <c r="Z174" s="5" t="n"/>
       <c r="AA174" s="5" t="n"/>
+      <c r="AB174" s="5" t="n"/>
+      <c r="AC174" s="5" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="6" t="n"/>
@@ -5862,6 +6230,8 @@
       <c r="Y175" s="6" t="n"/>
       <c r="Z175" s="6" t="n"/>
       <c r="AA175" s="6" t="n"/>
+      <c r="AB175" s="6" t="n"/>
+      <c r="AC175" s="6" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="3" t="n"/>
@@ -5876,8 +6246,8 @@
       <c r="J176" s="3" t="n"/>
       <c r="K176" s="3" t="n"/>
       <c r="L176" s="3" t="n"/>
-      <c r="M176" s="5" t="n"/>
-      <c r="N176" s="5" t="n"/>
+      <c r="M176" s="3" t="n"/>
+      <c r="N176" s="3" t="n"/>
       <c r="O176" s="5" t="n"/>
       <c r="P176" s="5" t="n"/>
       <c r="Q176" s="5" t="n"/>
@@ -5891,6 +6261,8 @@
       <c r="Y176" s="5" t="n"/>
       <c r="Z176" s="5" t="n"/>
       <c r="AA176" s="5" t="n"/>
+      <c r="AB176" s="5" t="n"/>
+      <c r="AC176" s="5" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="6" t="n"/>
@@ -5920,6 +6292,8 @@
       <c r="Y177" s="6" t="n"/>
       <c r="Z177" s="6" t="n"/>
       <c r="AA177" s="6" t="n"/>
+      <c r="AB177" s="6" t="n"/>
+      <c r="AC177" s="6" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="3" t="n"/>
@@ -5934,8 +6308,8 @@
       <c r="J178" s="3" t="n"/>
       <c r="K178" s="3" t="n"/>
       <c r="L178" s="3" t="n"/>
-      <c r="M178" s="5" t="n"/>
-      <c r="N178" s="5" t="n"/>
+      <c r="M178" s="3" t="n"/>
+      <c r="N178" s="3" t="n"/>
       <c r="O178" s="5" t="n"/>
       <c r="P178" s="5" t="n"/>
       <c r="Q178" s="5" t="n"/>
@@ -5949,6 +6323,8 @@
       <c r="Y178" s="5" t="n"/>
       <c r="Z178" s="5" t="n"/>
       <c r="AA178" s="5" t="n"/>
+      <c r="AB178" s="5" t="n"/>
+      <c r="AC178" s="5" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="6" t="n"/>
@@ -5978,6 +6354,8 @@
       <c r="Y179" s="6" t="n"/>
       <c r="Z179" s="6" t="n"/>
       <c r="AA179" s="6" t="n"/>
+      <c r="AB179" s="6" t="n"/>
+      <c r="AC179" s="6" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="3" t="n"/>
@@ -5992,8 +6370,8 @@
       <c r="J180" s="3" t="n"/>
       <c r="K180" s="3" t="n"/>
       <c r="L180" s="3" t="n"/>
-      <c r="M180" s="5" t="n"/>
-      <c r="N180" s="5" t="n"/>
+      <c r="M180" s="3" t="n"/>
+      <c r="N180" s="3" t="n"/>
       <c r="O180" s="5" t="n"/>
       <c r="P180" s="5" t="n"/>
       <c r="Q180" s="5" t="n"/>
@@ -6007,6 +6385,8 @@
       <c r="Y180" s="5" t="n"/>
       <c r="Z180" s="5" t="n"/>
       <c r="AA180" s="5" t="n"/>
+      <c r="AB180" s="5" t="n"/>
+      <c r="AC180" s="5" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="6" t="n"/>
@@ -6036,6 +6416,8 @@
       <c r="Y181" s="6" t="n"/>
       <c r="Z181" s="6" t="n"/>
       <c r="AA181" s="6" t="n"/>
+      <c r="AB181" s="6" t="n"/>
+      <c r="AC181" s="6" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="3" t="n"/>
@@ -6050,8 +6432,8 @@
       <c r="J182" s="3" t="n"/>
       <c r="K182" s="3" t="n"/>
       <c r="L182" s="3" t="n"/>
-      <c r="M182" s="5" t="n"/>
-      <c r="N182" s="5" t="n"/>
+      <c r="M182" s="3" t="n"/>
+      <c r="N182" s="3" t="n"/>
       <c r="O182" s="5" t="n"/>
       <c r="P182" s="5" t="n"/>
       <c r="Q182" s="5" t="n"/>
@@ -6065,6 +6447,8 @@
       <c r="Y182" s="5" t="n"/>
       <c r="Z182" s="5" t="n"/>
       <c r="AA182" s="5" t="n"/>
+      <c r="AB182" s="5" t="n"/>
+      <c r="AC182" s="5" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="6" t="n"/>
@@ -6094,6 +6478,8 @@
       <c r="Y183" s="6" t="n"/>
       <c r="Z183" s="6" t="n"/>
       <c r="AA183" s="6" t="n"/>
+      <c r="AB183" s="6" t="n"/>
+      <c r="AC183" s="6" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="3" t="n"/>
@@ -6108,8 +6494,8 @@
       <c r="J184" s="3" t="n"/>
       <c r="K184" s="3" t="n"/>
       <c r="L184" s="3" t="n"/>
-      <c r="M184" s="5" t="n"/>
-      <c r="N184" s="5" t="n"/>
+      <c r="M184" s="3" t="n"/>
+      <c r="N184" s="3" t="n"/>
       <c r="O184" s="5" t="n"/>
       <c r="P184" s="5" t="n"/>
       <c r="Q184" s="5" t="n"/>
@@ -6123,6 +6509,8 @@
       <c r="Y184" s="5" t="n"/>
       <c r="Z184" s="5" t="n"/>
       <c r="AA184" s="5" t="n"/>
+      <c r="AB184" s="5" t="n"/>
+      <c r="AC184" s="5" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="6" t="n"/>
@@ -6152,6 +6540,8 @@
       <c r="Y185" s="6" t="n"/>
       <c r="Z185" s="6" t="n"/>
       <c r="AA185" s="6" t="n"/>
+      <c r="AB185" s="6" t="n"/>
+      <c r="AC185" s="6" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="3" t="n"/>
@@ -6166,8 +6556,8 @@
       <c r="J186" s="3" t="n"/>
       <c r="K186" s="3" t="n"/>
       <c r="L186" s="3" t="n"/>
-      <c r="M186" s="5" t="n"/>
-      <c r="N186" s="5" t="n"/>
+      <c r="M186" s="3" t="n"/>
+      <c r="N186" s="3" t="n"/>
       <c r="O186" s="5" t="n"/>
       <c r="P186" s="5" t="n"/>
       <c r="Q186" s="5" t="n"/>
@@ -6181,6 +6571,8 @@
       <c r="Y186" s="5" t="n"/>
       <c r="Z186" s="5" t="n"/>
       <c r="AA186" s="5" t="n"/>
+      <c r="AB186" s="5" t="n"/>
+      <c r="AC186" s="5" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="6" t="n"/>
@@ -6210,6 +6602,8 @@
       <c r="Y187" s="6" t="n"/>
       <c r="Z187" s="6" t="n"/>
       <c r="AA187" s="6" t="n"/>
+      <c r="AB187" s="6" t="n"/>
+      <c r="AC187" s="6" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="3" t="n"/>
@@ -6224,8 +6618,8 @@
       <c r="J188" s="3" t="n"/>
       <c r="K188" s="3" t="n"/>
       <c r="L188" s="3" t="n"/>
-      <c r="M188" s="5" t="n"/>
-      <c r="N188" s="5" t="n"/>
+      <c r="M188" s="3" t="n"/>
+      <c r="N188" s="3" t="n"/>
       <c r="O188" s="5" t="n"/>
       <c r="P188" s="5" t="n"/>
       <c r="Q188" s="5" t="n"/>
@@ -6239,6 +6633,8 @@
       <c r="Y188" s="5" t="n"/>
       <c r="Z188" s="5" t="n"/>
       <c r="AA188" s="5" t="n"/>
+      <c r="AB188" s="5" t="n"/>
+      <c r="AC188" s="5" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="6" t="n"/>
@@ -6268,6 +6664,8 @@
       <c r="Y189" s="6" t="n"/>
       <c r="Z189" s="6" t="n"/>
       <c r="AA189" s="6" t="n"/>
+      <c r="AB189" s="6" t="n"/>
+      <c r="AC189" s="6" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="3" t="n"/>
@@ -6282,8 +6680,8 @@
       <c r="J190" s="3" t="n"/>
       <c r="K190" s="3" t="n"/>
       <c r="L190" s="3" t="n"/>
-      <c r="M190" s="5" t="n"/>
-      <c r="N190" s="5" t="n"/>
+      <c r="M190" s="3" t="n"/>
+      <c r="N190" s="3" t="n"/>
       <c r="O190" s="5" t="n"/>
       <c r="P190" s="5" t="n"/>
       <c r="Q190" s="5" t="n"/>
@@ -6297,6 +6695,8 @@
       <c r="Y190" s="5" t="n"/>
       <c r="Z190" s="5" t="n"/>
       <c r="AA190" s="5" t="n"/>
+      <c r="AB190" s="5" t="n"/>
+      <c r="AC190" s="5" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="6" t="n"/>
@@ -6326,6 +6726,8 @@
       <c r="Y191" s="6" t="n"/>
       <c r="Z191" s="6" t="n"/>
       <c r="AA191" s="6" t="n"/>
+      <c r="AB191" s="6" t="n"/>
+      <c r="AC191" s="6" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="3" t="n"/>
@@ -6340,8 +6742,8 @@
       <c r="J192" s="3" t="n"/>
       <c r="K192" s="3" t="n"/>
       <c r="L192" s="3" t="n"/>
-      <c r="M192" s="5" t="n"/>
-      <c r="N192" s="5" t="n"/>
+      <c r="M192" s="3" t="n"/>
+      <c r="N192" s="3" t="n"/>
       <c r="O192" s="5" t="n"/>
       <c r="P192" s="5" t="n"/>
       <c r="Q192" s="5" t="n"/>
@@ -6355,6 +6757,8 @@
       <c r="Y192" s="5" t="n"/>
       <c r="Z192" s="5" t="n"/>
       <c r="AA192" s="5" t="n"/>
+      <c r="AB192" s="5" t="n"/>
+      <c r="AC192" s="5" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="6" t="n"/>
@@ -6384,6 +6788,8 @@
       <c r="Y193" s="6" t="n"/>
       <c r="Z193" s="6" t="n"/>
       <c r="AA193" s="6" t="n"/>
+      <c r="AB193" s="6" t="n"/>
+      <c r="AC193" s="6" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="3" t="n"/>
@@ -6398,8 +6804,8 @@
       <c r="J194" s="3" t="n"/>
       <c r="K194" s="3" t="n"/>
       <c r="L194" s="3" t="n"/>
-      <c r="M194" s="5" t="n"/>
-      <c r="N194" s="5" t="n"/>
+      <c r="M194" s="3" t="n"/>
+      <c r="N194" s="3" t="n"/>
       <c r="O194" s="5" t="n"/>
       <c r="P194" s="5" t="n"/>
       <c r="Q194" s="5" t="n"/>
@@ -6413,6 +6819,8 @@
       <c r="Y194" s="5" t="n"/>
       <c r="Z194" s="5" t="n"/>
       <c r="AA194" s="5" t="n"/>
+      <c r="AB194" s="5" t="n"/>
+      <c r="AC194" s="5" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="6" t="n"/>
@@ -6442,6 +6850,8 @@
       <c r="Y195" s="6" t="n"/>
       <c r="Z195" s="6" t="n"/>
       <c r="AA195" s="6" t="n"/>
+      <c r="AB195" s="6" t="n"/>
+      <c r="AC195" s="6" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="3" t="n"/>
@@ -6456,8 +6866,8 @@
       <c r="J196" s="3" t="n"/>
       <c r="K196" s="3" t="n"/>
       <c r="L196" s="3" t="n"/>
-      <c r="M196" s="5" t="n"/>
-      <c r="N196" s="5" t="n"/>
+      <c r="M196" s="3" t="n"/>
+      <c r="N196" s="3" t="n"/>
       <c r="O196" s="5" t="n"/>
       <c r="P196" s="5" t="n"/>
       <c r="Q196" s="5" t="n"/>
@@ -6471,6 +6881,8 @@
       <c r="Y196" s="5" t="n"/>
       <c r="Z196" s="5" t="n"/>
       <c r="AA196" s="5" t="n"/>
+      <c r="AB196" s="5" t="n"/>
+      <c r="AC196" s="5" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="6" t="n"/>
@@ -6500,6 +6912,8 @@
       <c r="Y197" s="6" t="n"/>
       <c r="Z197" s="6" t="n"/>
       <c r="AA197" s="6" t="n"/>
+      <c r="AB197" s="6" t="n"/>
+      <c r="AC197" s="6" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="3" t="n"/>
@@ -6514,8 +6928,8 @@
       <c r="J198" s="3" t="n"/>
       <c r="K198" s="3" t="n"/>
       <c r="L198" s="3" t="n"/>
-      <c r="M198" s="5" t="n"/>
-      <c r="N198" s="5" t="n"/>
+      <c r="M198" s="3" t="n"/>
+      <c r="N198" s="3" t="n"/>
       <c r="O198" s="5" t="n"/>
       <c r="P198" s="5" t="n"/>
       <c r="Q198" s="5" t="n"/>
@@ -6529,6 +6943,8 @@
       <c r="Y198" s="5" t="n"/>
       <c r="Z198" s="5" t="n"/>
       <c r="AA198" s="5" t="n"/>
+      <c r="AB198" s="5" t="n"/>
+      <c r="AC198" s="5" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="6" t="n"/>
@@ -6558,6 +6974,8 @@
       <c r="Y199" s="6" t="n"/>
       <c r="Z199" s="6" t="n"/>
       <c r="AA199" s="6" t="n"/>
+      <c r="AB199" s="6" t="n"/>
+      <c r="AC199" s="6" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="3" t="n"/>
@@ -6572,8 +6990,8 @@
       <c r="J200" s="3" t="n"/>
       <c r="K200" s="3" t="n"/>
       <c r="L200" s="3" t="n"/>
-      <c r="M200" s="5" t="n"/>
-      <c r="N200" s="5" t="n"/>
+      <c r="M200" s="3" t="n"/>
+      <c r="N200" s="3" t="n"/>
       <c r="O200" s="5" t="n"/>
       <c r="P200" s="5" t="n"/>
       <c r="Q200" s="5" t="n"/>
@@ -6587,6 +7005,8 @@
       <c r="Y200" s="5" t="n"/>
       <c r="Z200" s="5" t="n"/>
       <c r="AA200" s="5" t="n"/>
+      <c r="AB200" s="5" t="n"/>
+      <c r="AC200" s="5" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="6" t="n"/>
@@ -6616,6 +7036,8 @@
       <c r="Y201" s="6" t="n"/>
       <c r="Z201" s="6" t="n"/>
       <c r="AA201" s="6" t="n"/>
+      <c r="AB201" s="6" t="n"/>
+      <c r="AC201" s="6" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="3" t="n"/>
@@ -6630,8 +7052,8 @@
       <c r="J202" s="3" t="n"/>
       <c r="K202" s="3" t="n"/>
       <c r="L202" s="3" t="n"/>
-      <c r="M202" s="5" t="n"/>
-      <c r="N202" s="5" t="n"/>
+      <c r="M202" s="3" t="n"/>
+      <c r="N202" s="3" t="n"/>
       <c r="O202" s="5" t="n"/>
       <c r="P202" s="5" t="n"/>
       <c r="Q202" s="5" t="n"/>
@@ -6645,6 +7067,8 @@
       <c r="Y202" s="5" t="n"/>
       <c r="Z202" s="5" t="n"/>
       <c r="AA202" s="5" t="n"/>
+      <c r="AB202" s="5" t="n"/>
+      <c r="AC202" s="5" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="6" t="n"/>
@@ -6674,6 +7098,8 @@
       <c r="Y203" s="6" t="n"/>
       <c r="Z203" s="6" t="n"/>
       <c r="AA203" s="6" t="n"/>
+      <c r="AB203" s="6" t="n"/>
+      <c r="AC203" s="6" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="3" t="n"/>
@@ -6688,8 +7114,8 @@
       <c r="J204" s="3" t="n"/>
       <c r="K204" s="3" t="n"/>
       <c r="L204" s="3" t="n"/>
-      <c r="M204" s="5" t="n"/>
-      <c r="N204" s="5" t="n"/>
+      <c r="M204" s="3" t="n"/>
+      <c r="N204" s="3" t="n"/>
       <c r="O204" s="5" t="n"/>
       <c r="P204" s="5" t="n"/>
       <c r="Q204" s="5" t="n"/>
@@ -6703,6 +7129,8 @@
       <c r="Y204" s="5" t="n"/>
       <c r="Z204" s="5" t="n"/>
       <c r="AA204" s="5" t="n"/>
+      <c r="AB204" s="5" t="n"/>
+      <c r="AC204" s="5" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="6" t="n"/>
@@ -6732,6 +7160,8 @@
       <c r="Y205" s="6" t="n"/>
       <c r="Z205" s="6" t="n"/>
       <c r="AA205" s="6" t="n"/>
+      <c r="AB205" s="6" t="n"/>
+      <c r="AC205" s="6" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="3" t="n"/>
@@ -6746,8 +7176,8 @@
       <c r="J206" s="3" t="n"/>
       <c r="K206" s="3" t="n"/>
       <c r="L206" s="3" t="n"/>
-      <c r="M206" s="5" t="n"/>
-      <c r="N206" s="5" t="n"/>
+      <c r="M206" s="3" t="n"/>
+      <c r="N206" s="3" t="n"/>
       <c r="O206" s="5" t="n"/>
       <c r="P206" s="5" t="n"/>
       <c r="Q206" s="5" t="n"/>
@@ -6761,6 +7191,8 @@
       <c r="Y206" s="5" t="n"/>
       <c r="Z206" s="5" t="n"/>
       <c r="AA206" s="5" t="n"/>
+      <c r="AB206" s="5" t="n"/>
+      <c r="AC206" s="5" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="6" t="n"/>
@@ -6790,6 +7222,8 @@
       <c r="Y207" s="6" t="n"/>
       <c r="Z207" s="6" t="n"/>
       <c r="AA207" s="6" t="n"/>
+      <c r="AB207" s="6" t="n"/>
+      <c r="AC207" s="6" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="3" t="n"/>
@@ -6804,8 +7238,8 @@
       <c r="J208" s="3" t="n"/>
       <c r="K208" s="3" t="n"/>
       <c r="L208" s="3" t="n"/>
-      <c r="M208" s="5" t="n"/>
-      <c r="N208" s="5" t="n"/>
+      <c r="M208" s="3" t="n"/>
+      <c r="N208" s="3" t="n"/>
       <c r="O208" s="5" t="n"/>
       <c r="P208" s="5" t="n"/>
       <c r="Q208" s="5" t="n"/>
@@ -6819,6 +7253,8 @@
       <c r="Y208" s="5" t="n"/>
       <c r="Z208" s="5" t="n"/>
       <c r="AA208" s="5" t="n"/>
+      <c r="AB208" s="5" t="n"/>
+      <c r="AC208" s="5" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="6" t="n"/>
@@ -6848,6 +7284,8 @@
       <c r="Y209" s="6" t="n"/>
       <c r="Z209" s="6" t="n"/>
       <c r="AA209" s="6" t="n"/>
+      <c r="AB209" s="6" t="n"/>
+      <c r="AC209" s="6" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="3" t="n"/>
@@ -6862,8 +7300,8 @@
       <c r="J210" s="3" t="n"/>
       <c r="K210" s="3" t="n"/>
       <c r="L210" s="3" t="n"/>
-      <c r="M210" s="5" t="n"/>
-      <c r="N210" s="5" t="n"/>
+      <c r="M210" s="3" t="n"/>
+      <c r="N210" s="3" t="n"/>
       <c r="O210" s="5" t="n"/>
       <c r="P210" s="5" t="n"/>
       <c r="Q210" s="5" t="n"/>
@@ -6877,6 +7315,8 @@
       <c r="Y210" s="5" t="n"/>
       <c r="Z210" s="5" t="n"/>
       <c r="AA210" s="5" t="n"/>
+      <c r="AB210" s="5" t="n"/>
+      <c r="AC210" s="5" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="6" t="n"/>
@@ -6906,6 +7346,8 @@
       <c r="Y211" s="6" t="n"/>
       <c r="Z211" s="6" t="n"/>
       <c r="AA211" s="6" t="n"/>
+      <c r="AB211" s="6" t="n"/>
+      <c r="AC211" s="6" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="3" t="n"/>
@@ -6920,8 +7362,8 @@
       <c r="J212" s="3" t="n"/>
       <c r="K212" s="3" t="n"/>
       <c r="L212" s="3" t="n"/>
-      <c r="M212" s="5" t="n"/>
-      <c r="N212" s="5" t="n"/>
+      <c r="M212" s="3" t="n"/>
+      <c r="N212" s="3" t="n"/>
       <c r="O212" s="5" t="n"/>
       <c r="P212" s="5" t="n"/>
       <c r="Q212" s="5" t="n"/>
@@ -6935,6 +7377,8 @@
       <c r="Y212" s="5" t="n"/>
       <c r="Z212" s="5" t="n"/>
       <c r="AA212" s="5" t="n"/>
+      <c r="AB212" s="5" t="n"/>
+      <c r="AC212" s="5" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="6" t="n"/>
@@ -6964,6 +7408,8 @@
       <c r="Y213" s="6" t="n"/>
       <c r="Z213" s="6" t="n"/>
       <c r="AA213" s="6" t="n"/>
+      <c r="AB213" s="6" t="n"/>
+      <c r="AC213" s="6" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="3" t="n"/>
@@ -6978,8 +7424,8 @@
       <c r="J214" s="3" t="n"/>
       <c r="K214" s="3" t="n"/>
       <c r="L214" s="3" t="n"/>
-      <c r="M214" s="5" t="n"/>
-      <c r="N214" s="5" t="n"/>
+      <c r="M214" s="3" t="n"/>
+      <c r="N214" s="3" t="n"/>
       <c r="O214" s="5" t="n"/>
       <c r="P214" s="5" t="n"/>
       <c r="Q214" s="5" t="n"/>
@@ -6993,6 +7439,8 @@
       <c r="Y214" s="5" t="n"/>
       <c r="Z214" s="5" t="n"/>
       <c r="AA214" s="5" t="n"/>
+      <c r="AB214" s="5" t="n"/>
+      <c r="AC214" s="5" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="6" t="n"/>
@@ -7022,6 +7470,8 @@
       <c r="Y215" s="6" t="n"/>
       <c r="Z215" s="6" t="n"/>
       <c r="AA215" s="6" t="n"/>
+      <c r="AB215" s="6" t="n"/>
+      <c r="AC215" s="6" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="3" t="n"/>
@@ -7036,8 +7486,8 @@
       <c r="J216" s="3" t="n"/>
       <c r="K216" s="3" t="n"/>
       <c r="L216" s="3" t="n"/>
-      <c r="M216" s="5" t="n"/>
-      <c r="N216" s="5" t="n"/>
+      <c r="M216" s="3" t="n"/>
+      <c r="N216" s="3" t="n"/>
       <c r="O216" s="5" t="n"/>
       <c r="P216" s="5" t="n"/>
       <c r="Q216" s="5" t="n"/>
@@ -7051,6 +7501,8 @@
       <c r="Y216" s="5" t="n"/>
       <c r="Z216" s="5" t="n"/>
       <c r="AA216" s="5" t="n"/>
+      <c r="AB216" s="5" t="n"/>
+      <c r="AC216" s="5" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="6" t="n"/>
@@ -7080,6 +7532,8 @@
       <c r="Y217" s="6" t="n"/>
       <c r="Z217" s="6" t="n"/>
       <c r="AA217" s="6" t="n"/>
+      <c r="AB217" s="6" t="n"/>
+      <c r="AC217" s="6" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="3" t="n"/>
@@ -7094,8 +7548,8 @@
       <c r="J218" s="3" t="n"/>
       <c r="K218" s="3" t="n"/>
       <c r="L218" s="3" t="n"/>
-      <c r="M218" s="5" t="n"/>
-      <c r="N218" s="5" t="n"/>
+      <c r="M218" s="3" t="n"/>
+      <c r="N218" s="3" t="n"/>
       <c r="O218" s="5" t="n"/>
       <c r="P218" s="5" t="n"/>
       <c r="Q218" s="5" t="n"/>
@@ -7109,6 +7563,8 @@
       <c r="Y218" s="5" t="n"/>
       <c r="Z218" s="5" t="n"/>
       <c r="AA218" s="5" t="n"/>
+      <c r="AB218" s="5" t="n"/>
+      <c r="AC218" s="5" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="6" t="n"/>
@@ -7138,6 +7594,8 @@
       <c r="Y219" s="6" t="n"/>
       <c r="Z219" s="6" t="n"/>
       <c r="AA219" s="6" t="n"/>
+      <c r="AB219" s="6" t="n"/>
+      <c r="AC219" s="6" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="3" t="n"/>
@@ -7152,8 +7610,8 @@
       <c r="J220" s="3" t="n"/>
       <c r="K220" s="3" t="n"/>
       <c r="L220" s="3" t="n"/>
-      <c r="M220" s="5" t="n"/>
-      <c r="N220" s="5" t="n"/>
+      <c r="M220" s="3" t="n"/>
+      <c r="N220" s="3" t="n"/>
       <c r="O220" s="5" t="n"/>
       <c r="P220" s="5" t="n"/>
       <c r="Q220" s="5" t="n"/>
@@ -7167,6 +7625,8 @@
       <c r="Y220" s="5" t="n"/>
       <c r="Z220" s="5" t="n"/>
       <c r="AA220" s="5" t="n"/>
+      <c r="AB220" s="5" t="n"/>
+      <c r="AC220" s="5" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="6" t="n"/>
@@ -7196,6 +7656,8 @@
       <c r="Y221" s="6" t="n"/>
       <c r="Z221" s="6" t="n"/>
       <c r="AA221" s="6" t="n"/>
+      <c r="AB221" s="6" t="n"/>
+      <c r="AC221" s="6" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="3" t="n"/>
@@ -7210,8 +7672,8 @@
       <c r="J222" s="3" t="n"/>
       <c r="K222" s="3" t="n"/>
       <c r="L222" s="3" t="n"/>
-      <c r="M222" s="5" t="n"/>
-      <c r="N222" s="5" t="n"/>
+      <c r="M222" s="3" t="n"/>
+      <c r="N222" s="3" t="n"/>
       <c r="O222" s="5" t="n"/>
       <c r="P222" s="5" t="n"/>
       <c r="Q222" s="5" t="n"/>
@@ -7225,6 +7687,8 @@
       <c r="Y222" s="5" t="n"/>
       <c r="Z222" s="5" t="n"/>
       <c r="AA222" s="5" t="n"/>
+      <c r="AB222" s="5" t="n"/>
+      <c r="AC222" s="5" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="6" t="n"/>
@@ -7254,6 +7718,8 @@
       <c r="Y223" s="6" t="n"/>
       <c r="Z223" s="6" t="n"/>
       <c r="AA223" s="6" t="n"/>
+      <c r="AB223" s="6" t="n"/>
+      <c r="AC223" s="6" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="3" t="n"/>
@@ -7268,8 +7734,8 @@
       <c r="J224" s="3" t="n"/>
       <c r="K224" s="3" t="n"/>
       <c r="L224" s="3" t="n"/>
-      <c r="M224" s="5" t="n"/>
-      <c r="N224" s="5" t="n"/>
+      <c r="M224" s="3" t="n"/>
+      <c r="N224" s="3" t="n"/>
       <c r="O224" s="5" t="n"/>
       <c r="P224" s="5" t="n"/>
       <c r="Q224" s="5" t="n"/>
@@ -7283,6 +7749,8 @@
       <c r="Y224" s="5" t="n"/>
       <c r="Z224" s="5" t="n"/>
       <c r="AA224" s="5" t="n"/>
+      <c r="AB224" s="5" t="n"/>
+      <c r="AC224" s="5" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="6" t="n"/>
@@ -7312,6 +7780,8 @@
       <c r="Y225" s="6" t="n"/>
       <c r="Z225" s="6" t="n"/>
       <c r="AA225" s="6" t="n"/>
+      <c r="AB225" s="6" t="n"/>
+      <c r="AC225" s="6" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="3" t="n"/>
@@ -7326,8 +7796,8 @@
       <c r="J226" s="3" t="n"/>
       <c r="K226" s="3" t="n"/>
       <c r="L226" s="3" t="n"/>
-      <c r="M226" s="5" t="n"/>
-      <c r="N226" s="5" t="n"/>
+      <c r="M226" s="3" t="n"/>
+      <c r="N226" s="3" t="n"/>
       <c r="O226" s="5" t="n"/>
       <c r="P226" s="5" t="n"/>
       <c r="Q226" s="5" t="n"/>
@@ -7341,6 +7811,8 @@
       <c r="Y226" s="5" t="n"/>
       <c r="Z226" s="5" t="n"/>
       <c r="AA226" s="5" t="n"/>
+      <c r="AB226" s="5" t="n"/>
+      <c r="AC226" s="5" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="6" t="n"/>
@@ -7370,6 +7842,8 @@
       <c r="Y227" s="6" t="n"/>
       <c r="Z227" s="6" t="n"/>
       <c r="AA227" s="6" t="n"/>
+      <c r="AB227" s="6" t="n"/>
+      <c r="AC227" s="6" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="3" t="n"/>
@@ -7384,8 +7858,8 @@
       <c r="J228" s="3" t="n"/>
       <c r="K228" s="3" t="n"/>
       <c r="L228" s="3" t="n"/>
-      <c r="M228" s="5" t="n"/>
-      <c r="N228" s="5" t="n"/>
+      <c r="M228" s="3" t="n"/>
+      <c r="N228" s="3" t="n"/>
       <c r="O228" s="5" t="n"/>
       <c r="P228" s="5" t="n"/>
       <c r="Q228" s="5" t="n"/>
@@ -7399,6 +7873,8 @@
       <c r="Y228" s="5" t="n"/>
       <c r="Z228" s="5" t="n"/>
       <c r="AA228" s="5" t="n"/>
+      <c r="AB228" s="5" t="n"/>
+      <c r="AC228" s="5" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="6" t="n"/>
@@ -7428,6 +7904,8 @@
       <c r="Y229" s="6" t="n"/>
       <c r="Z229" s="6" t="n"/>
       <c r="AA229" s="6" t="n"/>
+      <c r="AB229" s="6" t="n"/>
+      <c r="AC229" s="6" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="3" t="n"/>
@@ -7442,8 +7920,8 @@
       <c r="J230" s="3" t="n"/>
       <c r="K230" s="3" t="n"/>
       <c r="L230" s="3" t="n"/>
-      <c r="M230" s="5" t="n"/>
-      <c r="N230" s="5" t="n"/>
+      <c r="M230" s="3" t="n"/>
+      <c r="N230" s="3" t="n"/>
       <c r="O230" s="5" t="n"/>
       <c r="P230" s="5" t="n"/>
       <c r="Q230" s="5" t="n"/>
@@ -7457,6 +7935,8 @@
       <c r="Y230" s="5" t="n"/>
       <c r="Z230" s="5" t="n"/>
       <c r="AA230" s="5" t="n"/>
+      <c r="AB230" s="5" t="n"/>
+      <c r="AC230" s="5" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="6" t="n"/>
@@ -7486,6 +7966,8 @@
       <c r="Y231" s="6" t="n"/>
       <c r="Z231" s="6" t="n"/>
       <c r="AA231" s="6" t="n"/>
+      <c r="AB231" s="6" t="n"/>
+      <c r="AC231" s="6" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="3" t="n"/>
@@ -7500,8 +7982,8 @@
       <c r="J232" s="3" t="n"/>
       <c r="K232" s="3" t="n"/>
       <c r="L232" s="3" t="n"/>
-      <c r="M232" s="5" t="n"/>
-      <c r="N232" s="5" t="n"/>
+      <c r="M232" s="3" t="n"/>
+      <c r="N232" s="3" t="n"/>
       <c r="O232" s="5" t="n"/>
       <c r="P232" s="5" t="n"/>
       <c r="Q232" s="5" t="n"/>
@@ -7515,6 +7997,8 @@
       <c r="Y232" s="5" t="n"/>
       <c r="Z232" s="5" t="n"/>
       <c r="AA232" s="5" t="n"/>
+      <c r="AB232" s="5" t="n"/>
+      <c r="AC232" s="5" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="6" t="n"/>
@@ -7544,6 +8028,8 @@
       <c r="Y233" s="6" t="n"/>
       <c r="Z233" s="6" t="n"/>
       <c r="AA233" s="6" t="n"/>
+      <c r="AB233" s="6" t="n"/>
+      <c r="AC233" s="6" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="3" t="n"/>
@@ -7558,8 +8044,8 @@
       <c r="J234" s="3" t="n"/>
       <c r="K234" s="3" t="n"/>
       <c r="L234" s="3" t="n"/>
-      <c r="M234" s="5" t="n"/>
-      <c r="N234" s="5" t="n"/>
+      <c r="M234" s="3" t="n"/>
+      <c r="N234" s="3" t="n"/>
       <c r="O234" s="5" t="n"/>
       <c r="P234" s="5" t="n"/>
       <c r="Q234" s="5" t="n"/>
@@ -7573,6 +8059,8 @@
       <c r="Y234" s="5" t="n"/>
       <c r="Z234" s="5" t="n"/>
       <c r="AA234" s="5" t="n"/>
+      <c r="AB234" s="5" t="n"/>
+      <c r="AC234" s="5" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="6" t="n"/>
@@ -7602,6 +8090,8 @@
       <c r="Y235" s="6" t="n"/>
       <c r="Z235" s="6" t="n"/>
       <c r="AA235" s="6" t="n"/>
+      <c r="AB235" s="6" t="n"/>
+      <c r="AC235" s="6" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="3" t="n"/>
@@ -7616,8 +8106,8 @@
       <c r="J236" s="3" t="n"/>
       <c r="K236" s="3" t="n"/>
       <c r="L236" s="3" t="n"/>
-      <c r="M236" s="5" t="n"/>
-      <c r="N236" s="5" t="n"/>
+      <c r="M236" s="3" t="n"/>
+      <c r="N236" s="3" t="n"/>
       <c r="O236" s="5" t="n"/>
       <c r="P236" s="5" t="n"/>
       <c r="Q236" s="5" t="n"/>
@@ -7631,6 +8121,8 @@
       <c r="Y236" s="5" t="n"/>
       <c r="Z236" s="5" t="n"/>
       <c r="AA236" s="5" t="n"/>
+      <c r="AB236" s="5" t="n"/>
+      <c r="AC236" s="5" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="6" t="n"/>
@@ -7660,6 +8152,8 @@
       <c r="Y237" s="6" t="n"/>
       <c r="Z237" s="6" t="n"/>
       <c r="AA237" s="6" t="n"/>
+      <c r="AB237" s="6" t="n"/>
+      <c r="AC237" s="6" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="3" t="n"/>
@@ -7674,8 +8168,8 @@
       <c r="J238" s="3" t="n"/>
       <c r="K238" s="3" t="n"/>
       <c r="L238" s="3" t="n"/>
-      <c r="M238" s="5" t="n"/>
-      <c r="N238" s="5" t="n"/>
+      <c r="M238" s="3" t="n"/>
+      <c r="N238" s="3" t="n"/>
       <c r="O238" s="5" t="n"/>
       <c r="P238" s="5" t="n"/>
       <c r="Q238" s="5" t="n"/>
@@ -7689,6 +8183,8 @@
       <c r="Y238" s="5" t="n"/>
       <c r="Z238" s="5" t="n"/>
       <c r="AA238" s="5" t="n"/>
+      <c r="AB238" s="5" t="n"/>
+      <c r="AC238" s="5" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="6" t="n"/>
@@ -7718,6 +8214,8 @@
       <c r="Y239" s="6" t="n"/>
       <c r="Z239" s="6" t="n"/>
       <c r="AA239" s="6" t="n"/>
+      <c r="AB239" s="6" t="n"/>
+      <c r="AC239" s="6" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="3" t="n"/>
@@ -7732,8 +8230,8 @@
       <c r="J240" s="3" t="n"/>
       <c r="K240" s="3" t="n"/>
       <c r="L240" s="3" t="n"/>
-      <c r="M240" s="5" t="n"/>
-      <c r="N240" s="5" t="n"/>
+      <c r="M240" s="3" t="n"/>
+      <c r="N240" s="3" t="n"/>
       <c r="O240" s="5" t="n"/>
       <c r="P240" s="5" t="n"/>
       <c r="Q240" s="5" t="n"/>
@@ -7747,6 +8245,8 @@
       <c r="Y240" s="5" t="n"/>
       <c r="Z240" s="5" t="n"/>
       <c r="AA240" s="5" t="n"/>
+      <c r="AB240" s="5" t="n"/>
+      <c r="AC240" s="5" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="6" t="n"/>
@@ -7776,6 +8276,8 @@
       <c r="Y241" s="6" t="n"/>
       <c r="Z241" s="6" t="n"/>
       <c r="AA241" s="6" t="n"/>
+      <c r="AB241" s="6" t="n"/>
+      <c r="AC241" s="6" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="3" t="n"/>
@@ -7790,8 +8292,8 @@
       <c r="J242" s="3" t="n"/>
       <c r="K242" s="3" t="n"/>
       <c r="L242" s="3" t="n"/>
-      <c r="M242" s="5" t="n"/>
-      <c r="N242" s="5" t="n"/>
+      <c r="M242" s="3" t="n"/>
+      <c r="N242" s="3" t="n"/>
       <c r="O242" s="5" t="n"/>
       <c r="P242" s="5" t="n"/>
       <c r="Q242" s="5" t="n"/>
@@ -7805,6 +8307,8 @@
       <c r="Y242" s="5" t="n"/>
       <c r="Z242" s="5" t="n"/>
       <c r="AA242" s="5" t="n"/>
+      <c r="AB242" s="5" t="n"/>
+      <c r="AC242" s="5" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="6" t="n"/>
@@ -7834,6 +8338,8 @@
       <c r="Y243" s="6" t="n"/>
       <c r="Z243" s="6" t="n"/>
       <c r="AA243" s="6" t="n"/>
+      <c r="AB243" s="6" t="n"/>
+      <c r="AC243" s="6" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="3" t="n"/>
@@ -7848,8 +8354,8 @@
       <c r="J244" s="3" t="n"/>
       <c r="K244" s="3" t="n"/>
       <c r="L244" s="3" t="n"/>
-      <c r="M244" s="5" t="n"/>
-      <c r="N244" s="5" t="n"/>
+      <c r="M244" s="3" t="n"/>
+      <c r="N244" s="3" t="n"/>
       <c r="O244" s="5" t="n"/>
       <c r="P244" s="5" t="n"/>
       <c r="Q244" s="5" t="n"/>
@@ -7863,6 +8369,8 @@
       <c r="Y244" s="5" t="n"/>
       <c r="Z244" s="5" t="n"/>
       <c r="AA244" s="5" t="n"/>
+      <c r="AB244" s="5" t="n"/>
+      <c r="AC244" s="5" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="6" t="n"/>
@@ -7892,6 +8400,8 @@
       <c r="Y245" s="6" t="n"/>
       <c r="Z245" s="6" t="n"/>
       <c r="AA245" s="6" t="n"/>
+      <c r="AB245" s="6" t="n"/>
+      <c r="AC245" s="6" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="3" t="n"/>
@@ -7906,8 +8416,8 @@
       <c r="J246" s="3" t="n"/>
       <c r="K246" s="3" t="n"/>
       <c r="L246" s="3" t="n"/>
-      <c r="M246" s="5" t="n"/>
-      <c r="N246" s="5" t="n"/>
+      <c r="M246" s="3" t="n"/>
+      <c r="N246" s="3" t="n"/>
       <c r="O246" s="5" t="n"/>
       <c r="P246" s="5" t="n"/>
       <c r="Q246" s="5" t="n"/>
@@ -7921,6 +8431,8 @@
       <c r="Y246" s="5" t="n"/>
       <c r="Z246" s="5" t="n"/>
       <c r="AA246" s="5" t="n"/>
+      <c r="AB246" s="5" t="n"/>
+      <c r="AC246" s="5" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="6" t="n"/>
@@ -7950,6 +8462,8 @@
       <c r="Y247" s="6" t="n"/>
       <c r="Z247" s="6" t="n"/>
       <c r="AA247" s="6" t="n"/>
+      <c r="AB247" s="6" t="n"/>
+      <c r="AC247" s="6" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="3" t="n"/>
@@ -7964,8 +8478,8 @@
       <c r="J248" s="3" t="n"/>
       <c r="K248" s="3" t="n"/>
       <c r="L248" s="3" t="n"/>
-      <c r="M248" s="5" t="n"/>
-      <c r="N248" s="5" t="n"/>
+      <c r="M248" s="3" t="n"/>
+      <c r="N248" s="3" t="n"/>
       <c r="O248" s="5" t="n"/>
       <c r="P248" s="5" t="n"/>
       <c r="Q248" s="5" t="n"/>
@@ -7979,6 +8493,8 @@
       <c r="Y248" s="5" t="n"/>
       <c r="Z248" s="5" t="n"/>
       <c r="AA248" s="5" t="n"/>
+      <c r="AB248" s="5" t="n"/>
+      <c r="AC248" s="5" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="6" t="n"/>
@@ -8008,6 +8524,8 @@
       <c r="Y249" s="6" t="n"/>
       <c r="Z249" s="6" t="n"/>
       <c r="AA249" s="6" t="n"/>
+      <c r="AB249" s="6" t="n"/>
+      <c r="AC249" s="6" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="3" t="n"/>
@@ -8022,8 +8540,8 @@
       <c r="J250" s="3" t="n"/>
       <c r="K250" s="3" t="n"/>
       <c r="L250" s="3" t="n"/>
-      <c r="M250" s="5" t="n"/>
-      <c r="N250" s="5" t="n"/>
+      <c r="M250" s="3" t="n"/>
+      <c r="N250" s="3" t="n"/>
       <c r="O250" s="5" t="n"/>
       <c r="P250" s="5" t="n"/>
       <c r="Q250" s="5" t="n"/>
@@ -8037,6 +8555,8 @@
       <c r="Y250" s="5" t="n"/>
       <c r="Z250" s="5" t="n"/>
       <c r="AA250" s="5" t="n"/>
+      <c r="AB250" s="5" t="n"/>
+      <c r="AC250" s="5" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="6" t="n"/>
@@ -8066,6 +8586,8 @@
       <c r="Y251" s="6" t="n"/>
       <c r="Z251" s="6" t="n"/>
       <c r="AA251" s="6" t="n"/>
+      <c r="AB251" s="6" t="n"/>
+      <c r="AC251" s="6" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="3" t="n"/>
@@ -8080,8 +8602,8 @@
       <c r="J252" s="3" t="n"/>
       <c r="K252" s="3" t="n"/>
       <c r="L252" s="3" t="n"/>
-      <c r="M252" s="5" t="n"/>
-      <c r="N252" s="5" t="n"/>
+      <c r="M252" s="3" t="n"/>
+      <c r="N252" s="3" t="n"/>
       <c r="O252" s="5" t="n"/>
       <c r="P252" s="5" t="n"/>
       <c r="Q252" s="5" t="n"/>
@@ -8095,6 +8617,8 @@
       <c r="Y252" s="5" t="n"/>
       <c r="Z252" s="5" t="n"/>
       <c r="AA252" s="5" t="n"/>
+      <c r="AB252" s="5" t="n"/>
+      <c r="AC252" s="5" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="6" t="n"/>
@@ -8124,6 +8648,8 @@
       <c r="Y253" s="6" t="n"/>
       <c r="Z253" s="6" t="n"/>
       <c r="AA253" s="6" t="n"/>
+      <c r="AB253" s="6" t="n"/>
+      <c r="AC253" s="6" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="3" t="n"/>
@@ -8138,8 +8664,8 @@
       <c r="J254" s="3" t="n"/>
       <c r="K254" s="3" t="n"/>
       <c r="L254" s="3" t="n"/>
-      <c r="M254" s="5" t="n"/>
-      <c r="N254" s="5" t="n"/>
+      <c r="M254" s="3" t="n"/>
+      <c r="N254" s="3" t="n"/>
       <c r="O254" s="5" t="n"/>
       <c r="P254" s="5" t="n"/>
       <c r="Q254" s="5" t="n"/>
@@ -8153,6 +8679,8 @@
       <c r="Y254" s="5" t="n"/>
       <c r="Z254" s="5" t="n"/>
       <c r="AA254" s="5" t="n"/>
+      <c r="AB254" s="5" t="n"/>
+      <c r="AC254" s="5" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="6" t="n"/>
@@ -8182,6 +8710,8 @@
       <c r="Y255" s="6" t="n"/>
       <c r="Z255" s="6" t="n"/>
       <c r="AA255" s="6" t="n"/>
+      <c r="AB255" s="6" t="n"/>
+      <c r="AC255" s="6" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="3" t="n"/>
@@ -8196,8 +8726,8 @@
       <c r="J256" s="3" t="n"/>
       <c r="K256" s="3" t="n"/>
       <c r="L256" s="3" t="n"/>
-      <c r="M256" s="5" t="n"/>
-      <c r="N256" s="5" t="n"/>
+      <c r="M256" s="3" t="n"/>
+      <c r="N256" s="3" t="n"/>
       <c r="O256" s="5" t="n"/>
       <c r="P256" s="5" t="n"/>
       <c r="Q256" s="5" t="n"/>
@@ -8211,6 +8741,8 @@
       <c r="Y256" s="5" t="n"/>
       <c r="Z256" s="5" t="n"/>
       <c r="AA256" s="5" t="n"/>
+      <c r="AB256" s="5" t="n"/>
+      <c r="AC256" s="5" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="6" t="n"/>
@@ -8240,6 +8772,8 @@
       <c r="Y257" s="6" t="n"/>
       <c r="Z257" s="6" t="n"/>
       <c r="AA257" s="6" t="n"/>
+      <c r="AB257" s="6" t="n"/>
+      <c r="AC257" s="6" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="3" t="n"/>
@@ -8254,8 +8788,8 @@
       <c r="J258" s="3" t="n"/>
       <c r="K258" s="3" t="n"/>
       <c r="L258" s="3" t="n"/>
-      <c r="M258" s="5" t="n"/>
-      <c r="N258" s="5" t="n"/>
+      <c r="M258" s="3" t="n"/>
+      <c r="N258" s="3" t="n"/>
       <c r="O258" s="5" t="n"/>
       <c r="P258" s="5" t="n"/>
       <c r="Q258" s="5" t="n"/>
@@ -8269,6 +8803,8 @@
       <c r="Y258" s="5" t="n"/>
       <c r="Z258" s="5" t="n"/>
       <c r="AA258" s="5" t="n"/>
+      <c r="AB258" s="5" t="n"/>
+      <c r="AC258" s="5" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="6" t="n"/>
@@ -8298,6 +8834,8 @@
       <c r="Y259" s="6" t="n"/>
       <c r="Z259" s="6" t="n"/>
       <c r="AA259" s="6" t="n"/>
+      <c r="AB259" s="6" t="n"/>
+      <c r="AC259" s="6" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="3" t="n"/>
@@ -8312,8 +8850,8 @@
       <c r="J260" s="3" t="n"/>
       <c r="K260" s="3" t="n"/>
       <c r="L260" s="3" t="n"/>
-      <c r="M260" s="5" t="n"/>
-      <c r="N260" s="5" t="n"/>
+      <c r="M260" s="3" t="n"/>
+      <c r="N260" s="3" t="n"/>
       <c r="O260" s="5" t="n"/>
       <c r="P260" s="5" t="n"/>
       <c r="Q260" s="5" t="n"/>
@@ -8327,6 +8865,8 @@
       <c r="Y260" s="5" t="n"/>
       <c r="Z260" s="5" t="n"/>
       <c r="AA260" s="5" t="n"/>
+      <c r="AB260" s="5" t="n"/>
+      <c r="AC260" s="5" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="6" t="n"/>
@@ -8356,6 +8896,8 @@
       <c r="Y261" s="6" t="n"/>
       <c r="Z261" s="6" t="n"/>
       <c r="AA261" s="6" t="n"/>
+      <c r="AB261" s="6" t="n"/>
+      <c r="AC261" s="6" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="3" t="n"/>
@@ -8370,8 +8912,8 @@
       <c r="J262" s="3" t="n"/>
       <c r="K262" s="3" t="n"/>
       <c r="L262" s="3" t="n"/>
-      <c r="M262" s="5" t="n"/>
-      <c r="N262" s="5" t="n"/>
+      <c r="M262" s="3" t="n"/>
+      <c r="N262" s="3" t="n"/>
       <c r="O262" s="5" t="n"/>
       <c r="P262" s="5" t="n"/>
       <c r="Q262" s="5" t="n"/>
@@ -8385,6 +8927,8 @@
       <c r="Y262" s="5" t="n"/>
       <c r="Z262" s="5" t="n"/>
       <c r="AA262" s="5" t="n"/>
+      <c r="AB262" s="5" t="n"/>
+      <c r="AC262" s="5" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="6" t="n"/>
@@ -8414,6 +8958,8 @@
       <c r="Y263" s="6" t="n"/>
       <c r="Z263" s="6" t="n"/>
       <c r="AA263" s="6" t="n"/>
+      <c r="AB263" s="6" t="n"/>
+      <c r="AC263" s="6" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="3" t="n"/>
@@ -8428,8 +8974,8 @@
       <c r="J264" s="3" t="n"/>
       <c r="K264" s="3" t="n"/>
       <c r="L264" s="3" t="n"/>
-      <c r="M264" s="5" t="n"/>
-      <c r="N264" s="5" t="n"/>
+      <c r="M264" s="3" t="n"/>
+      <c r="N264" s="3" t="n"/>
       <c r="O264" s="5" t="n"/>
       <c r="P264" s="5" t="n"/>
       <c r="Q264" s="5" t="n"/>
@@ -8443,6 +8989,8 @@
       <c r="Y264" s="5" t="n"/>
       <c r="Z264" s="5" t="n"/>
       <c r="AA264" s="5" t="n"/>
+      <c r="AB264" s="5" t="n"/>
+      <c r="AC264" s="5" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="6" t="n"/>
@@ -8472,6 +9020,8 @@
       <c r="Y265" s="6" t="n"/>
       <c r="Z265" s="6" t="n"/>
       <c r="AA265" s="6" t="n"/>
+      <c r="AB265" s="6" t="n"/>
+      <c r="AC265" s="6" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="3" t="n"/>
@@ -8486,8 +9036,8 @@
       <c r="J266" s="3" t="n"/>
       <c r="K266" s="3" t="n"/>
       <c r="L266" s="3" t="n"/>
-      <c r="M266" s="5" t="n"/>
-      <c r="N266" s="5" t="n"/>
+      <c r="M266" s="3" t="n"/>
+      <c r="N266" s="3" t="n"/>
       <c r="O266" s="5" t="n"/>
       <c r="P266" s="5" t="n"/>
       <c r="Q266" s="5" t="n"/>
@@ -8501,6 +9051,8 @@
       <c r="Y266" s="5" t="n"/>
       <c r="Z266" s="5" t="n"/>
       <c r="AA266" s="5" t="n"/>
+      <c r="AB266" s="5" t="n"/>
+      <c r="AC266" s="5" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="6" t="n"/>
@@ -8530,6 +9082,8 @@
       <c r="Y267" s="6" t="n"/>
       <c r="Z267" s="6" t="n"/>
       <c r="AA267" s="6" t="n"/>
+      <c r="AB267" s="6" t="n"/>
+      <c r="AC267" s="6" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="3" t="n"/>
@@ -8544,8 +9098,8 @@
       <c r="J268" s="3" t="n"/>
       <c r="K268" s="3" t="n"/>
       <c r="L268" s="3" t="n"/>
-      <c r="M268" s="5" t="n"/>
-      <c r="N268" s="5" t="n"/>
+      <c r="M268" s="3" t="n"/>
+      <c r="N268" s="3" t="n"/>
       <c r="O268" s="5" t="n"/>
       <c r="P268" s="5" t="n"/>
       <c r="Q268" s="5" t="n"/>
@@ -8559,6 +9113,8 @@
       <c r="Y268" s="5" t="n"/>
       <c r="Z268" s="5" t="n"/>
       <c r="AA268" s="5" t="n"/>
+      <c r="AB268" s="5" t="n"/>
+      <c r="AC268" s="5" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="6" t="n"/>
@@ -8588,6 +9144,8 @@
       <c r="Y269" s="6" t="n"/>
       <c r="Z269" s="6" t="n"/>
       <c r="AA269" s="6" t="n"/>
+      <c r="AB269" s="6" t="n"/>
+      <c r="AC269" s="6" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="3" t="n"/>
@@ -8602,8 +9160,8 @@
       <c r="J270" s="3" t="n"/>
       <c r="K270" s="3" t="n"/>
       <c r="L270" s="3" t="n"/>
-      <c r="M270" s="5" t="n"/>
-      <c r="N270" s="5" t="n"/>
+      <c r="M270" s="3" t="n"/>
+      <c r="N270" s="3" t="n"/>
       <c r="O270" s="5" t="n"/>
       <c r="P270" s="5" t="n"/>
       <c r="Q270" s="5" t="n"/>
@@ -8617,6 +9175,8 @@
       <c r="Y270" s="5" t="n"/>
       <c r="Z270" s="5" t="n"/>
       <c r="AA270" s="5" t="n"/>
+      <c r="AB270" s="5" t="n"/>
+      <c r="AC270" s="5" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="6" t="n"/>
@@ -8646,6 +9206,8 @@
       <c r="Y271" s="6" t="n"/>
       <c r="Z271" s="6" t="n"/>
       <c r="AA271" s="6" t="n"/>
+      <c r="AB271" s="6" t="n"/>
+      <c r="AC271" s="6" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="3" t="n"/>
@@ -8660,8 +9222,8 @@
       <c r="J272" s="3" t="n"/>
       <c r="K272" s="3" t="n"/>
       <c r="L272" s="3" t="n"/>
-      <c r="M272" s="5" t="n"/>
-      <c r="N272" s="5" t="n"/>
+      <c r="M272" s="3" t="n"/>
+      <c r="N272" s="3" t="n"/>
       <c r="O272" s="5" t="n"/>
       <c r="P272" s="5" t="n"/>
       <c r="Q272" s="5" t="n"/>
@@ -8675,6 +9237,8 @@
       <c r="Y272" s="5" t="n"/>
       <c r="Z272" s="5" t="n"/>
       <c r="AA272" s="5" t="n"/>
+      <c r="AB272" s="5" t="n"/>
+      <c r="AC272" s="5" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="6" t="n"/>
@@ -8704,6 +9268,8 @@
       <c r="Y273" s="6" t="n"/>
       <c r="Z273" s="6" t="n"/>
       <c r="AA273" s="6" t="n"/>
+      <c r="AB273" s="6" t="n"/>
+      <c r="AC273" s="6" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="3" t="n"/>
@@ -8718,8 +9284,8 @@
       <c r="J274" s="3" t="n"/>
       <c r="K274" s="3" t="n"/>
       <c r="L274" s="3" t="n"/>
-      <c r="M274" s="5" t="n"/>
-      <c r="N274" s="5" t="n"/>
+      <c r="M274" s="3" t="n"/>
+      <c r="N274" s="3" t="n"/>
       <c r="O274" s="5" t="n"/>
       <c r="P274" s="5" t="n"/>
       <c r="Q274" s="5" t="n"/>
@@ -8733,6 +9299,8 @@
       <c r="Y274" s="5" t="n"/>
       <c r="Z274" s="5" t="n"/>
       <c r="AA274" s="5" t="n"/>
+      <c r="AB274" s="5" t="n"/>
+      <c r="AC274" s="5" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="6" t="n"/>
@@ -8762,6 +9330,8 @@
       <c r="Y275" s="6" t="n"/>
       <c r="Z275" s="6" t="n"/>
       <c r="AA275" s="6" t="n"/>
+      <c r="AB275" s="6" t="n"/>
+      <c r="AC275" s="6" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="3" t="n"/>
@@ -8776,8 +9346,8 @@
       <c r="J276" s="3" t="n"/>
       <c r="K276" s="3" t="n"/>
       <c r="L276" s="3" t="n"/>
-      <c r="M276" s="5" t="n"/>
-      <c r="N276" s="5" t="n"/>
+      <c r="M276" s="3" t="n"/>
+      <c r="N276" s="3" t="n"/>
       <c r="O276" s="5" t="n"/>
       <c r="P276" s="5" t="n"/>
       <c r="Q276" s="5" t="n"/>
@@ -8791,6 +9361,8 @@
       <c r="Y276" s="5" t="n"/>
       <c r="Z276" s="5" t="n"/>
       <c r="AA276" s="5" t="n"/>
+      <c r="AB276" s="5" t="n"/>
+      <c r="AC276" s="5" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="6" t="n"/>
@@ -8820,6 +9392,8 @@
       <c r="Y277" s="6" t="n"/>
       <c r="Z277" s="6" t="n"/>
       <c r="AA277" s="6" t="n"/>
+      <c r="AB277" s="6" t="n"/>
+      <c r="AC277" s="6" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="3" t="n"/>
@@ -8834,8 +9408,8 @@
       <c r="J278" s="3" t="n"/>
       <c r="K278" s="3" t="n"/>
       <c r="L278" s="3" t="n"/>
-      <c r="M278" s="5" t="n"/>
-      <c r="N278" s="5" t="n"/>
+      <c r="M278" s="3" t="n"/>
+      <c r="N278" s="3" t="n"/>
       <c r="O278" s="5" t="n"/>
       <c r="P278" s="5" t="n"/>
       <c r="Q278" s="5" t="n"/>
@@ -8849,6 +9423,8 @@
       <c r="Y278" s="5" t="n"/>
       <c r="Z278" s="5" t="n"/>
       <c r="AA278" s="5" t="n"/>
+      <c r="AB278" s="5" t="n"/>
+      <c r="AC278" s="5" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="6" t="n"/>
@@ -8878,6 +9454,8 @@
       <c r="Y279" s="6" t="n"/>
       <c r="Z279" s="6" t="n"/>
       <c r="AA279" s="6" t="n"/>
+      <c r="AB279" s="6" t="n"/>
+      <c r="AC279" s="6" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="3" t="n"/>
@@ -8892,8 +9470,8 @@
       <c r="J280" s="3" t="n"/>
       <c r="K280" s="3" t="n"/>
       <c r="L280" s="3" t="n"/>
-      <c r="M280" s="5" t="n"/>
-      <c r="N280" s="5" t="n"/>
+      <c r="M280" s="3" t="n"/>
+      <c r="N280" s="3" t="n"/>
       <c r="O280" s="5" t="n"/>
       <c r="P280" s="5" t="n"/>
       <c r="Q280" s="5" t="n"/>
@@ -8907,6 +9485,8 @@
       <c r="Y280" s="5" t="n"/>
       <c r="Z280" s="5" t="n"/>
       <c r="AA280" s="5" t="n"/>
+      <c r="AB280" s="5" t="n"/>
+      <c r="AC280" s="5" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="6" t="n"/>
@@ -8936,6 +9516,8 @@
       <c r="Y281" s="6" t="n"/>
       <c r="Z281" s="6" t="n"/>
       <c r="AA281" s="6" t="n"/>
+      <c r="AB281" s="6" t="n"/>
+      <c r="AC281" s="6" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="3" t="n"/>
@@ -8950,8 +9532,8 @@
       <c r="J282" s="3" t="n"/>
       <c r="K282" s="3" t="n"/>
       <c r="L282" s="3" t="n"/>
-      <c r="M282" s="5" t="n"/>
-      <c r="N282" s="5" t="n"/>
+      <c r="M282" s="3" t="n"/>
+      <c r="N282" s="3" t="n"/>
       <c r="O282" s="5" t="n"/>
       <c r="P282" s="5" t="n"/>
       <c r="Q282" s="5" t="n"/>
@@ -8965,6 +9547,8 @@
       <c r="Y282" s="5" t="n"/>
       <c r="Z282" s="5" t="n"/>
       <c r="AA282" s="5" t="n"/>
+      <c r="AB282" s="5" t="n"/>
+      <c r="AC282" s="5" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="6" t="n"/>
@@ -8994,6 +9578,8 @@
       <c r="Y283" s="6" t="n"/>
       <c r="Z283" s="6" t="n"/>
       <c r="AA283" s="6" t="n"/>
+      <c r="AB283" s="6" t="n"/>
+      <c r="AC283" s="6" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="3" t="n"/>
@@ -9008,8 +9594,8 @@
       <c r="J284" s="3" t="n"/>
       <c r="K284" s="3" t="n"/>
       <c r="L284" s="3" t="n"/>
-      <c r="M284" s="5" t="n"/>
-      <c r="N284" s="5" t="n"/>
+      <c r="M284" s="3" t="n"/>
+      <c r="N284" s="3" t="n"/>
       <c r="O284" s="5" t="n"/>
       <c r="P284" s="5" t="n"/>
       <c r="Q284" s="5" t="n"/>
@@ -9023,6 +9609,8 @@
       <c r="Y284" s="5" t="n"/>
       <c r="Z284" s="5" t="n"/>
       <c r="AA284" s="5" t="n"/>
+      <c r="AB284" s="5" t="n"/>
+      <c r="AC284" s="5" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="6" t="n"/>
@@ -9052,6 +9640,8 @@
       <c r="Y285" s="6" t="n"/>
       <c r="Z285" s="6" t="n"/>
       <c r="AA285" s="6" t="n"/>
+      <c r="AB285" s="6" t="n"/>
+      <c r="AC285" s="6" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="3" t="n"/>
@@ -9066,8 +9656,8 @@
       <c r="J286" s="3" t="n"/>
       <c r="K286" s="3" t="n"/>
       <c r="L286" s="3" t="n"/>
-      <c r="M286" s="5" t="n"/>
-      <c r="N286" s="5" t="n"/>
+      <c r="M286" s="3" t="n"/>
+      <c r="N286" s="3" t="n"/>
       <c r="O286" s="5" t="n"/>
       <c r="P286" s="5" t="n"/>
       <c r="Q286" s="5" t="n"/>
@@ -9081,6 +9671,8 @@
       <c r="Y286" s="5" t="n"/>
       <c r="Z286" s="5" t="n"/>
       <c r="AA286" s="5" t="n"/>
+      <c r="AB286" s="5" t="n"/>
+      <c r="AC286" s="5" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="6" t="n"/>
@@ -9110,6 +9702,8 @@
       <c r="Y287" s="6" t="n"/>
       <c r="Z287" s="6" t="n"/>
       <c r="AA287" s="6" t="n"/>
+      <c r="AB287" s="6" t="n"/>
+      <c r="AC287" s="6" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="3" t="n"/>
@@ -9124,8 +9718,8 @@
       <c r="J288" s="3" t="n"/>
       <c r="K288" s="3" t="n"/>
       <c r="L288" s="3" t="n"/>
-      <c r="M288" s="5" t="n"/>
-      <c r="N288" s="5" t="n"/>
+      <c r="M288" s="3" t="n"/>
+      <c r="N288" s="3" t="n"/>
       <c r="O288" s="5" t="n"/>
       <c r="P288" s="5" t="n"/>
       <c r="Q288" s="5" t="n"/>
@@ -9139,6 +9733,8 @@
       <c r="Y288" s="5" t="n"/>
       <c r="Z288" s="5" t="n"/>
       <c r="AA288" s="5" t="n"/>
+      <c r="AB288" s="5" t="n"/>
+      <c r="AC288" s="5" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="6" t="n"/>
@@ -9168,6 +9764,8 @@
       <c r="Y289" s="6" t="n"/>
       <c r="Z289" s="6" t="n"/>
       <c r="AA289" s="6" t="n"/>
+      <c r="AB289" s="6" t="n"/>
+      <c r="AC289" s="6" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="3" t="n"/>
@@ -9182,8 +9780,8 @@
       <c r="J290" s="3" t="n"/>
       <c r="K290" s="3" t="n"/>
       <c r="L290" s="3" t="n"/>
-      <c r="M290" s="5" t="n"/>
-      <c r="N290" s="5" t="n"/>
+      <c r="M290" s="3" t="n"/>
+      <c r="N290" s="3" t="n"/>
       <c r="O290" s="5" t="n"/>
       <c r="P290" s="5" t="n"/>
       <c r="Q290" s="5" t="n"/>
@@ -9197,6 +9795,8 @@
       <c r="Y290" s="5" t="n"/>
       <c r="Z290" s="5" t="n"/>
       <c r="AA290" s="5" t="n"/>
+      <c r="AB290" s="5" t="n"/>
+      <c r="AC290" s="5" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="6" t="n"/>
@@ -9226,6 +9826,8 @@
       <c r="Y291" s="6" t="n"/>
       <c r="Z291" s="6" t="n"/>
       <c r="AA291" s="6" t="n"/>
+      <c r="AB291" s="6" t="n"/>
+      <c r="AC291" s="6" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="3" t="n"/>
@@ -9240,8 +9842,8 @@
       <c r="J292" s="3" t="n"/>
       <c r="K292" s="3" t="n"/>
       <c r="L292" s="3" t="n"/>
-      <c r="M292" s="5" t="n"/>
-      <c r="N292" s="5" t="n"/>
+      <c r="M292" s="3" t="n"/>
+      <c r="N292" s="3" t="n"/>
       <c r="O292" s="5" t="n"/>
       <c r="P292" s="5" t="n"/>
       <c r="Q292" s="5" t="n"/>
@@ -9255,6 +9857,8 @@
       <c r="Y292" s="5" t="n"/>
       <c r="Z292" s="5" t="n"/>
       <c r="AA292" s="5" t="n"/>
+      <c r="AB292" s="5" t="n"/>
+      <c r="AC292" s="5" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="6" t="n"/>
@@ -9284,6 +9888,8 @@
       <c r="Y293" s="6" t="n"/>
       <c r="Z293" s="6" t="n"/>
       <c r="AA293" s="6" t="n"/>
+      <c r="AB293" s="6" t="n"/>
+      <c r="AC293" s="6" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="3" t="n"/>
@@ -9298,8 +9904,8 @@
       <c r="J294" s="3" t="n"/>
       <c r="K294" s="3" t="n"/>
       <c r="L294" s="3" t="n"/>
-      <c r="M294" s="5" t="n"/>
-      <c r="N294" s="5" t="n"/>
+      <c r="M294" s="3" t="n"/>
+      <c r="N294" s="3" t="n"/>
       <c r="O294" s="5" t="n"/>
       <c r="P294" s="5" t="n"/>
       <c r="Q294" s="5" t="n"/>
@@ -9313,6 +9919,8 @@
       <c r="Y294" s="5" t="n"/>
       <c r="Z294" s="5" t="n"/>
       <c r="AA294" s="5" t="n"/>
+      <c r="AB294" s="5" t="n"/>
+      <c r="AC294" s="5" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="6" t="n"/>
@@ -9342,6 +9950,8 @@
       <c r="Y295" s="6" t="n"/>
       <c r="Z295" s="6" t="n"/>
       <c r="AA295" s="6" t="n"/>
+      <c r="AB295" s="6" t="n"/>
+      <c r="AC295" s="6" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="3" t="n"/>
@@ -9356,8 +9966,8 @@
       <c r="J296" s="3" t="n"/>
       <c r="K296" s="3" t="n"/>
       <c r="L296" s="3" t="n"/>
-      <c r="M296" s="5" t="n"/>
-      <c r="N296" s="5" t="n"/>
+      <c r="M296" s="3" t="n"/>
+      <c r="N296" s="3" t="n"/>
       <c r="O296" s="5" t="n"/>
       <c r="P296" s="5" t="n"/>
       <c r="Q296" s="5" t="n"/>
@@ -9371,6 +9981,8 @@
       <c r="Y296" s="5" t="n"/>
       <c r="Z296" s="5" t="n"/>
       <c r="AA296" s="5" t="n"/>
+      <c r="AB296" s="5" t="n"/>
+      <c r="AC296" s="5" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="6" t="n"/>
@@ -9400,6 +10012,8 @@
       <c r="Y297" s="6" t="n"/>
       <c r="Z297" s="6" t="n"/>
       <c r="AA297" s="6" t="n"/>
+      <c r="AB297" s="6" t="n"/>
+      <c r="AC297" s="6" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="3" t="n"/>
@@ -9414,8 +10028,8 @@
       <c r="J298" s="3" t="n"/>
       <c r="K298" s="3" t="n"/>
       <c r="L298" s="3" t="n"/>
-      <c r="M298" s="5" t="n"/>
-      <c r="N298" s="5" t="n"/>
+      <c r="M298" s="3" t="n"/>
+      <c r="N298" s="3" t="n"/>
       <c r="O298" s="5" t="n"/>
       <c r="P298" s="5" t="n"/>
       <c r="Q298" s="5" t="n"/>
@@ -9429,6 +10043,8 @@
       <c r="Y298" s="5" t="n"/>
       <c r="Z298" s="5" t="n"/>
       <c r="AA298" s="5" t="n"/>
+      <c r="AB298" s="5" t="n"/>
+      <c r="AC298" s="5" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="6" t="n"/>
@@ -9458,6 +10074,8 @@
       <c r="Y299" s="6" t="n"/>
       <c r="Z299" s="6" t="n"/>
       <c r="AA299" s="6" t="n"/>
+      <c r="AB299" s="6" t="n"/>
+      <c r="AC299" s="6" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="3" t="n"/>
@@ -9472,8 +10090,8 @@
       <c r="J300" s="3" t="n"/>
       <c r="K300" s="3" t="n"/>
       <c r="L300" s="3" t="n"/>
-      <c r="M300" s="5" t="n"/>
-      <c r="N300" s="5" t="n"/>
+      <c r="M300" s="3" t="n"/>
+      <c r="N300" s="3" t="n"/>
       <c r="O300" s="5" t="n"/>
       <c r="P300" s="5" t="n"/>
       <c r="Q300" s="5" t="n"/>
@@ -9487,6 +10105,8 @@
       <c r="Y300" s="5" t="n"/>
       <c r="Z300" s="5" t="n"/>
       <c r="AA300" s="5" t="n"/>
+      <c r="AB300" s="5" t="n"/>
+      <c r="AC300" s="5" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="6" t="n"/>
@@ -9516,9 +10136,11 @@
       <c r="Y301" s="6" t="n"/>
       <c r="Z301" s="6" t="n"/>
       <c r="AA301" s="6" t="n"/>
+      <c r="AB301" s="6" t="n"/>
+      <c r="AC301" s="6" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="11">
+  <dataValidations count="13">
     <dataValidation sqref="B2:B301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="ذكر أو أنثى" type="list">
       <formula1>"ذكر,أنثى"</formula1>
     </dataValidation>
@@ -9534,22 +10156,28 @@
     <dataValidation sqref="E2:E301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر اليوم" type="list">
       <formula1>"الأحد,الاثنين,الثلاثاء,الأربعاء,الخميس,الجمعة,السبت"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
+    <dataValidation sqref="M2:M301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر أو اكتب ملاحظة" type="list">
+      <formula1>"انتهت المناقشة,تم التأجيل"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر أو اكتب اسم المنسق" type="list">
+      <formula1>"محمد الحربي"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q2:Q301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
       <formula1>"مشرفاً ومقرراً,مشرفاً,مشرفاً مشاركاً,مناقشاً,مناقشاً خارجياً,مشرفةً ومقررةً,مناقِشةً"</formula1>
     </dataValidation>
-    <dataValidation sqref="R2:R301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
+    <dataValidation sqref="T2:T301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
       <formula1>"مشرفاً ومقرراً,مشرفاً,مشرفاً مشاركاً,مناقشاً,مناقشاً خارجياً,مشرفةً ومقررةً,مناقِشةً"</formula1>
     </dataValidation>
-    <dataValidation sqref="U2:U301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
+    <dataValidation sqref="W2:W301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
       <formula1>"مشرفاً ومقرراً,مشرفاً,مشرفاً مشاركاً,مناقشاً,مناقشاً خارجياً,مشرفةً ومقررةً,مناقِشةً"</formula1>
     </dataValidation>
-    <dataValidation sqref="X2:X301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
+    <dataValidation sqref="Z2:Z301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
       <formula1>"مشرفاً ومقرراً,مشرفاً,مشرفاً مشاركاً,مناقشاً,مناقشاً خارجياً,مشرفةً ومقررةً,مناقِشةً"</formula1>
     </dataValidation>
-    <dataValidation sqref="AA2:AA301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
+    <dataValidation sqref="AC2:AC301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر من القائمة أو اكتب دوراً آخر" type="list">
       <formula1>"مشرفاً ومقرراً,مشرفاً,مشرفاً مشاركاً,مناقشاً,مناقشاً خارجياً,مشرفةً ومقررةً,مناقِشةً"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر أو اكتب الصفة" type="list">
+    <dataValidation sqref="P2:P301" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="اختيار" prompt="اختر أو اكتب الصفة" type="list">
       <formula1>"الأستاذ في قسم الفقه,الأستاذ المشارك في قسم الفقه,الأستاذ المساعد في قسم الفقه"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9564,7 +10192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -9622,174 +10250,209 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>7) في الموقع: «جدول بيانات الإعلانات» ← «📄 من ملف Excel / CSV» ← اختر هذا الملف. ستظهر البيانات في الجدول وتقدر تعدّلها ثم «📦 تحميل المحدد».</t>
+          <t>7) الملاحظات ومنسق الحجز للتنظيم الداخلي (لا تظهر في الإعلان). أسطر «إجازة أسبوعية» في الملف المصدَّر من الموقع تُتجاهل عند الاستيراد.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="9" t="inlineStr"/>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>8) في الموقع: «جدول بيانات الإعلانات» ← «📄 من ملف Excel / CSV» ← اختر هذا الملف. ستظهر البيانات في الجدول وتقدر تعدّلها ثم «📦 تحميل المحدد».</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="9" t="inlineStr"/>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>استخدامه في Google Sheets</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>ارفع هذا الملف إلى Google Drive ثم افتحه بـ Google Sheets (أو: ملف ← استيراد). بعد التعبئة: «مشاركة» ← «أي شخص لديه الرابط» (عارض)،</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>ثم انسخ الرابط والصقه في الموقع واضغط «🔗 من Google Sheets». وكل ما عدّلت الشيت اضغط «🔄 تحديث» في الموقع.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="9" t="inlineStr"/>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="9" t="inlineStr"/>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>مثال على سطر معبّأ</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>الدرجة:   الماجستير في الفقه المقارن</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>الجنس:   ذكر</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>الطالب:   عبد الله بن عادل السعدي</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>العنوان:   المسائل الفقهية التي خالف فيها الإمام محمد بن عبد الوهاب المذهب الحنبلي | (جمعاً ودراسة)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>اليوم:   الأحد</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>التاريخ:   1448/4/16 هـ</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>الوقت:   8 صباحاً</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>المكان:   قاعة ابن عثيمين</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>ملاحظة المكان:   (والبث عبر الإنترنت)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>رابط البث:   https://www.youtube.com/@src.sds1</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>رابط اللجنة:   أ.د. عمر بن علي السديس</t>
+          <t xml:space="preserve">رابط اللجنة:   </t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>رابط التسجيل:   الأستاذ في قسم الفقه</t>
+          <t xml:space="preserve">رابط التسجيل:   </t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>عضو1 الاسم:   مشرفاً ومقرراً</t>
+          <t xml:space="preserve">الملاحظات:   </t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>عضو1 الصفة:   أ.د. فهد بن صالح الحمود</t>
+          <t>منسق الحجز:   محمد الحربي</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>عضو1 الدور:   الأستاذ في قسم الفقه</t>
+          <t>عضو1 الاسم:   أ.د. عمر بن علي السديس</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>عضو2 الاسم:   مناقشاً</t>
+          <t>عضو1 الصفة:   الأستاذ في قسم الفقه</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="10" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>عضو2 الصفة:   د. أحمد بن سليمان العودة</t>
+          <t>عضو1 الدور:   مشرفاً ومقرراً</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>عضو2 الدور:   الأستاذ المساعد في قسم الفقه</t>
+          <t>عضو2 الاسم:   أ.د. فهد بن صالح الحمود</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>عضو3 الاسم:   مناقشاً</t>
+          <t>عضو2 الصفة:   الأستاذ في قسم الفقه</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>عضو2 الدور:   مناقشاً</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>عضو3 الاسم:   د. أحمد بن سليمان العودة</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>عضو3 الصفة:   الأستاذ المساعد في قسم الفقه</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>عضو3 الدور:   مناقشاً</t>
         </is>
       </c>
     </row>

</xml_diff>